<commit_message>
docs: finalize shift handover syllabus and bounded classroom AI handoff
</commit_message>
<xml_diff>
--- a/문서/교재/실라버스/피지컬AI_실라버스_최종본.xlsx
+++ b/문서/교재/실라버스/피지컬AI_실라버스_최종본.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="통합반 온라인 44H" sheetId="1" r:id="R20013cea40554f14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="실전반 온라인 32H" sheetId="2" r:id="R1e906291cad74cf2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="통합반 오프라인 정규 10회" sheetId="3" r:id="Rcd676307fc7e43ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="실전반 오프라인 정규 9회" sheetId="4" r:id="R8e2c1419cc4449ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="통합반 온라인 44H" sheetId="1" r:id="R0aca771b9b7e4936"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="실전반 온라인 32H" sheetId="2" r:id="Rb2ce782d014c4cc0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="통합반 오프라인 정규 10회" sheetId="3" r:id="Rb5aac374f1d04105"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="실전반 오프라인 정규 9회" sheetId="4" r:id="Rb9a564940b9b4b2c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2593,10 +2593,8 @@
     </x:row>
     <x:row r="107"/>
     <x:row r="108" s="1" customFormat="1" ht="39" customHeight="1">
-      <x:c r="A108" s="43" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">11일차  |  온톨로지·에이전트·프로세스를 내 주제에 적용하고 마무리하기</x:t>
-        </x:is>
+      <x:c r="A108" s="43" t="str">
+        <x:v>11일차  |  추가 지식과 에이전트로 교대 인수인계 완성하기</x:v>
       </x:c>
       <x:c r="D108" s="44" t="inlineStr">
         <x:is>
@@ -2672,13 +2670,11 @@
           <x:t xml:space="preserve">실습</x:t>
         </x:is>
       </x:c>
-      <x:c r="B112" s="55" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">내 주제의 자료·업무 목표·완료 조건 정의하기</x:t>
-        </x:is>
+      <x:c r="B112" s="55" t="str">
+        <x:v>교대 인수인계의 입력과 완료 조건 정의하기</x:v>
       </x:c>
       <x:c r="C112" s="53" t="str">
-        <x:v>배운 로컬 랩에서 직접 만들 목적·입력·근거·완료 조건을 정한다. 제공 제조 자료를 활용하거나 준비된 자료로 완주 가능한 개인 주제를 선택한다.</x:v>
+        <x:v>대상 설비·교대·기준 시각과 작업 메모를 입력으로 정한다. 설비 상태, 미완료 작업지시, 부품 대기 정보를 대조하여 다음 근무자의 확인 사항을 인계한다. ABC의 조치·정비·구매를 다시 실행하지 않고 인계자 검토와 인수자 확인을 완료 조건으로 정한다.</x:v>
       </x:c>
       <x:c r="D112" s="54" t="n">
         <x:v>30</x:v>
@@ -2690,15 +2686,11 @@
           <x:t xml:space="preserve">실습</x:t>
         </x:is>
       </x:c>
-      <x:c r="B113" s="62" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">내 문서에서 주요 정보를 뽑아 작은 지식 구조 만들기</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C113" s="60" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">제공 문서 또는 본인의 공개 가능 자료에서 핵심 개념·속성·관계를 구분해 스키마와 샘플 인스턴스를 작성한다. 출처와 식별자를 남기며 수업용 별도 이름 공간 또는 샘플 데이터로 검증한다.</x:t>
-        </x:is>
+      <x:c r="B113" s="62" t="str">
+        <x:v>보충 매뉴얼을 추출·검토하여 기존 지식에 추가하기</x:v>
+      </x:c>
+      <x:c r="C113" s="60" t="str">
+        <x:v>강사가 제공한 설비 점검·이상 확인 보충 매뉴얼에서 절차·조건·근거를 추출하고 원문 대조 후 적재한다. 기존 제조 스키마와 지식은 유지하며 새 문서로 추가한다. 동일 조건의 추출 결과를 재사용할 때는 이를 표시한다. 임의 문서는 허용하지 않는다.</x:v>
       </x:c>
       <x:c r="D113" s="61" t="n">
         <x:v>30</x:v>
@@ -2710,15 +2702,11 @@
           <x:t xml:space="preserve">실습</x:t>
         </x:is>
       </x:c>
-      <x:c r="B114" s="55" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">내 지식과 연결 도구를 사용해 업무를 제안하는 에이전트 만들기</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C114" s="53" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">앞서 만든 스키마·자료를 활용하는 작은 에이전트를 VS Code에서 구성한다. 사용할 수 있는 읽기 MCP를 연결하여 정보가 확인될 때만 제안하고, 미확인 값과 권한 없는 작업은 보류하는 결과를 만든다.</x:t>
-        </x:is>
+      <x:c r="B114" s="55" t="str">
+        <x:v>설비·정비·ERP를 대조하는 인수인계 에이전트 만들기</x:v>
+      </x:c>
+      <x:c r="C114" s="53" t="str">
+        <x:v>기존 지식과 허용된 설비·정비·ERP 조회 도구로 인계안을 작성하는 에이전트·스킬을 구성한다. 완료 메모와 열린 작업지시, 부품 도착 예정과 실제 재고의 불일치를 확인 사항으로 남긴다. 최신 값은 원천에서 조회하고 미확인 업무를 완료로 추정하지 않는다.</x:v>
       </x:c>
       <x:c r="D114" s="54" t="n">
         <x:v>30</x:v>
@@ -2731,10 +2719,10 @@
         </x:is>
       </x:c>
       <x:c r="B115" s="62" t="str">
-        <x:v>공통 업무 흐름을 확인하고 개인 결과 완성하기</x:v>
+        <x:v>교대 인수인계 BPMN을 등록하고 검토·확인 흐름 실행하기</x:v>
       </x:c>
       <x:c r="C115" s="60" t="str">
-        <x:v>기존 검증된 포털 예제로 업무 흐름을 실행하고 역할·승인·완료 상태를 확인한다. 개인 로컬 결과는 별도로 실행·수정하고 사용 방법을 저장한다. 학생 코드를 포털 기본 에이전트에 자동 등록하거나 새로 연결하지 않는다.</x:v>
+        <x:v>bpmn.io에서 자료 조회→인계안 작성→인계자 검토→인수자 확인 또는 보완 요청→완료 기록을 설계한다. 포털에서 별도 정의·시작 폼·에이전트·역할을 연결해 등록한다. 설비·교대를 입력해 시작하고 정상·불일치·보완 경로와 인계 기록을 확인한다.</x:v>
       </x:c>
       <x:c r="D115" s="61" t="n">
         <x:v>30</x:v>
@@ -4251,10 +4239,8 @@
       <x:c r="D86" s="50" t="n"/>
     </x:row>
     <x:row r="87" s="1" customFormat="1" ht="39" customHeight="1">
-      <x:c r="A87" s="43" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">08일차  |  배운 전 과정을 내 주제에 활용하고 지식 자산으로 마무리하기</x:t>
-        </x:is>
+      <x:c r="A87" s="43" t="str">
+        <x:v>08일차  |  추가 지식과 에이전트로 교대 인수인계 완성하기</x:v>
       </x:c>
       <x:c r="D87" s="44" t="inlineStr">
         <x:is>
@@ -4330,13 +4316,11 @@
           <x:t xml:space="preserve">실습</x:t>
         </x:is>
       </x:c>
-      <x:c r="B91" s="55" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">내 주제의 자료와 업무 완료 조건 정의하기</x:t>
-        </x:is>
+      <x:c r="B91" s="55" t="str">
+        <x:v>교대 인수인계의 입력과 완료 조건 정의하기</x:v>
       </x:c>
       <x:c r="C91" s="53" t="str">
-        <x:v>앞 활용 랩에서 기능 하나를 골라 직접 사용할 목적·입력·근거·완료 기준을 정한다. 기존 자료와 로컬 코드·스킬로 완주 가능한 범위를 선택한다.</x:v>
+        <x:v>대상 설비·교대·기준 시각과 작업 메모를 입력으로 정한다. 설비 상태, 미완료 작업지시, 부품 대기 정보를 대조하여 다음 근무자의 확인 사항을 인계한다. ABC의 조치·정비·구매를 다시 실행하지 않고 인계자 검토와 인수자 확인을 완료 조건으로 정한다.</x:v>
       </x:c>
       <x:c r="D91" s="54" t="n">
         <x:v>30</x:v>
@@ -4348,13 +4332,11 @@
           <x:t xml:space="preserve">실습</x:t>
         </x:is>
       </x:c>
-      <x:c r="B92" s="62" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">개인 자료에서 작은 지식 구조 만들기</x:t>
-        </x:is>
+      <x:c r="B92" s="62" t="str">
+        <x:v>보충 매뉴얼을 추출·검토하여 기존 지식에 추가하기</x:v>
       </x:c>
       <x:c r="C92" s="60" t="str">
-        <x:v>선택한 목적에 필요한 문서·기존 랩 자료로 작은 지식 구조를 구성한다. 고유 ID와 출처를 보존하고 목적에 필요한 질문의 답을 확인한다.</x:v>
+        <x:v>강사가 제공한 설비 점검·이상 확인 보충 매뉴얼에서 절차·조건·근거를 추출하고 원문 대조 후 적재한다. 기존 제조 스키마와 지식은 유지하며 새 문서로 추가한다. 동일 조건의 추출 결과를 재사용할 때는 이를 표시한다. 임의 문서는 허용하지 않는다.</x:v>
       </x:c>
       <x:c r="D92" s="61" t="n">
         <x:v>30</x:v>
@@ -4366,13 +4348,11 @@
           <x:t xml:space="preserve">실습</x:t>
         </x:is>
       </x:c>
-      <x:c r="B93" s="55" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">내 지식과 연결 도구로 업무 제안 에이전트 만들기</x:t>
-        </x:is>
+      <x:c r="B93" s="55" t="str">
+        <x:v>설비·정비·ERP를 대조하는 인수인계 에이전트 만들기</x:v>
       </x:c>
       <x:c r="C93" s="53" t="str">
-        <x:v>앞 지식과 제공 도구를 활용해 목적에 맞는 제안·카드·보고서 등 로컬 결과를 만든다. 미확인·근거 부족을 표시하고 실제 출력과 완료 기준을 대조한다.</x:v>
+        <x:v>기존 지식과 허용된 설비·정비·ERP 조회 도구로 인계안을 작성하는 에이전트·스킬을 구성한다. 완료 메모와 열린 작업지시, 부품 도착 예정과 실제 재고의 불일치를 확인 사항으로 남긴다. 최신 값은 원천에서 조회하고 미확인 업무를 완료로 추정하지 않는다.</x:v>
       </x:c>
       <x:c r="D93" s="54" t="n">
         <x:v>30</x:v>
@@ -4385,10 +4365,10 @@
         </x:is>
       </x:c>
       <x:c r="B94" s="62" t="str">
-        <x:v>공통 업무 흐름을 확인하고 개인 결과 완성하기</x:v>
+        <x:v>교대 인수인계 BPMN을 등록하고 검토·확인 흐름 실행하기</x:v>
       </x:c>
       <x:c r="C94" s="60" t="str">
-        <x:v>기존 검증된 포털 예제로 업무 흐름을 실행하고 역할·승인·완료 상태를 확인한다. 개인 로컬 결과는 별도로 실행·수정하고 사용 방법을 저장한다. 학생 코드를 포털 기본 에이전트에 자동 등록하거나 새로 연결하지 않는다.</x:v>
+        <x:v>bpmn.io에서 자료 조회→인계안 작성→인계자 검토→인수자 확인 또는 보완 요청→완료 기록을 설계한다. 포털에서 별도 정의·시작 폼·에이전트·역할을 연결해 등록한다. 설비·교대를 입력해 시작하고 정상·불일치·보완 경로와 인계 기록을 확인한다.</x:v>
       </x:c>
       <x:c r="D94" s="61" t="n">
         <x:v>30</x:v>
@@ -6049,7 +6029,7 @@
     </x:row>
     <x:row r="94" s="1" customFormat="1" ht="36" customHeight="1">
       <x:c r="A94" s="43" t="str">
-        <x:v>09회차 | 프로세스를 실행·검증하고 개인 제작 시작하기</x:v>
+        <x:v>09회차 | 프로세스를 실행·검증하고 교대 인수인계 제작 시작하기</x:v>
       </x:c>
       <x:c r="B94"/>
       <x:c r="C94"/>
@@ -6079,7 +6059,7 @@
         <x:v>정의·실행 상태·오류 위치와 복구</x:v>
       </x:c>
       <x:c r="C96" s="127" t="str">
-        <x:v>정의·실행 상태·오류 위치와 복구을(를) 오늘 수행할 과제와 연결해 설명한다. 온라인 대응: 통합 온라인9 + 11 개인 적용 / 실전 온라인6 + 8 개인 적용. 복습 대신 적용에 필요한 설명으로 한정한다.</x:v>
+        <x:v>정의·실행 상태·오류 위치와 복구를 오늘 과제와 연결해 설명한다. 온라인 대응: 통합 온라인9·11 / 실전 온라인6·8. 교대 인수인계의 시작 폼·역할·완료 조건을 구분한다.</x:v>
       </x:c>
       <x:c r="D96" s="128" t="n">
         <x:v>15</x:v>
@@ -6132,10 +6112,10 @@
         <x:v>실습</x:v>
       </x:c>
       <x:c r="B100" s="130" t="str">
-        <x:v>개인 제작: 앞선 로컬 랩 하나를 선택하고 용도·입력·완료 기준 정하기</x:v>
+        <x:v>교대 인수인계의 입력·근거·완료 조건 정하기</x:v>
       </x:c>
       <x:c r="C100" s="131" t="str">
-        <x:v>앞 로컬 랩 하나를 골라 사용할 목적·입력·완료 기준을 정한다.</x:v>
+        <x:v>대상 설비·교대·기준 시각과 작업 메모를 입력으로 정한다. 설비 상태, 미완료 작업지시, 부품 대기 정보를 대조하여 다음 근무자의 확인 사항을 인계한다. ABC의 조치·정비·구매를 다시 실행하지 않고 인계자 검토와 인수자 확인을 완료 조건으로 정한다.</x:v>
       </x:c>
       <x:c r="D100" s="132" t="n">
         <x:v>25</x:v>
@@ -6146,10 +6126,10 @@
         <x:v>실습</x:v>
       </x:c>
       <x:c r="B101" s="130" t="str">
-        <x:v>개인 제작: 기존 자료·기능으로 첫 결과 구현</x:v>
+        <x:v>보충 매뉴얼 적재와 인수인계 에이전트 구성</x:v>
       </x:c>
       <x:c r="C101" s="131" t="str">
-        <x:v>기존 자료·코드·스킬로 개인 결과를 구현한다. 새 포털 연동은 요구하지 않는다.</x:v>
+        <x:v>제공 보충 매뉴얼의 추출 결과를 원문 대조하여 기존 제조 지식에 추가한다. 허용된 설비·정비·ERP 조회를 사용해 인계안을 만들고, 기록 불일치와 미확인 사항을 남긴다. 같은 조건의 추출 재사용은 표시한다.</x:v>
       </x:c>
       <x:c r="D101" s="132" t="n">
         <x:v>60</x:v>
@@ -6160,10 +6140,10 @@
         <x:v>실습</x:v>
       </x:c>
       <x:c r="B102" s="130" t="str">
-        <x:v>개별 오류 해결·중간 결과 저장</x:v>
+        <x:v>교대 인수인계 BPMN 설계·매핑과 중간 결과 저장</x:v>
       </x:c>
       <x:c r="C102" s="131" t="str">
-        <x:v>오류를 해결하고 중간 결과를 저장해 마지막 회차에서 이어 쓴다.</x:v>
+        <x:v>bpmn.io에서 조회·인계안·인계자 검토·인수자 확인·보완·완료 흐름을 작성한다. 포털의 별도 정의에 시작 폼·에이전트·역할을 연결하고 판본을 저장한다. 실제 실행은 다음 회차로 이어간다.</x:v>
       </x:c>
       <x:c r="D102" s="132" t="n">
         <x:v>20</x:v>
@@ -6182,7 +6162,7 @@
     </x:row>
     <x:row r="104" ht="58" customHeight="1">
       <x:c r="A104" s="66" t="str">
-        <x:v>완료 결과: 공통 포털 실행 결과와 별개의 개인 로컬 프로젝트. 포털에 개인 코드를 자동 등록하거나 연결하지 않는다.</x:v>
+        <x:v>완료 결과: 추가 지식의 검토·적재 기록, 인수인계 에이전트·스킬, 별도 BPMN·매핑·시작 폼. 기존 ABC 정의는 보존한다. 임의 코드 자동 연결이나 임의 외부 도구는 요구하지 않는다.</x:v>
       </x:c>
       <x:c r="B104"/>
       <x:c r="C104"/>
@@ -6193,7 +6173,7 @@
     </x:row>
     <x:row r="106" ht="36" customHeight="1">
       <x:c r="A106" s="43" t="str">
-        <x:v>10회차 | 정비·구매에 적용하고 개인 결과물 완성하기</x:v>
+        <x:v>10회차 | 정비·구매에 적용하고 교대 인수인계 완성하기</x:v>
       </x:c>
       <x:c r="B106"/>
       <x:c r="C106"/>
@@ -6290,10 +6270,10 @@
         <x:v>실습</x:v>
       </x:c>
       <x:c r="B113" s="130" t="str">
-        <x:v>앞 회차 개인 결과물 완성·실행·사용 방법 저장</x:v>
+        <x:v>교대 인수인계 흐름 실행·보완·완료 기록 확인</x:v>
       </x:c>
       <x:c r="C113" s="131" t="str">
-        <x:v>앞 회차 개인 프로젝트를 실행·수정하고 결과와 사용 방법을 저장한다.</x:v>
+        <x:v>앞 회차의 인수인계 흐름을 설비·교대 입력으로 시작한다. 정상·기록 불일치·정보 누락 사례에서 인계자 검토와 인수자 확인 또는 보완 요청을 수행하고, 근거·판본·완료 기록을 저장한다.</x:v>
       </x:c>
       <x:c r="D113" s="132" t="n">
         <x:v>30</x:v>
@@ -6326,7 +6306,7 @@
     </x:row>
     <x:row r="116" ht="58" customHeight="1">
       <x:c r="A116" s="66" t="str">
-        <x:v>완료 결과: 정비·구매는 공통 시나리오 그대로 수행. 개인 결과는 로컬 코드·스킬·보고서로 완료하며 새 포털 기능이나 외부 서비스 쓰기를 요구하지 않는다. ProcessGPT는 준비된 제품 화면을 강사가 20분 시연한다. 학생 계정 설정이나 별도 제품 실습은 포함하지 않는다.</x:v>
+        <x:v>완료 결과: 정비·구매는 기존 공통 시나리오로 수행하고 교대 인수인계는 별도 정의로 실행한다. 실제 설비 제어·발주를 인계 확인과 혼동하지 않는다. ProcessGPT는 강사가 20분 시연한다. 준비·실행 시간과 완주는 별도 실측한다.</x:v>
       </x:c>
       <x:c r="B116"/>
       <x:c r="C116"/>
@@ -7724,7 +7704,7 @@
     </x:row>
     <x:row r="81" s="1" customFormat="1" ht="36" customHeight="1">
       <x:c r="A81" s="43" t="str">
-        <x:v>08회차 | 프로세스를 실행·검증하고 개인 제작 시작하기</x:v>
+        <x:v>08회차 | 프로세스를 실행·검증하고 교대 인수인계 제작 시작하기</x:v>
       </x:c>
       <x:c r="B81"/>
       <x:c r="C81"/>
@@ -7754,7 +7734,7 @@
         <x:v>정의·실행 상태·오류 위치와 복구</x:v>
       </x:c>
       <x:c r="C83" s="127" t="str">
-        <x:v>정의·실행 상태·오류 위치와 복구을(를) 오늘 수행할 과제와 연결해 설명한다. 온라인 대응: 통합 온라인9 + 11 개인 적용 / 실전 온라인6 + 8 개인 적용. 복습 대신 적용에 필요한 설명으로 한정한다.</x:v>
+        <x:v>정의·실행 상태·오류 위치와 복구를 오늘 과제와 연결해 설명한다. 온라인 대응: 통합 온라인9·11 / 실전 온라인6·8. 교대 인수인계의 시작 폼·역할·완료 조건을 구분한다.</x:v>
       </x:c>
       <x:c r="D83" s="128" t="n">
         <x:v>15</x:v>
@@ -7807,10 +7787,10 @@
         <x:v>실습</x:v>
       </x:c>
       <x:c r="B87" s="130" t="str">
-        <x:v>개인 제작: 앞선 로컬 랩 하나를 선택하고 용도·입력·완료 기준 정하기</x:v>
+        <x:v>교대 인수인계의 입력·근거·완료 조건 정하기</x:v>
       </x:c>
       <x:c r="C87" s="131" t="str">
-        <x:v>앞 로컬 랩 하나를 골라 사용할 목적·입력·완료 기준을 정한다.</x:v>
+        <x:v>대상 설비·교대·기준 시각과 작업 메모를 입력으로 정한다. 설비 상태, 미완료 작업지시, 부품 대기 정보를 대조하여 다음 근무자의 확인 사항을 인계한다. ABC의 조치·정비·구매를 다시 실행하지 않고 인계자 검토와 인수자 확인을 완료 조건으로 정한다.</x:v>
       </x:c>
       <x:c r="D87" s="132" t="n">
         <x:v>25</x:v>
@@ -7821,10 +7801,10 @@
         <x:v>실습</x:v>
       </x:c>
       <x:c r="B88" s="130" t="str">
-        <x:v>개인 제작: 기존 자료·기능으로 첫 결과 구현</x:v>
+        <x:v>보충 매뉴얼 적재와 인수인계 에이전트 구성</x:v>
       </x:c>
       <x:c r="C88" s="131" t="str">
-        <x:v>기존 자료·코드·스킬로 개인 결과를 구현한다. 새 포털 연동은 요구하지 않는다.</x:v>
+        <x:v>제공 보충 매뉴얼의 추출 결과를 원문 대조하여 기존 제조 지식에 추가한다. 허용된 설비·정비·ERP 조회를 사용해 인계안을 만들고, 기록 불일치와 미확인 사항을 남긴다. 같은 조건의 추출 재사용은 표시한다.</x:v>
       </x:c>
       <x:c r="D88" s="132" t="n">
         <x:v>60</x:v>
@@ -7835,10 +7815,10 @@
         <x:v>실습</x:v>
       </x:c>
       <x:c r="B89" s="130" t="str">
-        <x:v>개별 오류 해결·중간 결과 저장</x:v>
+        <x:v>교대 인수인계 BPMN 설계·매핑과 중간 결과 저장</x:v>
       </x:c>
       <x:c r="C89" s="131" t="str">
-        <x:v>오류를 해결하고 중간 결과를 저장해 마지막 회차에서 이어 쓴다.</x:v>
+        <x:v>bpmn.io에서 조회·인계안·인계자 검토·인수자 확인·보완·완료 흐름을 작성한다. 포털의 별도 정의에 시작 폼·에이전트·역할을 연결하고 판본을 저장한다. 실제 실행은 다음 회차로 이어간다.</x:v>
       </x:c>
       <x:c r="D89" s="132" t="n">
         <x:v>20</x:v>
@@ -7857,7 +7837,7 @@
     </x:row>
     <x:row r="91" ht="58" customHeight="1">
       <x:c r="A91" s="66" t="str">
-        <x:v>완료 결과: 공통 포털 실행 결과와 별개의 개인 로컬 프로젝트. 포털에 개인 코드를 자동 등록하거나 연결하지 않는다.</x:v>
+        <x:v>완료 결과: 추가 지식의 검토·적재 기록, 인수인계 에이전트·스킬, 별도 BPMN·매핑·시작 폼. 기존 ABC 정의는 보존한다. 임의 코드 자동 연결이나 임의 외부 도구는 요구하지 않는다.</x:v>
       </x:c>
       <x:c r="B91"/>
       <x:c r="C91"/>
@@ -7868,7 +7848,7 @@
     </x:row>
     <x:row r="93" ht="36" customHeight="1">
       <x:c r="A93" s="43" t="str">
-        <x:v>09회차 | 정비·구매에 적용하고 개인 결과물 완성하기</x:v>
+        <x:v>09회차 | 정비·구매에 적용하고 교대 인수인계 완성하기</x:v>
       </x:c>
       <x:c r="B93"/>
       <x:c r="C93"/>
@@ -7965,10 +7945,10 @@
         <x:v>실습</x:v>
       </x:c>
       <x:c r="B100" s="130" t="str">
-        <x:v>앞 회차 개인 결과물 완성·실행·사용 방법 저장</x:v>
+        <x:v>교대 인수인계 흐름 실행·보완·완료 기록 확인</x:v>
       </x:c>
       <x:c r="C100" s="131" t="str">
-        <x:v>앞 회차 개인 프로젝트를 실행·수정하고 결과와 사용 방법을 저장한다.</x:v>
+        <x:v>앞 회차의 인수인계 흐름을 설비·교대 입력으로 시작한다. 정상·기록 불일치·정보 누락 사례에서 인계자 검토와 인수자 확인 또는 보완 요청을 수행하고, 근거·판본·완료 기록을 저장한다.</x:v>
       </x:c>
       <x:c r="D100" s="132" t="n">
         <x:v>30</x:v>
@@ -8001,7 +7981,7 @@
     </x:row>
     <x:row r="103" ht="58" customHeight="1">
       <x:c r="A103" s="66" t="str">
-        <x:v>완료 결과: 정비·구매는 공통 시나리오 그대로 수행. 개인 결과는 로컬 코드·스킬·보고서로 완료하며 새 포털 기능이나 외부 서비스 쓰기를 요구하지 않는다. ProcessGPT는 준비된 제품 화면을 강사가 20분 시연한다. 학생 계정 설정이나 별도 제품 실습은 포함하지 않는다.</x:v>
+        <x:v>완료 결과: 정비·구매는 기존 공통 시나리오로 수행하고 교대 인수인계는 별도 정의로 실행한다. 실제 설비 제어·발주를 인계 확인과 혼동하지 않는다. ProcessGPT는 강사가 20분 시연한다. 준비·실행 시간과 완주는 별도 실측한다.</x:v>
       </x:c>
       <x:c r="B103"/>
       <x:c r="C103"/>

</xml_diff>

<commit_message>
Restore HYD introduction and revise course progression and offline allocation
</commit_message>
<xml_diff>
--- a/문서/교재/실라버스/피지컬AI_실라버스_최종본.xlsx
+++ b/문서/교재/실라버스/피지컬AI_실라버스_최종본.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="통합반 온라인 44H" sheetId="1" r:id="Rb671491d80264b7c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="실전반 온라인 32H" sheetId="2" r:id="R7f4a1a1f640b4bb5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="통합반 오프라인 정규 10회" sheetId="3" r:id="R86cff5214ecc4afa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="실전반 오프라인 정규 9회" sheetId="4" r:id="Raaeb30ffe83747c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="통합반 온라인 44H" sheetId="1" r:id="R8bf50ea5b26f4890"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="실전반 온라인 32H" sheetId="2" r:id="R604ce3e088134b2b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="통합반 오프라인 정규 10회" sheetId="3" r:id="Rf4d11f162fb44998"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="실전반 오프라인 정규 9회" sheetId="4" r:id="Rbb8e2240d91e468a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -974,7 +974,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="6" s="1" customFormat="1" ht="65" customHeight="1">
+    <x:row r="6" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A6" s="22" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">이론</x:t>
@@ -986,7 +986,7 @@
         </x:is>
       </x:c>
       <x:c r="C6" s="19" t="str">
-        <x:v>단순히 내용을 기록하는 것과 나중에 다시 찾아 활용할 수 있는 지식 자산으로 축적하는 것의 차이를 이해한다. 학습한 개념, 핵심 원리, 참고 자료와 출처, 실습 과정 및 결과를 체계적으로 연결해 기록하는 이유를 배운다. Notion을 활용해 수업이 끝난 뒤에도 지식을 검색·보완·재사용할 수 있는 개인 학습 체계를 마련하는 목적을 살펴본다.</x:v>
+        <x:v>HYD의 전체 흐름을 보고 이후 실습에서 만들 지식·에이전트·업무 연결의 목표를 확인한다. 단순히 내용을 기록하는 것과 나중에 다시 찾아 활용할 수 있는 지식 자산으로 축적하는 것의 차이를 이해한다. 학습한 개념, 핵심 원리, 참고 자료와 출처, 실습 과정 및 결과를 체계적으로 연결해 기록하는 이유를 배운다. Notion을 활용해 수업이 끝난 뒤에도 지식을 검색·보완·재사용할 수 있는 개인 학습 체계를 마련하는 목적을 살펴본다.</x:v>
       </x:c>
       <x:c r="D6" s="25" t="n">
         <x:v>10</x:v>
@@ -1082,7 +1082,7 @@
         <x:v>50</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" s="1" customFormat="1" ht="77.80000305175781" customHeight="1">
+    <x:row r="12" s="1" customFormat="1" ht="118" customHeight="1">
       <x:c r="A12" s="30" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">실습</x:t>
@@ -1094,7 +1094,7 @@
         </x:is>
       </x:c>
       <x:c r="C12" s="19" t="str">
-        <x:v>arrows.app의 노드·관계·레이블 작성 방법을 익힌다. 간단한 설비 이상 사례를 바탕으로 설비·센서·증상·원인·조치를 배치하고 각각의 연결 관계를 직접 그린다. 어떤 대상이 다른 대상과 연결되는지, 관계의 방향을 어떻게 표현하는지 살펴본다. 완성한 관계도를 통해 단순히 정보를 나열하는 방식과 관계를 중심으로 표현하는 방식의 차이를 확인한다. 복잡한 온톨로지 스키마와 제약은 다음 학습에서 다룬다.</x:v>
+        <x:v>arrows.app의 노드·관계·레이블 작성 방법을 익힌다. 간단한 설비 이상 사례를 바탕으로 설비·센서·증상·원인·조치를 배치하고 각각의 연결 관계를 직접 그린다. 어떤 대상이 다른 대상과 연결되는지, 관계의 방향을 어떻게 표현하는지 살펴본다. 완성한 관계도를 통해 단순히 정보를 나열하는 방식과 관계를 중심으로 표현하는 방식의 차이를 확인한다. 복잡한 온톨로지 스키마와 제약은 다음 학습에서 다룬다. 이 관계를 다음 회차에서 식별자와 속성을 갖춘 모델로 옮겨 실제 질의로 확인한다.</x:v>
       </x:c>
       <x:c r="D12" s="25" t="n">
         <x:v>30</x:v>
@@ -1151,7 +1151,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="17" s="1" customFormat="1" ht="93.5" customHeight="1">
+    <x:row r="17" s="1" customFormat="1" ht="136" customHeight="1">
       <x:c r="A17" s="22" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">이론</x:t>
@@ -1163,7 +1163,7 @@
         </x:is>
       </x:c>
       <x:c r="C17" s="27" t="str">
-        <x:v>온톨로지에서 클래스·인스턴스·속성·관계의 정확한 정의와 역할을 학습한다. 클래스가 공통 특성을 가진 대상의 유형을 표현하고, 인스턴스는 그 유형에 속하는 실제 개별 대상을 나타낸다는 점을 살펴본다. 설비·센서·부품과 HYD-01·TS1·쿨러를 비교하며 구분한다. 클래스 계층과 상속의 기초, 데이터 속성과 객체 간 관계의 차이, 속성값과 인스턴스의 구별, 관계 유형·방향·카디널리티(1:1, 1:N, N:M)를 배운다. 언제 새로운 클래스를 정의하고 언제 속성이나 관계로 표현해야 하는지 구체적인 설비 사례로 비교한다.</x:v>
+        <x:v>앞서 그린 관계도에 같은 대상의 식별 기준을 정하고, 질문에 답할 수 있는 그래프를 만든다. 온톨로지에서 클래스·인스턴스·속성·관계의 정확한 정의와 역할을 학습한다. 클래스가 공통 특성을 가진 대상의 유형을 표현하고, 인스턴스는 그 유형에 속하는 실제 개별 대상을 나타낸다는 점을 살펴본다. 설비·센서·부품과 HYD-01·TS1·쿨러를 비교하며 구분한다. 클래스 계층과 상속의 기초, 데이터 속성과 객체 간 관계의 차이, 속성값과 인스턴스의 구별, 관계 유형·방향·카디널리티(1:1, 1:N, N:M)를 배운다. 언제 새로운 클래스를 정의하고 언제 속성이나 관계로 표현해야 하는지 구체적인 설비 사례로 비교한다.</x:v>
       </x:c>
       <x:c r="D17" s="33" t="n">
         <x:v>50</x:v>
@@ -1257,7 +1257,7 @@
         <x:v>40</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" s="1" customFormat="1" ht="65" customHeight="1">
+    <x:row r="23" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A23" s="30" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">실습</x:t>
@@ -1267,7 +1267,7 @@
         <x:v>설계한 온톨로지를 그래프 DB에 구현하고 검증하기</x:v>
       </x:c>
       <x:c r="C23" s="27" t="str">
-        <x:v>앞 실습의 스키마·인스턴스·요구사항·원자료 검토 기록을 이어 쓴다. VS Code의 GitHub Copilot·Codex로 Cypher를 작성하고 별도 랩 DB에 적재한다. 식별자·관계 끝점·방향과 원자료 질문의 답, 반복 적재 시 중복 여부를 확인한다. 오류가 있으면 근거에 따라 수정하고 질의·결과를 저장한다.</x:v>
+        <x:v>앞 실습의 스키마·인스턴스·요구사항·원자료 검토 기록을 이어 쓴다. VS Code의 GitHub Copilot·Codex로 Cypher를 작성하고 별도 랩 DB에 적재한다. 식별자·관계 끝점·방향과 원자료 질문의 답, 반복 적재 시 중복 여부를 확인한다. 오류가 있으면 근거에 따라 수정하고 질의·결과를 저장한다. 확인한 설비 식별자와 관계는 다음 회차에서 작업 절차와 조치 조건을 연결하는 기준이 된다.</x:v>
       </x:c>
       <x:c r="D23" s="33" t="n">
         <x:v>40</x:v>
@@ -1324,7 +1324,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="28" s="1" customFormat="1" ht="93.5" customHeight="1">
+    <x:row r="28" s="1" customFormat="1" ht="136" customHeight="1">
       <x:c r="A28" s="22" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">이론</x:t>
@@ -1336,7 +1336,7 @@
         </x:is>
       </x:c>
       <x:c r="C28" s="19" t="str">
-        <x:v>설비 고장 원인을 진단하는 것과 실제 조치 방법을 결정하는 것이 서로 다른 단계임을 이해한다. SOP(Standard Operating Procedure)의 목적과 역할을 배우고, 적용 대상·작업 전제 조건·안전 조건·준비사항·수행 단계·금지 사항·담당 역할·완료 확인 기준 등 SOP의 구성요소를 살펴본다. 작업 절차의 순서와 조건을 구분하고, 동일한 조치도 설비 운전 상태에 따라 수행 가능 여부가 달라지는 이유를 학습한다. HYD 온톨로지에서 고장 유형·원인·조치 방법(Skill)·작업 단계(Step)·근거 매뉴얼이 연결되는 구조와, 즉시 완화·근본 조치·예방 조치의 차이를 살펴본다.</x:v>
+        <x:v>설비 관계를 안다는 것만으로 조치를 실행할 수 없으므로, 허용 조건과 선택 근거를 구분한다. 설비 고장 원인을 진단하는 것과 실제 조치 방법을 결정하는 것이 서로 다른 단계임을 이해한다. SOP(Standard Operating Procedure)의 목적과 역할을 배우고, 적용 대상·작업 전제 조건·안전 조건·준비사항·수행 단계·금지 사항·담당 역할·완료 확인 기준 등 SOP의 구성요소를 살펴본다. 작업 절차의 순서와 조건을 구분하고, 동일한 조치도 설비 운전 상태에 따라 수행 가능 여부가 달라지는 이유를 학습한다. HYD 온톨로지에서 고장 유형·원인·조치 방법(Skill)·작업 단계(Step)·근거 매뉴얼이 연결되는 구조와, 즉시 완화·근본 조치·예방 조치의 차이를 살펴본다.</x:v>
       </x:c>
       <x:c r="D28" s="25" t="n">
         <x:v>35</x:v>
@@ -1396,7 +1396,7 @@
         <x:v>35</x:v>
       </x:c>
     </x:row>
-    <x:row r="32" s="1" customFormat="1" ht="77.80000305175781" customHeight="1">
+    <x:row r="32" s="1" customFormat="1" ht="118" customHeight="1">
       <x:c r="A32" s="30" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">실습</x:t>
@@ -1408,13 +1408,13 @@
         </x:is>
       </x:c>
       <x:c r="C32" s="19" t="str">
-        <x:v>VS Code에서 GitHub Copilot·Codex를 활용해 이미 작업 조건이 정리된 랩 전용 SOP 자료를 사용한다. 2일차에 만든 설비 모델과 식별자를 재사용하고, 제공된 고장 유형과 조치 방법을 연결한다. 작업의 적용 조건·금지 조건·수행 단계·완료 기준을 구분해 구조화하고, 이를 DMN 형태의 입력 조건과 판단 결과로 구성한다. 조치 방법과 단계, 판단 규칙의 의미적 관계를 정리해 SOP 구조와 결정표 자료를 완성한다. 이 과정에서는 원문 문서를 자동 추출하는 인제스천을 구현하지 않는다.</x:v>
+        <x:v>VS Code에서 GitHub Copilot·Codex를 활용해 이미 작업 조건이 정리된 랩 전용 SOP 자료를 사용한다. 제공된 이전 단계의 설비 모델과 식별자를 재사용하고, 제공된 고장 유형과 조치 방법을 연결한다. 작업의 적용 조건·금지 조건·수행 단계·완료 기준을 구분해 구조화하고, 이를 DMN 형태의 입력 조건과 판단 결과로 구성한다. 조치 방법과 단계, 판단 규칙의 의미적 관계를 정리해 SOP 구조와 결정표 자료를 완성한다. 이 과정에서는 원문 문서를 자동 추출하는 인제스천을 구현하지 않는다.</x:v>
       </x:c>
       <x:c r="D32" s="25" t="n">
         <x:v>45</x:v>
       </x:c>
     </x:row>
-    <x:row r="33" s="1" customFormat="1" ht="77.80000305175781" customHeight="1">
+    <x:row r="33" s="1" customFormat="1" ht="118" customHeight="1">
       <x:c r="A33" s="30" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">실습</x:t>
@@ -1426,7 +1426,7 @@
         </x:is>
       </x:c>
       <x:c r="C33" s="27" t="str">
-        <x:v>VS Code에서 앞서 작성한 결정표를 활용해 GitHub Copilot·Codex로 간단한 조치 판정 기능을 제작한다. 설비 상태·운전 조건·금지 조건 등 입력값에 따라 가능한 조치와 제외해야 하는 조치를 구분하도록 구현한다. 제공된 효과·비용·성과 지표 값을 이용해 허용된 조치 후보를 비교하고 선택 이유를 표시한다. 정상 조건·경계값·복수 규칙 일치·조치 불가 상황을 실행해 결과를 확인하고, 조건을 변경했을 때 판단이 어떻게 달라지는지 살펴본다.</x:v>
+        <x:v>VS Code에서 앞서 작성한 결정표를 활용해 GitHub Copilot·Codex로 간단한 조치 판정 기능을 제작한다. 설비 상태·운전 조건·금지 조건 등 입력값에 따라 가능한 조치와 제외해야 하는 조치를 구분하도록 구현한다. 제공된 효과·비용·성과 지표 값을 이용해 허용된 조치 후보를 비교하고 선택 이유를 표시한다. 정상 조건·경계값·복수 규칙 일치·조치 불가 상황을 실행해 결과를 확인하고, 조건을 변경했을 때 판단이 어떻게 달라지는지 살펴본다. 다음 회차에는 이 조건의 근거가 된 매뉴얼에서 지식을 추출하고 원문과 대조한다.</x:v>
       </x:c>
       <x:c r="D33" s="33" t="n">
         <x:v>50</x:v>
@@ -1483,7 +1483,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="38" s="1" customFormat="1" ht="145" customHeight="1">
+    <x:row r="38" s="1" customFormat="1" ht="208" customHeight="1">
       <x:c r="A38" s="22" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">이론</x:t>
@@ -1495,7 +1495,7 @@
         </x:is>
       </x:c>
       <x:c r="C38" s="19" t="str">
-        <x:v>인제스천(Ingestion)의 의미와 필요성을 학습하고, 매뉴얼·SOP 문서·업무 DB 등 서로 다른 형태의 원천 자료를 지식으로 전환하는 전체 과정을 이해한다. 원천 확보와 보관 → 문서 내용 분석 → 증상·원인·부품·조치·판단 조건 등 지식 후보 추출 → 기존 온톨로지 스키마와 식별자에 매핑 → 원문 근거 대조와 사람 검토 → 승인된 지식 적재 → 그래프 관계·출처 조회의 단계별 역할을 살펴본다. LLM의 문서 이해 및 구조화 출력 원리를 살펴보고, 추출 과정에서 발생할 수 있는 부정 조건 누락·수치/단위 오류·잘못된 관계 추론·근거 없는 내용 생성의 위험을 배운다. 원문 페이지·문단·인용 구간, 문서 식별자와 개정 이력, 지식 소유 관계 및 변경 추적이 필요한 이유를 살펴본다. 검색해 문서를 참고하는 방식과 구조화된 지식으로 등록하는 방식의 차이도 이해한다. 마지막으로 설비의 원인·절차·규칙처럼 상대적으로 안정적인 지식과 센서·재고·운전시간처럼 지속적으로 변하는 값을 구분하고, 실제 값은 업무 DB·시계열 DB 등 원천에서 조회하도록 연결하는 원리를 살펴본다.</x:v>
+        <x:v>앞서 사용한 조치 조건을 문서에서 찾아 검토하고, 다시 출처를 확인할 수 있는 지식으로 만든다. 인제스천(Ingestion)의 의미와 필요성을 학습하고, 매뉴얼·SOP 문서·업무 DB 등 서로 다른 형태의 원천 자료를 지식으로 전환하는 전체 과정을 이해한다. 원천 확보와 보관 → 문서 내용 분석 → 증상·원인·부품·조치·판단 조건 등 지식 후보 추출 → 기존 온톨로지 스키마와 식별자에 매핑 → 원문 근거 대조와 사람 검토 → 승인된 지식 적재 → 그래프 관계·출처 조회의 단계별 역할을 살펴본다. LLM의 문서 이해 및 구조화 출력 원리를 살펴보고, 추출 과정에서 발생할 수 있는 부정 조건 누락·수치/단위 오류·잘못된 관계 추론·근거 없는 내용 생성의 위험을 배운다. 원문 페이지·문단·인용 구간, 문서 식별자와 개정 이력, 지식 소유 관계 및 변경 추적이 필요한 이유를 살펴본다. 검색해 문서를 참고하는 방식과 구조화된 지식으로 등록하는 방식의 차이도 이해한다. 마지막으로 설비의 원인·절차·규칙처럼 상대적으로 안정적인 지식과 센서·재고·운전시간처럼 지속적으로 변하는 값을 구분하고, 실제 값은 업무 DB·시계열 DB 등 원천에서 조회하도록 연결하는 원리를 살펴본다.</x:v>
       </x:c>
       <x:c r="D38" s="25" t="n">
         <x:v>40</x:v>
@@ -1507,10 +1507,8 @@
           <x:t xml:space="preserve">실습</x:t>
         </x:is>
       </x:c>
-      <x:c r="B39" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">현장 매뉴얼에서 판단 근거를 추출하고 검증된 지식으로 등록하기</x:t>
-        </x:is>
+      <x:c r="B39" s="31" t="str">
+        <x:v>매뉴얼 원문과 등록된 지식의 조건·출처 대조하기</x:v>
       </x:c>
       <x:c r="C39" s="27" t="str">
         <x:v>제공 매뉴얼의 원문과 포털에 등록된 추출·검토 결과를 나란히 확인한다. 작업 순서·단위·금지 조건·대상 설비를 비교하고 수정하거나 제외할 후보를 표시한다. 지식 지도에서 채택된 항목의 설비·조치·출처 연결을 찾는다. 직접 추가 적재는 마지막 교대 실습에서 제공 보충 매뉴얼로 수행한다.</x:v>
@@ -1537,7 +1535,7 @@
         <x:v>50</x:v>
       </x:c>
     </x:row>
-    <x:row r="41" s="1" customFormat="1" ht="77.80000305175781" customHeight="1">
+    <x:row r="41" s="1" customFormat="1" ht="118" customHeight="1">
       <x:c r="A41" s="30" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">실습</x:t>
@@ -1549,13 +1547,13 @@
         </x:is>
       </x:c>
       <x:c r="C41" s="27" t="str">
-        <x:v>VS Code에서 앞서 추출한 지식 후보를 원문과 대조해 채택·수정·제외한다. 2일차에 만든 모델과 3일차에 학습한 조치·규칙의 구조를 재사용하여 후보를 해당 클래스·인스턴스·관계에 매핑한다. GitHub Copilot·Codex로 기존 식별자를 활용한 그래프 DB 적재 코드를 구현하고, 검토한 항목만 랩 전용 그래프 DB에 반영한다. 이후 고장 유형에서 원인·조치·판단 규칙·원문 출처로 이어지는 관계를 조회하고, 문서에서 추출한 지식이 앞서 만든 그래프에 보강된 결과를 확인한다.</x:v>
+        <x:v>VS Code에서 앞서 추출한 지식 후보를 원문과 대조해 채택·수정·제외한다. 제공된 이전 단계의 모델과 3일차에 학습한 조치·규칙의 구조를 재사용하여 후보를 해당 클래스·인스턴스·관계에 매핑한다. GitHub Copilot·Codex로 기존 식별자를 활용한 그래프 DB 적재 코드를 구현하고, 검토한 항목만 랩 전용 그래프 DB에 반영한다. 이후 고장 유형에서 원인·조치·판단 규칙·원문 출처로 이어지는 관계를 조회하고, 문서에서 추출한 지식이 앞서 만든 그래프에 보강된 결과를 확인한다.</x:v>
       </x:c>
       <x:c r="D41" s="33" t="n">
         <x:v>50</x:v>
       </x:c>
     </x:row>
-    <x:row r="42" s="1" customFormat="1" ht="77.80000305175781" customHeight="1">
+    <x:row r="42" s="1" customFormat="1" ht="118" customHeight="1">
       <x:c r="A42" s="22" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">이론</x:t>
@@ -1567,7 +1565,7 @@
         </x:is>
       </x:c>
       <x:c r="C42" s="19" t="str">
-        <x:v>1일차 온톨로지의 필요성에서 시작해 2일차 클래스·인스턴스·속성·관계·스키마와 그래프 DB, 3일차 SOP·DMN·BSC/KPI의 조치·판단·성과 체계, 4일차 원천 자료 추출·검토·인제스천·출처 관리를 하나의 흐름으로 복습한다. 각 단계의 입력과 결과물, 지식 구조와 실제 데이터의 차이, 판단 규칙과 근거 문서의 관계를 되짚는다. 이렇게 구축된 지식과 규칙이 이후 에이전트의 업무 판단과 도구 활용에 어떤 역할을 하는지 연결해 살펴본다. 새로운 실습은 진행하지 않는다.</x:v>
+        <x:v>1일차 온톨로지의 필요성에서 시작해 2일차 클래스·인스턴스·속성·관계·스키마와 그래프 DB, 3일차 SOP·DMN·BSC/KPI의 조치·판단·성과 체계, 4일차 원천 자료 추출·검토·인제스천·출처 관리를 하나의 흐름으로 복습한다. 각 단계의 입력과 결과물, 지식 구조와 실제 데이터의 차이, 판단 규칙과 근거 문서의 관계를 되짚는다. 이렇게 구축된 지식과 규칙이 이후 에이전트의 업무 판단과 도구 활용에 어떤 역할을 하는지 연결해 살펴본다. 새로운 실습은 진행하지 않는다. 검토한 지식은 다음 회차 에이전트가 원인 후보와 점검 순서를 제안할 때 사용하는 근거가 된다.</x:v>
       </x:c>
       <x:c r="D42" s="25" t="n">
         <x:v>30</x:v>
@@ -1619,7 +1617,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="47" s="1" customFormat="1" ht="69" customHeight="1">
+    <x:row r="47" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A47" s="56" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">이론</x:t>
@@ -1631,7 +1629,7 @@
         </x:is>
       </x:c>
       <x:c r="C47" s="53" t="str">
-        <x:v>LLM의 응답 생성, RAG의 근거 검색, Agent의 목표 지향 작업 수행을 구분한다. 요청 해석→계획→도구 선택·호출→결과 관찰→필요 시 재시도→종료의 실행 고리를 살펴보고, 단순 답변과 점검·요청 등 업무 산출물 생성의 차이를 쿨러 사례로 연결한다.</x:v>
+        <x:v>지식 조회 결과를 실제 요청의 답과 점검 제안으로 바꾸고, 근거 없는 단정을 찾아낸다. LLM의 응답 생성, RAG의 근거 검색, Agent의 목표 지향 작업 수행을 구분한다. 요청 해석→계획→도구 선택·호출→결과 관찰→필요 시 재시도→종료의 실행 고리를 살펴보고, 단순 답변과 점검·요청 등 업무 산출물 생성의 차이를 쿨러 사례로 연결한다.</x:v>
       </x:c>
       <x:c r="D47" s="54" t="n">
         <x:v>40</x:v>
@@ -1707,7 +1705,7 @@
         <x:v>45</x:v>
       </x:c>
     </x:row>
-    <x:row r="52" s="1" customFormat="1" ht="60" customHeight="1">
+    <x:row r="52" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A52" s="65" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">실습</x:t>
@@ -1719,7 +1717,7 @@
         </x:is>
       </x:c>
       <x:c r="C52" s="60" t="str">
-        <x:v>기존 HYD 센서 시계열 또는 사전 배포 CSV에서 온도·압력·시간 변화와 상승 구간을 비교하고 도표를 생성한다. 이상 구간·관련 태그·조회 기간을 근거와 함께 요약하되 상관관계로 고장 원인을 단정하지 않는 출력을 점검한다.</x:v>
+        <x:v>기존 HYD 센서 시계열 또는 사전 배포 CSV에서 온도·압력·시간 변화와 상승 구간을 비교하고 도표를 생성한다. 이상 구간·관련 태그·조회 기간을 근거와 함께 요약하되 상관관계로 고장 원인을 단정하지 않는 출력을 점검한다. 다음 회차에는 반복하는 작업 방법을 스킬로 정리하고 필요한 도구를 연결한다.</x:v>
       </x:c>
       <x:c r="D52" s="61" t="n">
         <x:v>40</x:v>
@@ -1771,7 +1769,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="57" s="1" customFormat="1" ht="60" customHeight="1">
+    <x:row r="57" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A57" s="56" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">이론</x:t>
@@ -1783,7 +1781,7 @@
         </x:is>
       </x:c>
       <x:c r="C57" s="53" t="str">
-        <x:v>Agent Skill의 목적, SKILL.md의 작업 목적·호출 조건·입력·출력·순서·예외 지침, SOP의 현장 작업 절차와 에이전트 실행 지침의 차이를 살펴본다. 재사용 지침과 한번의 프롬프트를 구분한다.</x:v>
+        <x:v>앞서 만든 에이전트가 같은 작업을 반복할 수 있도록 지침과 도구의 역할을 구분한다. Agent Skill의 목적, SKILL.md의 작업 목적·호출 조건·입력·출력·순서·예외 지침, SOP의 현장 작업 절차와 에이전트 실행 지침의 차이를 살펴본다. 재사용 지침과 한번의 프롬프트를 구분한다.</x:v>
       </x:c>
       <x:c r="D57" s="54" t="n">
         <x:v>35</x:v>
@@ -1807,7 +1805,7 @@
         <x:v>30</x:v>
       </x:c>
     </x:row>
-    <x:row r="59" s="1" customFormat="1" ht="92" customHeight="1">
+    <x:row r="59" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A59" s="56" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">이론</x:t>
@@ -1819,7 +1817,7 @@
         </x:is>
       </x:c>
       <x:c r="C59" s="53" t="str">
-        <x:v>도구별 읽기/쓰기 권한, 파일 접근 범위, 인증 비밀값, 외부 응답의 불완전성, 실패·타임아웃과 근거 표시를 살펴본다. HYD 포털에서 학생이 등록한 서버는 연결 검사 후 읽기 전용 도구를 선택해 사용하는 범위를 확인한다.</x:v>
+        <x:v>도구별 읽기·쓰기 권한, 파일 접근 범위, 인증 정보, 실패·시간 초과와 근거 표시를 살펴본다. 포털에서 허용된 수업 도구 사용과 로컬 VS Code의 MCP 연결을 구분한다. 포털에 임의 서버를 추가하는 기능은 사용하지 않는다.</x:v>
       </x:c>
       <x:c r="D59" s="54" t="n">
         <x:v>20</x:v>
@@ -1877,7 +1875,7 @@
         <x:v>45</x:v>
       </x:c>
     </x:row>
-    <x:row r="63" s="1" customFormat="1" ht="69" customHeight="1">
+    <x:row r="63" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A63" s="64" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">실습</x:t>
@@ -1889,7 +1887,7 @@
         </x:is>
       </x:c>
       <x:c r="C63" s="53" t="str">
-        <x:v>Notion에서 내보낸 Markdown 학습노트나 제공 매뉴얼로 문항 생성→학생 답변 입력→정답·출처 기반 피드백→다음 문항 제공의 대화를 구성한다. 텍스트 파일 기반으로 우선 완주하며 실서비스 Notion API 연동은 필수로 가정하지 않는다.</x:v>
+        <x:v>Notion에서 내보낸 Markdown 학습노트나 제공 매뉴얼로 문항 생성→학생 답변 입력→정답·출처 기반 피드백→다음 문항 제공의 대화를 구성한다. 텍스트 파일 기반으로 우선 완주하며 실서비스 Notion API 연동은 필수로 가정하지 않는다. 다음 회차에는 정보가 부족한 요청을 질문으로 보완하고 기능 변경의 조건을 명세한다.</x:v>
       </x:c>
       <x:c r="D63" s="54" t="n">
         <x:v>45</x:v>
@@ -1941,7 +1939,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="68" s="1" customFormat="1" ht="60" customHeight="1">
+    <x:row r="68" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A68" s="56" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">이론</x:t>
@@ -1953,7 +1951,7 @@
         </x:is>
       </x:c>
       <x:c r="C68" s="53" t="str">
-        <x:v>HITL의 정의, 자동 처리와 승인·보류·거절의 구분, 승인권자와 권한의 경계, 사람의 책임과 결정 기록을 살펴본다. AI의 자기 검토와 실제 사람 승인 절차는 다른 것임을 구분한다.</x:v>
+        <x:v>앞서 만든 업무 요청 기능이 정보 누락이나 새 요구를 만났을 때 지켜야 할 동작을 정한다. HITL의 정의, 자동 처리와 승인·보류·거절의 구분, 승인권자와 권한의 경계, 사람의 책임과 결정 기록을 살펴본다. AI의 자기 검토와 실제 사람 승인 절차는 다른 것임을 구분한다.</x:v>
       </x:c>
       <x:c r="D68" s="54" t="n">
         <x:v>20</x:v>
@@ -1977,7 +1975,7 @@
         <x:v>20</x:v>
       </x:c>
     </x:row>
-    <x:row r="70" s="1" customFormat="1" ht="69" customHeight="1">
+    <x:row r="70" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A70" s="64" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">실습</x:t>
@@ -1989,7 +1987,7 @@
         </x:is>
       </x:c>
       <x:c r="C70" s="53" t="str">
-        <x:v>5회차에서 만든 후속 업무 요청 결과와 처리 프로젝트를 재사용한다. 해당 업무의 필수 정보가 빠지면 확정하지 않고 확인 질문을 생성하며, 추가 입력 후 다시 판단해 상태 변화를 기록한다.</x:v>
+        <x:v>제공된 5회차 완성 시작본의 후속 업무 요청 결과와 처리 프로젝트를 재사용한다. 해당 업무의 필수 정보가 빠지면 확정하지 않고 확인 질문을 생성하며, 추가 입력 후 다시 판단해 상태 변화를 기록한다.</x:v>
       </x:c>
       <x:c r="D70" s="54" t="n">
         <x:v>45</x:v>
@@ -2047,7 +2045,7 @@
         <x:v>50</x:v>
       </x:c>
     </x:row>
-    <x:row r="74" s="1" customFormat="1" ht="69" customHeight="1">
+    <x:row r="74" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A74" s="64" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">실습</x:t>
@@ -2059,7 +2057,7 @@
         </x:is>
       </x:c>
       <x:c r="C74" s="53" t="str">
-        <x:v>같은 프로젝트의 spec.md에 일반·긴급 요청, 필수 정보 누락 시 보류, 승인 없이 확정 금지, 결과 형식·수용 기준을 명시한다. 구현 후 두 요청을 재실행하고 실제 출력과 명세의 기대 결과를 비교한다.</x:v>
+        <x:v>같은 프로젝트의 spec.md에 일반·긴급 요청, 필수 정보 누락 시 보류, 승인 없이 확정 금지, 결과 형식·수용 기준을 명시한다. 구현 후 두 요청을 재실행하고 실제 출력과 명세의 기대 결과를 비교한다. 이 명세와 출력 사례를 다음 회차에서 실행 가능한 검증 시나리오로 바꾼다.</x:v>
       </x:c>
       <x:c r="D74" s="54" t="n">
         <x:v>25</x:v>
@@ -2111,7 +2109,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="79" s="1" customFormat="1" ht="60" customHeight="1">
+    <x:row r="79" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A79" s="56" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">이론</x:t>
@@ -2123,13 +2121,13 @@
         </x:is>
       </x:c>
       <x:c r="C79" s="53" t="str">
-        <x:v>BDD의 Given/When/Then 구조, 요구 명세(SDD)와 행동 검증(BDD)의 차이, 정상·경계·예외·회귀 테스트를 살펴본다. 자연어 시나리오가 실행 가능한 검증 입력·기대 결과와 연결돼야 하는 이유를 살펴본다.</x:v>
+        <x:v>앞서 정한 명세가 실제 출력에서도 지켜지는지 확인하고 여러 출처를 연결한 결과를 검증한다. BDD의 Given/When/Then 구조, 요구 명세(SDD)와 행동 검증(BDD)의 차이, 정상·경계·예외·회귀 테스트를 살펴본다. 자연어 시나리오가 실행 가능한 검증 입력·기대 결과와 연결돼야 하는 이유를 살펴본다.</x:v>
       </x:c>
       <x:c r="D79" s="54" t="n">
         <x:v>40</x:v>
       </x:c>
     </x:row>
-    <x:row r="80" s="1" customFormat="1" ht="60" customHeight="1">
+    <x:row r="80" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A80" s="65" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">실습</x:t>
@@ -2141,7 +2139,7 @@
         </x:is>
       </x:c>
       <x:c r="C80" s="60" t="str">
-        <x:v>7일차 spec.md와 동일 에이전트를 활용한다. 일반 정비, 긴급 정비, 필수 정보 누락, 승인 거절, 도구 오류에 대해 Given·When·Then과 입력값·기대 상태·출력 계약을 작성한다.</x:v>
+        <x:v>제공된 7일차 시작본의 spec.md와 동일 에이전트를 활용한다. 일반 정비, 긴급 정비, 필수 정보 누락, 승인 거절, 도구 오류에 대해 Given·When·Then과 입력값·기대 상태·출력 계약을 작성한다.</x:v>
       </x:c>
       <x:c r="D80" s="61" t="n">
         <x:v>40</x:v>
@@ -2201,7 +2199,7 @@
         <x:v>45</x:v>
       </x:c>
     </x:row>
-    <x:row r="84" s="1" customFormat="1" ht="60" customHeight="1">
+    <x:row r="84" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A84" s="63" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">이론</x:t>
@@ -2213,7 +2211,7 @@
         </x:is>
       </x:c>
       <x:c r="C84" s="60" t="str">
-        <x:v>에이전트의 목표와 도구, Skill·MCP의 구분, HITL, SDD·BDD와 회귀 검증, 응용별 산출물의 차이를 복습한다. 신규 실습·과제 없이 배운 내용을 정리한다.</x:v>
+        <x:v>에이전트의 목표와 도구, Skill·MCP의 구분, HITL, SDD·BDD와 회귀 검증, 응용별 산출물의 차이를 복습한다. 신규 실습·과제 없이 배운 내용을 정리한다. 다음 회차에는 검증한 작업을 사람의 승인과 함께 하나의 BPMN 흐름으로 표현한다.</x:v>
       </x:c>
       <x:c r="D84" s="61" t="n">
         <x:v>30</x:v>
@@ -2265,7 +2263,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="89" s="1" customFormat="1" ht="69" customHeight="1">
+    <x:row r="89" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A89" s="56" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">이론</x:t>
@@ -2277,7 +2275,7 @@
         </x:is>
       </x:c>
       <x:c r="C89" s="53" t="str">
-        <x:v>비즈니스 프로세스의 정의, Task와 End-to-End의 차이, 시작 조건·입력·출력·책임자·완료 조건을 살펴본다. BPM의 분석→설계→실행→모니터링→개선과 AS-IS/TO-BE를 다루고 에이전트만으로 전체 업무 순서와 책임이 보장되지 않는 이유를 연결한다.</x:v>
+        <x:v>개별 에이전트의 답을 넘어서 작업 순서·담당자·승인·완료를 하나의 흐름으로 표현한다. 비즈니스 프로세스의 정의, Task와 End-to-End의 차이, 시작 조건·입력·출력·책임자·완료 조건을 살펴본다. BPM의 분석→설계→실행→모니터링→개선과 AS-IS/TO-BE를 다루고 에이전트만으로 전체 업무 순서와 책임이 보장되지 않는 이유를 연결한다.</x:v>
       </x:c>
       <x:c r="D89" s="54" t="n">
         <x:v>35</x:v>
@@ -2371,7 +2369,7 @@
         <x:v>40</x:v>
       </x:c>
     </x:row>
-    <x:row r="95" s="1" customFormat="1" ht="69" customHeight="1">
+    <x:row r="95" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A95" s="64" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">실습</x:t>
@@ -2383,7 +2381,7 @@
         </x:is>
       </x:c>
       <x:c r="C95" s="53" t="str">
-        <x:v>포털에 이미 등록된 설비 대응 흐름을 쿨러 열화 시나리오로 실행한다. 에이전트 판단→운전원 승인→설비 명령→재관측→완료 기록을 따라간다. 승인 대기와 반려 결과를 비교하고, 자신이 그린 BPMN의 작업·분기와 실행 이력을 대조한다.</x:v>
+        <x:v>포털에 이미 등록된 설비 대응 흐름을 쿨러 열화 시나리오로 실행한다. 에이전트 판단→운전원 승인→설비 명령→재관측→완료 기록을 따라간다. 승인 대기와 반려 결과를 비교하고, 자신이 그린 BPMN의 작업·분기와 실행 이력을 대조한다. 이 승인·반려 패턴을 다음 회차의 정기 점검과 재고 보충 흐름에 적용한다.</x:v>
       </x:c>
       <x:c r="D95" s="54" t="n">
         <x:v>35</x:v>
@@ -2435,7 +2433,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="100" s="1" customFormat="1" ht="69" customHeight="1">
+    <x:row r="100" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A100" s="56" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">이론</x:t>
@@ -2447,7 +2445,7 @@
         </x:is>
       </x:c>
       <x:c r="C100" s="53" t="str">
-        <x:v>설비 경보, 정기 점검 도래, 재고 부족이라는 시작 조건과 에이전트·승인자·실행 시스템의 차이를 비교한다. 프로세스 정의·인스턴스·배포, 대기와 완료 상태, 실행 기록·모니터링·병목·지표를 설명하고 같은 BPMN 패턴의 재사용 원리를 정리한다.</x:v>
+        <x:v>앞서 익힌 승인 흐름을 정비와 구매에 적용하며 시작 조건과 처리 결과의 차이를 비교한다. 설비 경보, 정기 점검 도래, 재고 부족이라는 시작 조건과 에이전트·승인자·실행 시스템의 차이를 비교한다. 프로세스 정의·인스턴스·배포, 대기와 완료 상태, 실행 기록·모니터링·병목·지표를 설명하고 같은 BPMN 패턴의 재사용 원리를 정리한다.</x:v>
       </x:c>
       <x:c r="D100" s="54" t="n">
         <x:v>35</x:v>
@@ -2525,7 +2523,7 @@
         <x:v>40</x:v>
       </x:c>
     </x:row>
-    <x:row r="105" s="1" customFormat="1" ht="60" customHeight="1">
+    <x:row r="105" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A105" s="63" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">이론</x:t>
@@ -2537,7 +2535,7 @@
         </x:is>
       </x:c>
       <x:c r="C105" s="60" t="str">
-        <x:v>설비 조치·정기 점검·재고 보충의 시작 이벤트, 에이전트 판단, 사람 승인·반려, 시스템 처리와 종료 기록을 되짚는다. 온톨로지→에이전트→프로세스의 연결을 복습하며 새로운 실습은 하지 않는다.</x:v>
+        <x:v>설비 조치·정기 점검·재고 보충의 시작 이벤트, 에이전트 판단, 사람 승인·반려, 시스템 처리와 종료 기록을 되짚는다. 온톨로지→에이전트→프로세스의 연결을 복습하며 새로운 실습은 하지 않는다. 다음 회차에는 설비·정비·재고 기록을 교대 인계안으로 묶고 사람이 검토·확인하는 흐름을 완성한다.</x:v>
       </x:c>
       <x:c r="D105" s="61" t="n">
         <x:v>30</x:v>
@@ -2587,7 +2585,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="110" s="1" customFormat="1" ht="69" customHeight="1">
+    <x:row r="110" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A110" s="56" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">이론</x:t>
@@ -2599,7 +2597,7 @@
         </x:is>
       </x:c>
       <x:c r="C110" s="53" t="str">
-        <x:v>설비·센서·고장 관계를 정의하는 클래스·인스턴스·스키마, 그래프 질의, SOP·DMN·BSC/KPI, 문서 인제스천과 출처, 정적 지식과 현재 DB 값의 구분을 되짚는다. 앞선 영역 Wrap-up의 단순 반복보다 에이전트 입력으로 연결되는 구조를 중심으로 정리한다.</x:v>
+        <x:v>그동안 만든 지식·에이전트·업무 흐름을 교대 인수인계 한 건에 연결한다. 설비·센서·고장 관계를 정의하는 클래스·인스턴스·스키마, 그래프 질의, SOP·DMN·BSC/KPI, 문서 인제스천과 출처, 정적 지식과 현재 DB 값의 구분을 되짚는다. 앞선 영역 Wrap-up의 단순 반복보다 에이전트 입력으로 연결되는 구조를 중심으로 정리한다.</x:v>
       </x:c>
       <x:c r="D110" s="54" t="n">
         <x:v>30</x:v>
@@ -2705,7 +2703,7 @@
         <x:v>40</x:v>
       </x:c>
     </x:row>
-    <x:row r="117" s="1" customFormat="1" ht="69" customHeight="1">
+    <x:row r="117" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A117" s="65" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">실습</x:t>
@@ -2717,7 +2715,7 @@
         </x:is>
       </x:c>
       <x:c r="C117" s="60" t="str">
-        <x:v>첫날 준비한 Notion 학습노트에 개념·참고 자료·실습 산출물·검증 결과를 연결해 기록한다. 수업 계정에서 Notion 연결과 쓰기 권한이 검증된 경우 MCP 연동을 시연하고, 미연결 환경에서는 준비한 Markdown을 Notion에 직접 정리한다.</x:v>
+        <x:v>첫날 준비한 Notion 학습노트에 개념·참고 자료·실습 산출물·검증 결과를 연결해 기록한다. 수업 계정에서 Notion 연결과 쓰기 권한이 검증된 경우 MCP 연동을 시연하고, 미연결 환경에서는 준비한 Markdown을 Notion에 직접 정리한다. 관계 모델·판단 근거·명세·검증 결과·인계 기록을 함께 찾아볼 수 있게 정리하며 과정을 마친다.</x:v>
       </x:c>
       <x:c r="D117" s="61" t="n">
         <x:v>20</x:v>
@@ -2872,7 +2870,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="6" s="1" customFormat="1" ht="60" customHeight="1">
+    <x:row r="6" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A6" s="56" t="str">
         <x:v>이론</x:v>
       </x:c>
@@ -2880,7 +2878,7 @@
         <x:v>학습 내용을 지식 자산으로 전환하는 방법 이해하기</x:v>
       </x:c>
       <x:c r="C6" s="53" t="str">
-        <x:v>단순히 내용을 기록하는 것과 나중에 다시 찾아 활용할 수 있는 지식 자산으로 축적하는 것의 차이를 이해한다. 학습한 개념, 핵심 원리, 참고 자료와 출처, 실습 과정 및 결과를 체계적으로 연결해 기록하는 이유를 배운다. Notion을 활용해 수업이 끝난 뒤에도 지식을 검색·보완·재사용할 수 있는 개인 학습 체계를 마련하는 목적을 살펴본다.</x:v>
+        <x:v>HYD의 전체 흐름을 보고 이후 실습에서 만들 지식·에이전트·업무 연결의 목표를 확인한다. 단순히 내용을 기록하는 것과 나중에 다시 찾아 활용할 수 있는 지식 자산으로 축적하는 것의 차이를 이해한다. 학습한 개념, 핵심 원리, 참고 자료와 출처, 실습 과정 및 결과를 체계적으로 연결해 기록하는 이유를 배운다. Notion을 활용해 수업이 끝난 뒤에도 지식을 검색·보완·재사용할 수 있는 개인 학습 체계를 마련하는 목적을 살펴본다.</x:v>
       </x:c>
       <x:c r="D6" s="54" t="n">
         <x:v>10</x:v>
@@ -2956,7 +2954,7 @@
         <x:v>50</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" s="1" customFormat="1" ht="60" customHeight="1">
+    <x:row r="12" s="1" customFormat="1" ht="118" customHeight="1">
       <x:c r="A12" s="64" t="str">
         <x:v>실습</x:v>
       </x:c>
@@ -2964,7 +2962,7 @@
         <x:v>설비 이상과 원인·조치의 관계를 시각화하기</x:v>
       </x:c>
       <x:c r="C12" s="53" t="str">
-        <x:v>arrows.app의 노드·관계·레이블 작성 방법을 익힌다. 간단한 설비 이상 사례를 바탕으로 설비·센서·증상·원인·조치를 배치하고 각각의 연결 관계를 직접 그린다. 어떤 대상이 다른 대상과 연결되는지, 관계의 방향을 어떻게 표현하는지 살펴본다. 완성한 관계도를 통해 단순히 정보를 나열하는 방식과 관계를 중심으로 표현하는 방식의 차이를 확인한다. 복잡한 온톨로지 스키마와 제약은 다음 학습에서 다룬다.</x:v>
+        <x:v>arrows.app의 노드·관계·레이블 작성 방법을 익힌다. 간단한 설비 이상 사례를 바탕으로 설비·센서·증상·원인·조치를 배치하고 각각의 연결 관계를 직접 그린다. 어떤 대상이 다른 대상과 연결되는지, 관계의 방향을 어떻게 표현하는지 살펴본다. 완성한 관계도를 통해 단순히 정보를 나열하는 방식과 관계를 중심으로 표현하는 방식의 차이를 확인한다. 복잡한 온톨로지 스키마와 제약은 다음 학습에서 다룬다. 이 관계를 다음 회차에서 식별자와 속성을 갖춘 모델로 옮겨 실제 질의로 확인한다.</x:v>
       </x:c>
       <x:c r="D12" s="54" t="n">
         <x:v>30</x:v>
@@ -3021,7 +3019,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="17" s="1" customFormat="1" ht="60" customHeight="1">
+    <x:row r="17" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A17" s="56" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">이론</x:t>
@@ -3033,13 +3031,13 @@
         </x:is>
       </x:c>
       <x:c r="C17" s="53" t="str">
-        <x:v>클래스·인스턴스·속성·관계, 관계 방향, 카디널리티를 HYD 설비와 센서 실례로 살펴본다. 같은 종류의 설비와 실제 설비 1대를 구별한다.</x:v>
+        <x:v>관계도에서 부품이 쓰이는 설비와 공급 정보를 찾고, 작업 조건을 판단에 쓸 수 있는 형태로 바꾼다. 클래스·인스턴스·속성·관계, 관계 방향, 카디널리티를 HYD 설비와 센서 실례로 살펴본다. 같은 종류의 설비와 실제 설비 1대를 구별한다.</x:v>
       </x:c>
       <x:c r="D17" s="54" t="n">
         <x:v>25</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" s="1" customFormat="1" ht="60" customHeight="1">
+    <x:row r="18" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A18" s="63" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">이론</x:t>
@@ -3051,7 +3049,7 @@
         </x:is>
       </x:c>
       <x:c r="C18" s="60" t="str">
-        <x:v>고유 식별자, 자료형, 필수값, 레이블, 노드 간 관계·제약, 스키마와 인스턴스의 역할 차이를 살펴본다. 중복 부품 명칭과 동일 설비 구분 문제를 예로 든다.</x:v>
+        <x:v>고유 식별자, 자료형, 필수값, 레이블, 노드 간 관계·제약, 스키마와 인스턴스의 역할 차이를 살펴본다. 중복 부품 명칭과 고유 식별자로 대상을 구분한 결과를 비교한다.</x:v>
       </x:c>
       <x:c r="D18" s="61" t="n">
         <x:v>20</x:v>
@@ -3159,7 +3157,7 @@
         <x:v>35</x:v>
       </x:c>
     </x:row>
-    <x:row r="25" s="1" customFormat="1" ht="60" customHeight="1">
+    <x:row r="25" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A25" s="64" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">실습</x:t>
@@ -3169,7 +3167,7 @@
         <x:v>작업 기준의 복합 조건과 예외를 조치 조건표로 표현하기</x:v>
       </x:c>
       <x:c r="C25" s="53" t="str">
-        <x:v>제공 SOP에서 경고·감점·제외를 구분해 입력·단위·연산자·경계·출력·출처를 조건표로 작성한다. 복수 사유를 함께 남기고, 입력 누락이 있어도 확인된 제외 근거는 보존한다. 후보 유지와 실행 승인을 구별한다.</x:v>
+        <x:v>제공 SOP에서 경고·감점·제외를 구분해 입력·단위·연산자·경계·출력·출처를 조건표로 작성한다. 복수 사유를 함께 남기고, 입력 누락이 있어도 확인된 제외 근거는 보존한다. 후보 유지와 실행 승인을 구별한다. 다음 회차에는 이 조건표로 조치 검토 결과를 만들고 매뉴얼 근거를 연결한다.</x:v>
       </x:c>
       <x:c r="D25" s="54" t="n">
         <x:v>40</x:v>
@@ -3226,7 +3224,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="30" s="1" customFormat="1" ht="60" customHeight="1">
+    <x:row r="30" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A30" s="56" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">이론</x:t>
@@ -3238,7 +3236,7 @@
         </x:is>
       </x:c>
       <x:c r="C30" s="53" t="str">
-        <x:v>BSC 4관점과 전략 목표·KPI의 역할, 안전을 만족한 후보 사이에서 예상 비용·생산 영향·품질·에너지 측면을 비교하는 이유, What-if 분석의 개념을 살펴본다.</x:v>
+        <x:v>조건표에 따른 조치 선택과 문서의 원문 근거를 연결해 검토 결과와 작업 확인 카드를 만든다. BSC 4관점과 전략 목표·KPI의 역할, 안전을 만족한 후보 사이에서 예상 비용·생산 영향·품질·에너지 측면을 비교하는 이유, What-if 분석의 개념을 살펴본다.</x:v>
       </x:c>
       <x:c r="D30" s="54" t="n">
         <x:v>20</x:v>
@@ -3302,10 +3300,8 @@
           <x:t xml:space="preserve">실습</x:t>
         </x:is>
       </x:c>
-      <x:c r="B34" s="55" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">현장 매뉴얼을 검토해 근거 있는 지식으로 등록하기</x:t>
-        </x:is>
+      <x:c r="B34" s="55" t="str">
+        <x:v>매뉴얼 근거를 대조하고 작업 확인 항목 정리하기</x:v>
       </x:c>
       <x:c r="C34" s="53" t="str">
         <x:v>제공 매뉴얼의 원문과 포털에 등록된 추출·검토 결과를 나란히 확인한다. 작업 순서·단위·금지 조건·대상 설비를 비교하고 수정하거나 제외할 후보를 표시한다. 지식 지도에서 채택된 항목의 설비·조치·출처 연결을 찾는다. 직접 추가 적재는 마지막 교대 실습에서 제공 보충 매뉴얼로 수행한다. 선택한 작업에 필요한 준비·금지·완료 조건을 원문 근거와 함께 정리한다.</x:v>
@@ -3346,7 +3342,7 @@
         <x:v>35</x:v>
       </x:c>
     </x:row>
-    <x:row r="37" s="1" customFormat="1" ht="60" customHeight="1">
+    <x:row r="37" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A37" s="63" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">이론</x:t>
@@ -3358,7 +3354,7 @@
         </x:is>
       </x:c>
       <x:c r="C37" s="60" t="str">
-        <x:v>온톨로지 WHY→클래스·스키마→그래프 DB→SOP·DMN→BSC·KPI→매뉴얼 인제스천의 역할과 다음 에이전트 학습으로 이어지는 지식 자산을 복습한다. 신규 실습 없음.</x:v>
+        <x:v>온톨로지 WHY→클래스·스키마→그래프 DB→SOP·DMN→BSC·KPI→매뉴얼 인제스천의 역할과 다음 에이전트 학습으로 이어지는 지식 자산을 복습한다. 신규 실습 없음. 검토한 근거와 확인 항목은 다음 회차 점검 요청을 작성하는 에이전트의 입력으로 활용한다.</x:v>
       </x:c>
       <x:c r="D37" s="61" t="n">
         <x:v>30</x:v>
@@ -3415,7 +3411,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="42" s="1" customFormat="1" ht="60" customHeight="1">
+    <x:row r="42" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A42" s="56" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">이론</x:t>
@@ -3427,7 +3423,7 @@
         </x:is>
       </x:c>
       <x:c r="C42" s="53" t="str">
-        <x:v>LLM·RAG·Agent의 목표·도구·반복 실행 차이, 온톨로지·업무 DB·SOP를 근거로 선택하는 과정과 실패 시 확인해야 할 실행 기록을 사례로 살펴본다.</x:v>
+        <x:v>설비·문서 근거를 점검 요청으로 연결하고 반복하는 후속 업무를 스킬과 도구로 처리한다. LLM·RAG·Agent의 목표·도구·반복 실행 차이, 온톨로지·업무 DB·SOP를 근거로 선택하는 과정과 실패 시 확인해야 할 실행 기록을 사례로 살펴본다.</x:v>
       </x:c>
       <x:c r="D42" s="54" t="n">
         <x:v>30</x:v>
@@ -3517,7 +3513,7 @@
         <x:v>25</x:v>
       </x:c>
     </x:row>
-    <x:row r="48" s="1" customFormat="1" ht="69" customHeight="1">
+    <x:row r="48" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A48" s="64" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">실습</x:t>
@@ -3527,7 +3523,7 @@
         <x:v>파일·Git·시간 도구로 다음 협의 안건 만들기</x:v>
       </x:c>
       <x:c r="C48" s="53" t="str">
-        <x:v>공통 HYD 읽기 도구 연결을 확인하고 준비된 파일·Git·시간 MCP를 VS Code에서 호출한다. 앞 업무 목록과 변경 이력을 연결해 완료·미결·변경 내용 및 다음 확인 안건을 생성한다. 원자료와 대조해 로컬 파일로 저장한다. 새 서버나 외부 계정 연동은 만들지 않는다.</x:v>
+        <x:v>공통 HYD 읽기 도구 연결을 확인하고 준비된 파일·Git·시간 MCP를 VS Code에서 호출한다. 앞 업무 목록과 변경 이력을 연결해 완료·미결·변경 내용 및 다음 확인 안건을 생성한다. 원자료와 대조해 로컬 파일로 저장한다. 새 서버나 외부 계정 연동은 만들지 않는다. 다음 회차에는 점검 요청의 정보 누락을 질문으로 보완하고 기능 변경 전후의 동작을 검증한다.</x:v>
       </x:c>
       <x:c r="D48" s="54" t="n">
         <x:v>45</x:v>
@@ -3584,7 +3580,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="53" s="1" customFormat="1" ht="60" customHeight="1">
+    <x:row r="53" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A53" s="56" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">이론</x:t>
@@ -3596,7 +3592,7 @@
         </x:is>
       </x:c>
       <x:c r="C53" s="53" t="str">
-        <x:v>HITL의 승인·보류·거절, 역할별 책임·감사 기록, AI의 자체 검토와 사람 결정의 차이를 살펴본다.</x:v>
+        <x:v>점검 요청을 바로 확정할 수 없는 경우를 구분하고, 새 요구를 반영해도 기존 조건을 지키게 한다. HITL의 승인·보류·거절, 역할별 책임·감사 기록, AI의 자체 검토와 사람 결정의 차이를 살펴본다.</x:v>
       </x:c>
       <x:c r="D53" s="54" t="n">
         <x:v>20</x:v>
@@ -3620,7 +3616,7 @@
         <x:v>15</x:v>
       </x:c>
     </x:row>
-    <x:row r="55" s="1" customFormat="1" ht="60" customHeight="1">
+    <x:row r="55" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A55" s="64" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">실습</x:t>
@@ -3630,7 +3626,7 @@
         <x:v>점검 요청의 부족한 정보를 질문하고 재개하기</x:v>
       </x:c>
       <x:c r="C55" s="53" t="str">
-        <x:v>4회차 점검 요청 초안 프로젝트의 필수 입력과 완료 기준을 정한다. 누락 시 보류·질문·추가 답변 반영·재판단을 구현하고 근거와 처리 상태를 보존한다. 사람 승인이 필요한 결과를 자동 확정하지 않는다.</x:v>
+        <x:v>제공된 4회차 점검 요청 시작본의 필수 입력과 완료 기준을 정한다. 누락 시 보류·질문·추가 답변 반영·재판단을 구현하고 근거와 처리 상태를 보존한다. 사람 승인이 필요한 결과를 자동 확정하지 않는다.</x:v>
       </x:c>
       <x:c r="D55" s="54" t="n">
         <x:v>35</x:v>
@@ -3704,7 +3700,7 @@
         <x:v>40</x:v>
       </x:c>
     </x:row>
-    <x:row r="60" s="1" customFormat="1" ht="60" customHeight="1">
+    <x:row r="60" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A60" s="63" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">이론</x:t>
@@ -3716,7 +3712,7 @@
         </x:is>
       </x:c>
       <x:c r="C60" s="60" t="str">
-        <x:v>Agent·Skill·MCP·HITL·SDD·BDD가 각각 해결하는 문제와 구현 산출물을 복습하고 BPMN 업무 연결을 예고한다. 새로운 실습 없음.</x:v>
+        <x:v>Agent·Skill·MCP·HITL·SDD·BDD가 각각 해결하는 문제와 구현 산출물을 복습하고 BPMN 업무 연결을 예고한다. 새로운 실습 없음. 검증한 개별 작업을 다음 회차에서 사람의 승인과 연결한 BPMN 흐름으로 표현한다.</x:v>
       </x:c>
       <x:c r="D60" s="61" t="n">
         <x:v>30</x:v>
@@ -3773,7 +3769,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="65" s="1" customFormat="1" ht="60" customHeight="1">
+    <x:row r="65" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A65" s="56" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">이론</x:t>
@@ -3785,7 +3781,7 @@
         </x:is>
       </x:c>
       <x:c r="C65" s="53" t="str">
-        <x:v>End-to-End 업무, 시작·입력·담당·완료와 BPM의 분석·설계·실행·모니터링·개선, 에이전트의 단일 작업과 오케스트레이션의 전체 흐름 책임을 살펴본다.</x:v>
+        <x:v>개별 판단이 실제 조치로 이어지려면 어떤 역할·승인·실행 연결이 필요한지 흐름과 기록을 대조한다. End-to-End 업무, 시작·입력·담당·완료와 BPM의 분석·설계·실행·모니터링·개선, 에이전트의 단일 작업과 오케스트레이션의 전체 흐름 책임을 살펴본다.</x:v>
       </x:c>
       <x:c r="D65" s="54" t="n">
         <x:v>20</x:v>
@@ -3931,7 +3927,7 @@
         <x:v>25</x:v>
       </x:c>
     </x:row>
-    <x:row r="74" s="1" customFormat="1" ht="92" customHeight="1">
+    <x:row r="74" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A74" s="65" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">실습</x:t>
@@ -3943,7 +3939,7 @@
         </x:is>
       </x:c>
       <x:c r="C74" s="60" t="str">
-        <x:v>포털에 이미 등록된 설비 대응 흐름을 쿨러 열화 시나리오로 실행한다. 에이전트 판단→운전원 승인→설비 명령→재관측→완료 기록을 따라간다. 승인 대기와 반려 결과를 비교하고, 자신이 그린 BPMN의 작업·분기와 실행 이력을 대조한다. 명령이 실행된 시점과 그 전에 필요한 승인·근거를 실행 기록에서 짚는다.</x:v>
+        <x:v>포털에 이미 등록된 설비 대응 흐름을 쿨러 열화 시나리오로 실행한다. 에이전트 판단→운전원 승인→설비 명령→재관측→완료 기록을 따라간다. 승인 대기와 반려 결과를 비교하고, 자신이 그린 BPMN의 작업·분기와 실행 이력을 대조한다. 명령이 실행된 시점과 그 전에 필요한 승인·근거를 실행 기록에서 짚는다. 같은 패턴을 다음 회차 정비·구매에 적용하고 업무별 완료 결과를 비교한다.</x:v>
       </x:c>
       <x:c r="D74" s="61" t="n">
         <x:v>20</x:v>
@@ -4000,7 +3996,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="79" s="1" customFormat="1" ht="92" customHeight="1">
+    <x:row r="79" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A79" s="56" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">이론</x:t>
@@ -4012,7 +4008,7 @@
         </x:is>
       </x:c>
       <x:c r="C79" s="53" t="str">
-        <x:v>정기 점검 도래와 재고 부족 시작 이벤트, 승인자·시스템 차이, 프로세스 정의 재사용·인스턴스 상태·배포·오류·반려 기록을 사례로 살펴본다.</x:v>
+        <x:v>설비 제어와 정비·구매 처리가 끝나는 지점을 구분하고 각 결과를 실행 기록에서 확인한다. 정기 점검 도래와 재고 부족 시작 이벤트, 승인자·시스템 차이, 프로세스 정의 재사용·인스턴스 상태·배포·오류·반려 기록을 사례로 살펴본다.</x:v>
       </x:c>
       <x:c r="D79" s="54" t="n">
         <x:v>20</x:v>
@@ -4090,7 +4086,7 @@
         <x:v>45</x:v>
       </x:c>
     </x:row>
-    <x:row r="84" s="1" customFormat="1" ht="60" customHeight="1">
+    <x:row r="84" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A84" s="63" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">이론</x:t>
@@ -4102,7 +4098,7 @@
         </x:is>
       </x:c>
       <x:c r="C84" s="60" t="str">
-        <x:v>BPMN 모델, 엔진의 정의·인스턴스, 이벤트·에이전트·사람·시스템의 역할과 온톨로지부터 프로세스까지의 학습 연결을 복습한다. 신규 실습 없음.</x:v>
+        <x:v>BPMN 모델, 엔진의 정의·인스턴스, 이벤트·에이전트·사람·시스템의 역할과 온톨로지부터 프로세스까지의 학습 연결을 복습한다. 신규 실습 없음. 다음 회차에는 이 기록의 미완료·불일치를 인계안으로 모아 사람의 검토·확인까지 연결한다.</x:v>
       </x:c>
       <x:c r="D84" s="61" t="n">
         <x:v>30</x:v>
@@ -4157,7 +4153,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="89" s="1" customFormat="1" ht="60" customHeight="1">
+    <x:row r="89" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A89" s="56" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">이론</x:t>
@@ -4169,7 +4165,7 @@
         </x:is>
       </x:c>
       <x:c r="C89" s="53" t="str">
-        <x:v>온톨로지·스키마·그래프·SOP·DMN·BSC/KPI·매뉴얼 인제스천에서 만든 공용 지식이 에이전트 도구 조회로 어떻게 쓰이는지 되짚는다.</x:v>
+        <x:v>지식·도구·에이전트·승인 흐름을 교대 인수인계 한 건에 연결하여 결과와 근거를 확인한다. 온톨로지·스키마·그래프·SOP·DMN·BSC/KPI·매뉴얼 인제스천에서 만든 공용 지식이 에이전트 도구 조회로 어떻게 쓰이는지 되짚는다.</x:v>
       </x:c>
       <x:c r="D89" s="54" t="n">
         <x:v>30</x:v>
@@ -4275,7 +4271,7 @@
         <x:v>40</x:v>
       </x:c>
     </x:row>
-    <x:row r="96" s="1" customFormat="1" ht="60" customHeight="1">
+    <x:row r="96" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A96" s="65" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">실습</x:t>
@@ -4287,7 +4283,7 @@
         </x:is>
       </x:c>
       <x:c r="C96" s="60" t="str">
-        <x:v>Notion 학습노트에 핵심 개념·실습 결과·참고 출처를 연결한다. 수업 환경에서 사용 가능한 경우 MCP로 기록을 반영하고, 그렇지 않은 경우 작성한 Markdown을 직접 붙여 학습노트를 완성한다.</x:v>
+        <x:v>Notion 학습노트에 핵심 개념·실습 결과·참고 출처를 연결한다. 수업 환경에서 사용 가능한 경우 MCP로 기록을 반영하고, 그렇지 않은 경우 작성한 Markdown을 직접 붙여 학습노트를 완성한다. 조회·판단·검토·실행 확인에 사용한 자료와 산출물을 연결해 이후에도 다시 활용할 수 있게 정리한다.</x:v>
       </x:c>
       <x:c r="D96" s="61" t="n">
         <x:v>20</x:v>
@@ -4791,15 +4787,15 @@
   <x:sheetData>
     <x:row r="1" s="1" customFormat="1" ht="38" customHeight="1">
       <x:c r="A1" s="137" t="str">
-        <x:v>HYD 제조 AI | 통합반 오프라인 정규 10회 | 50분 수업 단위</x:v>
+        <x:v>HYD 제조 AI | 통합반 오프라인 정규 10회 | 수업 계획</x:v>
       </x:c>
       <x:c r="B1" s="137"/>
       <x:c r="C1" s="137"/>
       <x:c r="D1" s="137"/>
     </x:row>
-    <x:row r="2" s="1" customFormat="1" ht="38" customHeight="1">
+    <x:row r="2" s="1" customFormat="1" ht="48" customHeight="1">
       <x:c r="A2" s="135" t="str">
-        <x:v>온라인 실습에서 주요 활동을 선별해 직접 수행합니다. 기본 편성은 수업200분·휴식40분이며, 강사가 학생 진행에 따라 시간을 조절합니다. 이론이 있는 회차는50분, 마지막 두 회차는 실습 중심입니다.</x:v>
+        <x:v>온라인 선행학습 후 목적·핵심 개념을 연결하고 주요 실습을 직접 수행합니다. 수업200분·휴식40분의 기본 배정이며 실제 진행은 강사가 조절합니다. 이전 개인 결과 없이 제공 시작본으로 시작할 수 있습니다.</x:v>
       </x:c>
       <x:c r="B2" s="135"/>
       <x:c r="C2" s="135"/>
@@ -4813,7 +4809,7 @@
     </x:row>
     <x:row r="4" s="1" customFormat="1" ht="38" customHeight="1">
       <x:c r="A4" s="138" t="str">
-        <x:v>01회차 | 설비 정보를 관계와 모델로 표현하기</x:v>
+        <x:v>01회차 | HYD 전체 흐름을 확인하고 설비 관계 표현하기</x:v>
       </x:c>
       <x:c r="B4" s="138"/>
       <x:c r="C4" s="138"/>
@@ -4833,32 +4829,32 @@
         <x:v>시간(분)</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" s="1" customFormat="1" ht="92" customHeight="1">
+    <x:row r="6" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A6" s="141" t="str">
         <x:v>이론</x:v>
       </x:c>
       <x:c r="B6" s="141" t="str">
-        <x:v>설비 정보와 관계 모델 이해하기</x:v>
+        <x:v>HYD 시스템과 이번 과정의 학습 목표 이해하기</x:v>
       </x:c>
       <x:c r="C6" s="141" t="str">
-        <x:v>설비·센서·부품이 각각 어떤 정보를 나타내는지 구분한다. 쿨러의 온도 변화가 센서 값, 이상 징후, 원인 후보, 조치 판단으로 이어지는 경로를 살펴본다. 같은 종류와 개별 대상을 클래스·인스턴스로 나누고, 식별자·속성·관계 방향을 설비 사례에 적용한다.</x:v>
+        <x:v>HYD의 완성 흐름을 먼저 확인하고, 판단 근거를 표현하는 관계도와 그래프를 직접 다룬다. HYD가 유압 설비와 업무 시스템을 연결한 수업용 시스템임을 이해한다. 설비·센서 데이터 수집→상태 관찰→지식에 근거한 판단→사람 승인→조치→결과 확인의 전체 구조를 살펴본다. 포털에서 확인할 설비 화면·지식 지도·에이전트·작업함의 역할을 구분한다. 이번 과정에서 관계 모델을 만들고, 근거를 조회하는 에이전트와 업무 흐름으로 연결할 학습 목표를 확인한다.</x:v>
       </x:c>
       <x:c r="D6" s="142" t="n">
-        <x:v>50</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" s="1" customFormat="1" ht="92" customHeight="1">
+        <x:v>40</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" s="1" customFormat="1" ht="125" customHeight="1">
       <x:c r="A7" s="143" t="str">
         <x:v>실습</x:v>
       </x:c>
       <x:c r="B7" s="143" t="str">
-        <x:v>관계도를 그리고 최소 모델 만들기</x:v>
+        <x:v>포털 시연으로 완성 흐름을 확인하고 관계도 그리기</x:v>
       </x:c>
       <x:c r="C7" s="143" t="str">
-        <x:v>arrows.app에서 쿨러·센서·부품·고장·조치를 노드로 만들고 관계를 연결한다. 각 화살표를 문장으로 읽어 방향을 확인한다. 제공 목록과 관계도를 대조해 클래스·고유 ID·속성을 갖춘 schema.json과 예시 인스턴스를 작성한다.</x:v>
+        <x:v>강사가 실제 HYD 포털을 열어 보여 주는 설비 상태·센서 값과 쿨러 열화 시나리오를 따라간다. 경보 발생→에이전트의 원인·조치 추천→운전원 승인→설비 명령→센서 값 재확인과 완료 기록을 보고, 추천·승인·실행의 차이를 구분한다. 지식 지도에서 판단에 사용된 설비·센서·고장·조치 연결을 확인한다. 이어 arrows.app에서 방금 본 대상을 노드와 관계로 그려 각 화살표를 문장으로 읽는다.</x:v>
       </x:c>
       <x:c r="D7" s="144" t="n">
-        <x:v>50</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="8" s="1" customFormat="1" ht="92" customHeight="1">
@@ -4875,15 +4871,15 @@
         <x:v>50</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" s="1" customFormat="1" ht="92" customHeight="1">
+    <x:row r="9" s="1" customFormat="1" ht="150" customHeight="1">
       <x:c r="A9" s="143" t="str">
         <x:v>실습</x:v>
       </x:c>
       <x:c r="B9" s="143" t="str">
-        <x:v>설비 모델을 적재하고 질문별 결과 확인하기</x:v>
+        <x:v>관계도를 설비 모델로 옮기고 적재·조회 결과 확인하기</x:v>
       </x:c>
       <x:c r="C9" s="143" t="str">
-        <x:v>작성한 설비 모델을 제공 절차로 별도 랩 DB에 적재한다. 설비의 센서·부품을 조회해 원자료와 비교하고 빠진 관계·식별자를 수정한다. 포털 기준 지도를 열어 자신의 모델과 연결 방향을 비교한다. 관계도·모델·조회 결과를 저장한다.</x:v>
+        <x:v>VS Code에서 탐색기의 자료 위치와 터미널 실행 방법을 확인한다. 앞서 그린 관계도와 제공 자료를 대조해 클래스와 개별 설비를 구분한다. 제공 파일 형식에 맞춰 고유 ID·속성·관계 방향을 갖춘 작은 schema.json과 예시 인스턴스를 작성한다. 제공 절차로 별도 랩 DB에 적재한 뒤 설비의 센서·부품을 조회하고 원자료와 비교한다. 빠진 관계나 잘못된 식별자를 수정하고 관계도·모델·조회 결과를 저장한다. 다음 회차에는 이 작은 모델을 여러 설비와 공용 부품으로 확장하고 SOP를 연결한다. Notion 학습노트의 해당 주제에 관계도와 확인 결과를 연결한다.</x:v>
       </x:c>
       <x:c r="D9" s="144" t="n">
         <x:v>50</x:v>
@@ -4928,7 +4924,7 @@
         <x:v>시간(분)</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" s="1" customFormat="1" ht="92" customHeight="1">
+    <x:row r="14" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A14" s="141" t="str">
         <x:v>이론</x:v>
       </x:c>
@@ -4936,10 +4932,10 @@
         <x:v>식별자·적재·SOP 연결 원리 이해하기</x:v>
       </x:c>
       <x:c r="C14" s="141" t="str">
-        <x:v>고유 식별자로 같은 대상을 구분하는 방법과 반복 적재 시 중복을 막는 원리를 살펴본다. 필수값·자료형·관계 끝점 제약을 설비 모델에 대어 확인하고, 고장·조치와 SOP의 전제·금지·완료 조건이 연결되는 구조를 이해한다.</x:v>
+        <x:v>앞서 만든 작은 모델을 다시 적재해도 중복되지 않게 하고 작업 절차를 연결한다. 고유 식별자로 같은 대상을 구분하는 방법과 반복 적재 시 중복을 막는 원리를 살펴본다. 필수값·자료형·관계 끝점 제약을 설비 모델에 대어 확인하고, 고장·조치와 SOP의 전제·금지·완료 조건이 연결되는 구조를 이해한다.</x:v>
       </x:c>
       <x:c r="D14" s="142" t="n">
-        <x:v>50</x:v>
+        <x:v>35</x:v>
       </x:c>
     </x:row>
     <x:row r="15" s="1" customFormat="1" ht="92" customHeight="1">
@@ -4953,7 +4949,7 @@
         <x:v>설비 모델의 고유 ID·자료형·필수값·관계 끝점을 원자료와 대조해 보완한다. 모델을 적재하고 설비별 센서·부품을 조회한다. 같은 자료를 다시 적재한 뒤 노드와 관계가 불필요하게 늘어나지 않았는지 확인한다.</x:v>
       </x:c>
       <x:c r="D15" s="144" t="n">
-        <x:v>50</x:v>
+        <x:v>55</x:v>
       </x:c>
     </x:row>
     <x:row r="16" s="1" customFormat="1" ht="92" customHeight="1">
@@ -4970,7 +4966,7 @@
         <x:v>50</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" s="1" customFormat="1" ht="92" customHeight="1">
+    <x:row r="17" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A17" s="143" t="str">
         <x:v>실습</x:v>
       </x:c>
@@ -4978,10 +4974,10 @@
         <x:v>SOP를 모델에 연결하고 결과 완성하기</x:v>
       </x:c>
       <x:c r="C17" s="143" t="str">
-        <x:v>제공 SOP에서 작업의 전제·금지·수행 단계·완료 조건을 구분한다. 고장 유형과 조치 방법을 기존 설비 모델의 식별자에 연결하고, 선택한 고장에 적용할 절차와 금지 조건을 조회해 원문과 비교한다.</x:v>
+        <x:v>제공 SOP에서 작업의 전제·금지·수행 단계·완료 조건을 구분한다. 고장 유형과 조치 방법을 기존 설비 모델의 식별자에 연결하고, 선택한 고장에 적용할 절차와 금지 조건을 조회해 원문과 비교한다. 다음 회차에는 연결한 SOP 조건으로 조치의 허용·제외와 성과를 판정한다.</x:v>
       </x:c>
       <x:c r="D17" s="144" t="n">
-        <x:v>50</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="18" s="1" customFormat="1" ht="28" customHeight="1">
@@ -5023,7 +5019,7 @@
         <x:v>시간(분)</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" s="1" customFormat="1" ht="92" customHeight="1">
+    <x:row r="22" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A22" s="141" t="str">
         <x:v>이론</x:v>
       </x:c>
@@ -5031,10 +5027,10 @@
         <x:v>안전한 판단 규칙과 성과 비교 기준 이해하기</x:v>
       </x:c>
       <x:c r="C22" s="141" t="str">
-        <x:v>SOP의 작업 순서와 DMN의 판단 조건을 구분한다. 입력값·단위·연산자·경계값으로 조치 허용·제외를 표현하고, 허용된 후보끼리 비용·생산·품질·에너지 성과를 비교하는 이유를 사례로 확인한다.</x:v>
+        <x:v>관계와 절차를 읽는 데서 나아가 입력 조건에 따라 가능한 조치와 그 이유를 반환한다. SOP의 작업 순서와 DMN의 판단 조건을 구분한다. 입력값·단위·연산자·경계값으로 조치 허용·제외를 표현하고, 허용된 후보끼리 비용·생산·품질·에너지 성과를 비교하는 이유를 사례로 확인한다.</x:v>
       </x:c>
       <x:c r="D22" s="142" t="n">
-        <x:v>50</x:v>
+        <x:v>40</x:v>
       </x:c>
     </x:row>
     <x:row r="23" s="1" customFormat="1" ht="92" customHeight="1">
@@ -5048,7 +5044,7 @@
         <x:v>포털 What-if에서 운전 조건을 바꿔 조치 허용·제외와 순위 변화를 비교한다. 제공 SOP에서 입력·단위·경계·출처를 뽑아 결정표를 작성하고, 각 조건이 어떤 조치를 허용하거나 제외하는지 표시한다.</x:v>
       </x:c>
       <x:c r="D23" s="144" t="n">
-        <x:v>50</x:v>
+        <x:v>45</x:v>
       </x:c>
     </x:row>
     <x:row r="24" s="1" customFormat="1" ht="92" customHeight="1">
@@ -5062,10 +5058,10 @@
         <x:v>VS Code에서 결정표를 입력으로 사용해 조치의 허용·제외와 사유를 반환하는 기능을 만든다. 정상 조건, 경계값, 여러 규칙이 동시에 맞는 경우, 금지 조건을 입력해 실제 결과를 조건표와 대조한다.</x:v>
       </x:c>
       <x:c r="D24" s="142" t="n">
-        <x:v>50</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" s="1" customFormat="1" ht="92" customHeight="1">
+        <x:v>60</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A25" s="143" t="str">
         <x:v>실습</x:v>
       </x:c>
@@ -5073,10 +5069,10 @@
         <x:v>성과를 비교하고 경계·누락 입력 검증하기</x:v>
       </x:c>
       <x:c r="C25" s="143" t="str">
-        <x:v>허용된 조치 후보만 비용·생산 영향·품질·에너지 기준으로 비교한다. 경계값이나 필수 정보 누락에 따라 결과가 달라지는지 확인하고, 선택 이유와 추가 확인 사항을 출력한다. 추천 결과와 사람의 실행 승인을 구분한다.</x:v>
+        <x:v>허용된 조치 후보만 비용·생산 영향·품질·에너지 기준으로 비교한다. 경계값이나 필수 정보 누락에 따라 결과가 달라지는지 확인하고, 선택 이유와 추가 확인 사항을 출력한다. 추천 결과와 사람의 실행 승인을 구분한다. 다음 회차에는 사용한 조건의 원문을 추출·검토하여 근거 지식을 보강한다.</x:v>
       </x:c>
       <x:c r="D25" s="144" t="n">
-        <x:v>50</x:v>
+        <x:v>55</x:v>
       </x:c>
     </x:row>
     <x:row r="26" s="1" customFormat="1" ht="28" customHeight="1">
@@ -5118,7 +5114,7 @@
         <x:v>시간(분)</x:v>
       </x:c>
     </x:row>
-    <x:row r="30" s="1" customFormat="1" ht="92" customHeight="1">
+    <x:row r="30" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A30" s="141" t="str">
         <x:v>이론</x:v>
       </x:c>
@@ -5126,10 +5122,10 @@
         <x:v>문서 추출·검토·출처 관리 원리 이해하기</x:v>
       </x:c>
       <x:c r="C30" s="141" t="str">
-        <x:v>매뉴얼 원문, AI가 추출한 후보, 검토를 거친 지식을 구분한다. 부정 조건·단위·작업 순서가 잘못 추출된 사례를 원문과 대조하고, 문서 ID·페이지·인용 구간을 지식과 함께 보존하는 이유를 이해한다.</x:v>
+        <x:v>판단에 쓰는 조건을 원문까지 확인할 수 있도록 문서 추출·검토·적재를 연결한다. 매뉴얼 원문, AI가 추출한 후보, 검토를 거친 지식을 구분한다. 부정 조건·단위·작업 순서가 잘못 추출된 사례를 원문과 대조하고, 문서 ID·페이지·인용 구간을 지식과 함께 보존하는 이유를 이해한다.</x:v>
       </x:c>
       <x:c r="D30" s="142" t="n">
-        <x:v>50</x:v>
+        <x:v>35</x:v>
       </x:c>
     </x:row>
     <x:row r="31" s="1" customFormat="1" ht="92" customHeight="1">
@@ -5137,13 +5133,13 @@
         <x:v>실습</x:v>
       </x:c>
       <x:c r="B31" s="143" t="str">
-        <x:v>문서 등록을 경험하고 추출 기능 만들기</x:v>
+        <x:v>등록된 문서 지식을 검토하고 로컬 추출 기능 만들기</x:v>
       </x:c>
       <x:c r="C31" s="143" t="str">
         <x:v>포털의 제공 매뉴얼 원문과 등록된 추출 결과를 비교한다. VS Code에서 제공 문서의 표·작업 절차·수치·단위·금지 조건을 구조화하는 기능을 만들고 문서 ID·페이지 또는 구간·인용을 함께 출력한다.</x:v>
       </x:c>
       <x:c r="D31" s="144" t="n">
-        <x:v>50</x:v>
+        <x:v>55</x:v>
       </x:c>
     </x:row>
     <x:row r="32" s="1" customFormat="1" ht="92" customHeight="1">
@@ -5157,10 +5153,10 @@
         <x:v>추출 후보의 조건·단위·순서를 원문과 비교해 채택·수정·제외한다. 채택한 항목을 기존 랩 그래프의 클래스와 식별자에 맞춰 적재하고, 고장→원인→조치→근거 문서 관계를 조회한다.</x:v>
       </x:c>
       <x:c r="D32" s="142" t="n">
-        <x:v>50</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33" s="1" customFormat="1" ht="92" customHeight="1">
+        <x:v>65</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A33" s="143" t="str">
         <x:v>실습</x:v>
       </x:c>
@@ -5168,10 +5164,10 @@
         <x:v>다른 문서에 적용하고 결과 검증하기</x:v>
       </x:c>
       <x:c r="C33" s="143" t="str">
-        <x:v>제공된 다른 매뉴얼에 같은 추출 기능을 적용한다. 빠진 조건이나 잘못 연결된 대상이 있는지 원문과 대조하고 수정한다. 그래프에 반영한 지식에서 문서 출처를 다시 찾아 검토 결과와 일치하는지 확인한다.</x:v>
+        <x:v>제공된 다른 매뉴얼에 같은 추출 기능을 적용한다. 빠진 조건이나 잘못 연결된 대상이 있는지 원문과 대조하고 수정한다. 그래프에 반영한 지식에서 문서 출처를 다시 찾아 검토 결과와 일치하는지 확인한다. 이 검토 지식과 센서 자료를 다음 회차 에이전트의 근거로 사용한다.</x:v>
       </x:c>
       <x:c r="D33" s="144" t="n">
-        <x:v>50</x:v>
+        <x:v>45</x:v>
       </x:c>
     </x:row>
     <x:row r="34" s="1" customFormat="1" ht="28" customHeight="1">
@@ -5213,7 +5209,7 @@
         <x:v>시간(분)</x:v>
       </x:c>
     </x:row>
-    <x:row r="38" s="1" customFormat="1" ht="92" customHeight="1">
+    <x:row r="38" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A38" s="141" t="str">
         <x:v>이론</x:v>
       </x:c>
@@ -5221,10 +5217,10 @@
         <x:v>에이전트의 근거·도구·종료 조건 이해하기</x:v>
       </x:c>
       <x:c r="C38" s="141" t="str">
-        <x:v>LLM의 답변, RAG의 근거 검색, 에이전트의 목표·도구·반복 실행을 구분한다. 설비 지식과 현재 센서 값을 각각 어디서 얻는지 살펴보고, 근거 부족이나 도구 오류가 생겼을 때 멈추거나 확인을 요청할 조건을 정한다.</x:v>
+        <x:v>검토한 지식과 현재 입력을 이용해 원인 후보·후속 업무·이상 구간을 확인한다. LLM의 답변, RAG의 근거 검색, 에이전트의 목표·도구·반복 실행을 구분한다. 설비 지식과 현재 센서 값을 각각 어디서 얻는지 살펴보고, 근거 부족이나 도구 오류가 생겼을 때 멈추거나 확인을 요청할 조건을 정한다.</x:v>
       </x:c>
       <x:c r="D38" s="142" t="n">
-        <x:v>50</x:v>
+        <x:v>35</x:v>
       </x:c>
     </x:row>
     <x:row r="39" s="1" customFormat="1" ht="92" customHeight="1">
@@ -5238,7 +5234,7 @@
         <x:v>포털 에이전트의 목표·도구·근거를 확인한다. VS Code에서 설비·센서·고장·SOP 관계와 센서 입력을 읽어 원인 후보·증거·다음 점검 순서를 제안하는 에이전트를 만든다. 확인되지 않은 원인이 가설로 표시되는지 검토한다.</x:v>
       </x:c>
       <x:c r="D39" s="144" t="n">
-        <x:v>50</x:v>
+        <x:v>65</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="92" customHeight="1">
@@ -5252,10 +5248,10 @@
         <x:v>제공 불량 접수 메시지와 분류 기준으로 품질 유형·추가 확인 항목·담당 부서·대응 초안을 출력하는 에이전트를 만든다. 원인이 확정되지 않은 사례를 입력해 단정 대신 조사 요청을 남기는지 확인한다.</x:v>
       </x:c>
       <x:c r="D40" s="142" t="n">
-        <x:v>50</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="41" s="1" customFormat="1" ht="92" customHeight="1">
+        <x:v>55</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A41" s="143" t="str">
         <x:v>실습</x:v>
       </x:c>
@@ -5263,10 +5259,10 @@
         <x:v>센서 시각화와 에이전트 결과 검증하기</x:v>
       </x:c>
       <x:c r="C41" s="143" t="str">
-        <x:v>센서 CSV의 시간·온도·압력 변화를 읽어 이상 구간을 시각화한다. 관련 태그와 조회 기간을 함께 표시하고 원자료와 비교한다. 원인 점검·품질 대응·시각화 결과에서 근거와 미확인 사항이 구분되는지 검토한다.</x:v>
+        <x:v>센서 CSV의 시간·온도·압력 변화를 읽어 이상 구간을 시각화한다. 관련 태그와 조회 기간을 함께 표시하고 원자료와 비교한다. 원인 점검·품질 대응·시각화 결과에서 근거와 미확인 사항이 구분되는지 검토한다. 다음 회차에는 반복 작업의 지침을 스킬로 만들고 파일·Git·시간 도구를 조합한다.</x:v>
       </x:c>
       <x:c r="D41" s="144" t="n">
-        <x:v>50</x:v>
+        <x:v>45</x:v>
       </x:c>
     </x:row>
     <x:row r="42" s="1" customFormat="1" ht="28" customHeight="1">
@@ -5308,7 +5304,7 @@
         <x:v>시간(분)</x:v>
       </x:c>
     </x:row>
-    <x:row r="46" s="1" customFormat="1" ht="92" customHeight="1">
+    <x:row r="46" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A46" s="141" t="str">
         <x:v>이론</x:v>
       </x:c>
@@ -5316,10 +5312,10 @@
         <x:v>스킬·MCP·접근 범위 이해하기</x:v>
       </x:c>
       <x:c r="C46" s="141" t="str">
-        <x:v>SKILL.md에 담는 목적·입력·출력·절차와 MCP 도구의 역할을 구분한다. 파일·Git·시간 도구의 입력과 반환값을 살펴보고, 읽기·쓰기 권한과 접근 가능한 경로가 작업에 미치는 영향을 확인한다.</x:v>
+        <x:v>에이전트의 반복 작업을 재사용 지침과 도구 호출로 나누어 구성한다. SKILL.md에 담는 목적·입력·출력·절차와 MCP 도구의 역할을 구분한다. 파일·Git·시간 도구의 입력과 반환값을 살펴보고, 읽기·쓰기 권한과 접근 가능한 경로가 작업에 미치는 영향을 확인한다.</x:v>
       </x:c>
       <x:c r="D46" s="142" t="n">
-        <x:v>50</x:v>
+        <x:v>30</x:v>
       </x:c>
     </x:row>
     <x:row r="47" s="1" customFormat="1" ht="92" customHeight="1">
@@ -5333,7 +5329,7 @@
         <x:v>준비된 MCP의 연결과 호출 결과를 확인한다. 회의록에서 결정사항·담당자·기한·출처를 추출하는 SKILL.md를 작성하고, 담당자나 기한이 없는 항목은 미정으로 남기는지 원문과 비교한다.</x:v>
       </x:c>
       <x:c r="D47" s="144" t="n">
-        <x:v>50</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="48" s="1" customFormat="1" ht="92" customHeight="1">
@@ -5347,10 +5343,10 @@
         <x:v>파일 내용 읽기→Git 변경 기록 확인→시간 정보 확인을 하나의 요청으로 연결한다. 각 도구의 반환값이 결과에 어떻게 사용됐는지 확인하고, 업무 목록의 변경 내용과 시점을 원자료에 대어 검증한다.</x:v>
       </x:c>
       <x:c r="D48" s="142" t="n">
-        <x:v>50</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="49" ht="92" customHeight="1">
+        <x:v>55</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="108" customHeight="1">
       <x:c r="A49" s="143" t="str">
         <x:v>실습</x:v>
       </x:c>
@@ -5358,10 +5354,10 @@
         <x:v>대화형 학습 코치를 만들고 검증하기</x:v>
       </x:c>
       <x:c r="C49" s="143" t="str">
-        <x:v>제공 학습 자료를 바탕으로 문항 생성→답변 입력→정답·원문 근거 피드백으로 이어지는 대화형 학습 코치를 만든다. 답변을 달리 입력해 피드백이 바뀌는지 확인하고, 피드백의 출처가 학습 자료에 있는지 대조한다.</x:v>
+        <x:v>제공 학습 자료를 바탕으로 문항 생성→답변 입력→정답·원문 근거 피드백으로 이어지는 대화형 학습 코치를 만든다. 답변을 달리 입력해 피드백이 바뀌는지 확인하고, 피드백의 출처가 학습 자료에 있는지 대조한다. 다음 회차에는 정보 누락과 요구 변경에도 결과를 확인할 수 있도록 질문·명세·검증을 연결한다.</x:v>
       </x:c>
       <x:c r="D49" s="144" t="n">
-        <x:v>50</x:v>
+        <x:v>55</x:v>
       </x:c>
     </x:row>
     <x:row r="50" s="1" customFormat="1" ht="28" customHeight="1">
@@ -5403,7 +5399,7 @@
         <x:v>시간(분)</x:v>
       </x:c>
     </x:row>
-    <x:row r="54" s="1" customFormat="1" ht="92" customHeight="1">
+    <x:row r="54" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A54" s="141" t="str">
         <x:v>이론</x:v>
       </x:c>
@@ -5411,21 +5407,21 @@
         <x:v>질문·승인·명세·행동 검증 이해하기</x:v>
       </x:c>
       <x:c r="C54" s="141" t="str">
-        <x:v>정보 확인 질문과 사람의 승인을 구분한다. 입력·출력·금지 조건·수용 기준을 명세로 표현하고, Given/When/Then으로 기대 행동을 정하는 방법을 익힌다. 새 기능의 동작과 기존 기능 보존을 함께 확인하는 이유를 이해한다.</x:v>
+        <x:v>앞서 만든 업무 요청 기능의 누락 입력과 변경 요구를 다루고 기존 동작이 유지되는지 확인한다. 정보 확인 질문과 사람의 승인을 구분한다. 입력·출력·금지 조건·수용 기준을 명세로 표현하고, Given/When/Then으로 기대 행동을 정하는 방법을 익힌다. 새 기능의 동작과 기존 기능 보존을 함께 확인하는 이유를 이해한다.</x:v>
       </x:c>
       <x:c r="D54" s="142" t="n">
-        <x:v>50</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="55" s="1" customFormat="1" ht="92" customHeight="1">
+        <x:v>40</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A55" s="143" t="str">
         <x:v>실습</x:v>
       </x:c>
       <x:c r="B55" s="143" t="str">
-        <x:v>질문과 재개·작성과 검토 흐름 구현하기</x:v>
+        <x:v>질문·답변·재개를 구현하고 작성·검토 결과 비교하기</x:v>
       </x:c>
       <x:c r="C55" s="143" t="str">
-        <x:v>포털의 승인 대기·승인·반려 상태를 비교한다. 품질 후속 업무 요청에 필수 정보가 빠졌을 때 질문하고 답변을 받은 뒤 다시 판단하는 흐름을 만든다. 작성·검토 에이전트의 결과와 사람의 최종 승인을 구분한다.</x:v>
+        <x:v>포털의 승인 대기·승인·반려 상태를 확인한다. 제공된 품질 후속 업무 시작본에서 필수 정보가 빠지면 질문하고 답변 뒤 다시 판단하도록 구현한다. 제공 작성·검토 결과를 대조해 AI 검토와 사람의 최종 승인을 구분한다.</x:v>
       </x:c>
       <x:c r="D55" s="144" t="n">
         <x:v>50</x:v>
@@ -5442,10 +5438,10 @@
         <x:v>같은 업무 요청 프로젝트에서 변경할 기능을 정하고 입력·출력·금지 조건·완료 기준을 spec.md로 작성한다. AI 코딩 도구로 변경을 구현한 뒤 기존 일반 요청과 변경 요청의 출력을 비교한다.</x:v>
       </x:c>
       <x:c r="D56" s="142" t="n">
-        <x:v>50</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="57" s="1" customFormat="1" ht="92" customHeight="1">
+        <x:v>55</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A57" s="143" t="str">
         <x:v>실습</x:v>
       </x:c>
@@ -5453,10 +5449,10 @@
         <x:v>행동을 검증하고 인수인계 결과 만들기</x:v>
       </x:c>
       <x:c r="C57" s="143" t="str">
-        <x:v>정상·정보 누락·변경 요구의 기대 결과를 Given/When/Then으로 작성해 실제 출력과 비교한다. 제공 센서·정비·부품 자료를 연결해 완료·미완료·다음 조치·근거 시각을 담은 인수인계 결과를 만들고 원자료와 대조한다.</x:v>
+        <x:v>정상·정보 누락·변경 요구의 기대 결과를 Given/When/Then으로 작성해 실제 출력과 비교한다. 제공 센서·정비·부품 자료를 연결해 완료·미완료·다음 조치·근거 시각을 담은 인수인계 결과를 만들고 원자료와 대조한다. 다음 회차에는 검증한 작업을 사람의 승인과 함께 BPMN으로 표현한다.</x:v>
       </x:c>
       <x:c r="D57" s="144" t="n">
-        <x:v>50</x:v>
+        <x:v>55</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="28" customHeight="1">
@@ -5498,7 +5494,7 @@
         <x:v>시간(분)</x:v>
       </x:c>
     </x:row>
-    <x:row r="62" s="1" customFormat="1" ht="92" customHeight="1">
+    <x:row r="62" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A62" s="141" t="str">
         <x:v>이론</x:v>
       </x:c>
@@ -5506,10 +5502,10 @@
         <x:v>BPMN 역할·분기·지연·실행 연결 이해하기</x:v>
       </x:c>
       <x:c r="C62" s="141" t="str">
-        <x:v>시작·종료 이벤트, 작업, 역할별 Lane, 승인 분기와 지연 알림의 의미를 설비 대응 사례로 구분한다. BPMN 그림의 각 작업이 에이전트·사람·시스템 중 누구에게 연결되는지 살펴보고, 승인 거절과 승인 대기 상태의 차이를 확인한다.</x:v>
+        <x:v>개별 작업의 결과가 다음 작업으로 넘어가는 조건과 담당 역할을 그림으로 명확히 한다. 시작·종료 이벤트, 작업, 역할별 Lane, 승인 분기와 지연 알림의 의미를 설비 대응 사례로 구분한다. BPMN 그림의 각 작업이 에이전트·사람·시스템 중 누구에게 연결되는지 살펴보고, 승인 거절과 승인 대기 상태의 차이를 확인한다.</x:v>
       </x:c>
       <x:c r="D62" s="142" t="n">
-        <x:v>50</x:v>
+        <x:v>35</x:v>
       </x:c>
     </x:row>
     <x:row r="63" s="1" customFormat="1" ht="92" customHeight="1">
@@ -5523,7 +5519,7 @@
         <x:v>bpmn.io에서 시작→요청 확인→승인 또는 반려→종료를 그린다. 이어 쿨러 경보→원인 분석·조치 제안→운전원 승인→설비 명령→효과 확인→보고로 흐름을 확장하고, 담당 역할에 맞게 작업을 Lane에 배치한다.</x:v>
       </x:c>
       <x:c r="D63" s="144" t="n">
-        <x:v>50</x:v>
+        <x:v>65</x:v>
       </x:c>
     </x:row>
     <x:row r="64" s="1" customFormat="1" ht="92" customHeight="1">
@@ -5537,10 +5533,10 @@
         <x:v>승인·거절 분기와 각각의 종료 경로를 연결한다. 거절 경로에서 설비 명령으로 진행되지 않는지 확인하고, 승인 작업을 취소하지 않는 지연 알림 Timer를 추가한다. 각 경로를 따라가며 분기 조건과 연결 누락을 점검한다.</x:v>
       </x:c>
       <x:c r="D64" s="142" t="n">
-        <x:v>50</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="65" s="1" customFormat="1" ht="92" customHeight="1">
+        <x:v>55</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A65" s="143" t="str">
         <x:v>실습</x:v>
       </x:c>
@@ -5548,10 +5544,10 @@
         <x:v>BPMN과 등록된 실행 연결 비교하기</x:v>
       </x:c>
       <x:c r="C65" s="143" t="str">
-        <x:v>bpmn.io에서 작성한 설비 대응 흐름과 포털에 등록된 기준 흐름을 비교한다. 제공 매핑 자료에서 시작 이벤트·에이전트·운전원 승인·설비 명령·재관측 작업의 연결을 찾는다. 자신이 그린 각 작업이 어떤 실행 기능에 대응하는지 표시하고, 그림 파일과 실행 정의를 구분한다.</x:v>
+        <x:v>bpmn.io에서 작성한 설비 대응 흐름과 포털에 등록된 기준 흐름을 비교한다. 제공 매핑 자료에서 시작 이벤트·에이전트·운전원 승인·설비 명령·재관측 작업의 연결을 찾는다. 자신이 그린 각 작업이 어떤 실행 기능에 대응하는지 표시하고, 그림 파일과 실행 정의를 구분한다. 다음 회차에는 등록된 흐름을 실행해 이 그림과 실제 처리 이력을 대조한다.</x:v>
       </x:c>
       <x:c r="D65" s="144" t="n">
-        <x:v>50</x:v>
+        <x:v>45</x:v>
       </x:c>
     </x:row>
     <x:row r="66" s="1" customFormat="1" ht="28" customHeight="1">
@@ -5593,7 +5589,7 @@
         <x:v>시간(분)</x:v>
       </x:c>
     </x:row>
-    <x:row r="70" s="1" customFormat="1" ht="92" customHeight="1">
+    <x:row r="70" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A70" s="141" t="str">
         <x:v>실습</x:v>
       </x:c>
@@ -5601,10 +5597,10 @@
         <x:v>실행 상태를 이해하고 정상·예외 경로 확인하기</x:v>
       </x:c>
       <x:c r="C70" s="141" t="str">
-        <x:v>포털에 이미 등록된 설비 대응 흐름을 쿨러 열화 시나리오로 실행한다. 에이전트 판단→운전원 승인→설비 명령→재관측→완료 기록을 따라간다. 승인 대기와 반려 결과를 비교하고, 자신이 그린 BPMN의 작업·분기와 실행 이력을 대조한다.</x:v>
+        <x:v>앞서 그린 BPMN과 실제 실행을 비교하고 같은 구조를 교대 검토·확인 흐름에 연결한다. 포털에 이미 등록된 설비 대응 흐름을 쿨러 열화 시나리오로 실행한다. 에이전트 판단→운전원 승인→설비 명령→재관측→완료 기록을 따라간다. 승인 대기와 반려 결과를 비교하고, 자신이 그린 BPMN의 작업·분기와 실행 이력을 대조한다.</x:v>
       </x:c>
       <x:c r="D70" s="142" t="n">
-        <x:v>50</x:v>
+        <x:v>45</x:v>
       </x:c>
     </x:row>
     <x:row r="71" s="1" customFormat="1" ht="92" customHeight="1">
@@ -5618,7 +5614,7 @@
         <x:v>자신의 BPMN 그림과 실행 이력의 작업·역할·분기 차이를 찾아 그림을 수정한다. 교대 인수인계에 필요한 설비·교대·기준 시각·작업 메모를 정하고, 인계자 검토와 인수자 확인을 완료 조건으로 작성한다.</x:v>
       </x:c>
       <x:c r="D71" s="144" t="n">
-        <x:v>50</x:v>
+        <x:v>35</x:v>
       </x:c>
     </x:row>
     <x:row r="72" s="1" customFormat="1" ht="98" customHeight="1">
@@ -5632,10 +5628,10 @@
         <x:v>강사 코드로 열린 교대 실습에서 제공 보충 매뉴얼을 선택한다. 준비된 추출 결과의 절차·조건·근거를 원문과 비교하고 검토한 항목을 기존 제조 지식에 추가한다. 추가된 지식의 식별자와 원문 연결을 확인한다. 교대 실습에서 허용된 설비·정비·ERP 조회 도구로 인계안을 작성하는 에이전트·스킬을 구성한다. 이름·설명·스킬에 확인할 항목을 적고, 완료 메모와 열린 작업지시 또는 입고 예정과 실제 재고가 다를 때 확인 사항으로 남기는지 결과와 원천을 대조한다.</x:v>
       </x:c>
       <x:c r="D72" s="142" t="n">
-        <x:v>50</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="73" s="1" customFormat="1" ht="92" customHeight="1">
+        <x:v>70</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A73" s="143" t="str">
         <x:v>실습</x:v>
       </x:c>
@@ -5643,7 +5639,7 @@
         <x:v>제공 인수인계 BPMN의 에이전트 배정·등록하기</x:v>
       </x:c>
       <x:c r="C73" s="143" t="str">
-        <x:v>제공 교대 BPMN을 bpmn.io에서 열어 작업 이름과 배치를 정리한다. 시작 입력·검토·보완 분기를 유지하고 세 초안 단계에 교대 에이전트를 배정하여 별도 판본을 등록한다. 설비·교대 정보를 입력해 인계안 작성→인계자 검토→인수자 보완 요청→재검토→인수 확인을 수행하고 근거와 완료 기록을 확인한다.</x:v>
+        <x:v>제공 교대 BPMN을 bpmn.io에서 열어 이름과 배치를 정리한다. 시작 입력·검토·보완 분기를 유지하고 세 초안 단계에 교대 에이전트를 배정하여 별도 판본을 등록한다. 시작 폼의 설비·교대 입력과 각 단계 배정을 확인한다. 다음 회차에는 정비·구매의 실행 결과를 확인하고 준비한 교대 흐름을 끝까지 수행한다.</x:v>
       </x:c>
       <x:c r="D73" s="144" t="n">
         <x:v>50</x:v>
@@ -5688,7 +5684,7 @@
         <x:v>시간(분)</x:v>
       </x:c>
     </x:row>
-    <x:row r="78" s="1" customFormat="1" ht="92" customHeight="1">
+    <x:row r="78" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A78" s="141" t="str">
         <x:v>실습</x:v>
       </x:c>
@@ -5696,10 +5692,10 @@
         <x:v>업무별 시작 조건을 비교하고 정비 흐름 설계하기</x:v>
       </x:c>
       <x:c r="C78" s="141" t="str">
-        <x:v>냉각 경보·정기 점검 도래·재고 부족의 시작 조건과 완료 결과를 비교한다. 정기 점검→정비 계획→설비보전팀장 승인 또는 거절→정비 오더→생산팀 공지 흐름을 bpmn.io에서 작성하고 담당 역할과 분기 조건을 연결한다.</x:v>
+        <x:v>설비 대응에서 익힌 패턴을 정비·구매에 적용하고 교대 인수인계의 검토·확인까지 마친다. 냉각 경보·정기 점검 도래·재고 부족의 시작 조건과 완료 결과를 비교한다. 정기 점검→정비 계획→설비보전팀장 승인 또는 거절→정비 오더→생산팀 공지 흐름을 bpmn.io에서 작성하고 담당 역할과 분기 조건을 연결한다.</x:v>
       </x:c>
       <x:c r="D78" s="142" t="n">
-        <x:v>50</x:v>
+        <x:v>35</x:v>
       </x:c>
     </x:row>
     <x:row r="79" s="1" customFormat="1" ht="92" customHeight="1">
@@ -5713,7 +5709,7 @@
         <x:v>포털의 정기 점검 시나리오로 등록된 정비 흐름을 실행한다. 정비 계획·승인·작업지시·예약 또는 출고·생산 공지의 처리 기록을 확인한다. 승인과 반려 사례를 비교하여 정비 오더가 만들어지는 조건을 자신의 BPMN과 대조한다.</x:v>
       </x:c>
       <x:c r="D79" s="144" t="n">
-        <x:v>50</x:v>
+        <x:v>35</x:v>
       </x:c>
     </x:row>
     <x:row r="80" s="1" customFormat="1" ht="92" customHeight="1">
@@ -5727,10 +5723,10 @@
         <x:v>bpmn.io에서 재고 부족→구매 제안→승인 또는 반려→발주→통지→입고 반영 흐름을 그린다. 포털의 재고 보충 시나리오로 등록된 구매 흐름을 실행한다. 수업용 업무 시스템에서 발주·공급사 통지·입고·재고 반영 기록을 확인하고, 반려 사례의 처리 결과와 비교한다. 자신의 BPMN에서 각 결과에 대응하는 작업을 찾는다.</x:v>
       </x:c>
       <x:c r="D80" s="142" t="n">
-        <x:v>50</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="81" s="1" customFormat="1" ht="92" customHeight="1">
+        <x:v>60</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81" s="1" customFormat="1" ht="145" customHeight="1">
       <x:c r="A81" s="143" t="str">
         <x:v>실습</x:v>
       </x:c>
@@ -5738,10 +5734,10 @@
         <x:v>교대 인수인계를 완성하고 ProcessGPT 연결 보기</x:v>
       </x:c>
       <x:c r="C81" s="143" t="str">
-        <x:v>교대 인수인계 흐름에 설비·교대 정보를 입력하고 정상·기록 불일치·정보 누락 사례를 실행한다. 인계자 검토, 인수자의 보완 요청과 확인을 거쳐 인계 내용·근거·완료 기록을 대조한다(30분). ProcessGPT 시연을 보며 자신이 만든 지식·에이전트·업무 흐름이 제품의 작업함과 실행 기록에 어떻게 연결되는지 비교한다(20분).</x:v>
+        <x:v>교대 흐름에 설비·교대 정보를 입력하고 인계안의 근거와 원천 기록을 대조한다. 인계자 검토→인수자 보완 요청→재검토→인수 확인을 거쳐 완료 기록을 확인한다. 실제 결과에서 빠진 정보나 불일치가 있으면 확인 사항으로 남긴다(50분). 이어 ProcessGPT 시연에서 지식·에이전트·사람 작업·실행 기록이 어떻게 연결되는지 자신이 수행한 흐름과 비교한다(20분). 관계 모델·판단 근거·실행 기록을 연결하여 전체 과정을 설명한다.</x:v>
       </x:c>
       <x:c r="D81" s="144" t="n">
-        <x:v>50</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="82" s="1" customFormat="1" ht="28" customHeight="1">
@@ -6384,15 +6380,15 @@
   <x:sheetData>
     <x:row r="1" s="1" customFormat="1" ht="38" customHeight="1">
       <x:c r="A1" s="137" t="str">
-        <x:v>HYD 제조 AI | 실전반 오프라인 정규 9회 | 50분 수업 단위</x:v>
+        <x:v>HYD 제조 AI | 실전반 오프라인 정규 9회 | 수업 계획</x:v>
       </x:c>
       <x:c r="B1" s="137"/>
       <x:c r="C1" s="137"/>
       <x:c r="D1" s="137"/>
     </x:row>
-    <x:row r="2" s="1" customFormat="1" ht="38" customHeight="1">
+    <x:row r="2" s="1" customFormat="1" ht="48" customHeight="1">
       <x:c r="A2" s="135" t="str">
-        <x:v>온라인 실습에서 주요 활동을 선별해 직접 수행합니다. 기본 편성은 수업200분·휴식40분이며, 강사가 학생 진행에 따라 시간을 조절합니다. 이론이 있는 회차는50분, 마지막 두 회차는 실습 중심입니다.</x:v>
+        <x:v>온라인 선행학습 후 목적·핵심 개념을 연결하고 주요 실습을 직접 수행합니다. 수업200분·휴식40분의 기본 배정이며 실제 진행은 강사가 조절합니다. 이전 개인 결과 없이 제공 시작본으로 시작할 수 있습니다.</x:v>
       </x:c>
       <x:c r="B2" s="135"/>
       <x:c r="C2" s="135"/>
@@ -6406,7 +6402,7 @@
     </x:row>
     <x:row r="4" s="1" customFormat="1" ht="38" customHeight="1">
       <x:c r="A4" s="138" t="str">
-        <x:v>01회차 | 설비 정보를 관계와 모델로 표현하기</x:v>
+        <x:v>01회차 | HYD 전체 흐름을 확인하고 설비 관계 표현하기</x:v>
       </x:c>
       <x:c r="B4" s="138"/>
       <x:c r="C4" s="138"/>
@@ -6426,32 +6422,32 @@
         <x:v>시간(분)</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" s="1" customFormat="1" ht="92" customHeight="1">
+    <x:row r="6" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A6" s="141" t="str">
         <x:v>이론</x:v>
       </x:c>
       <x:c r="B6" s="141" t="str">
-        <x:v>설비 정보와 관계 모델 이해하기</x:v>
+        <x:v>HYD 시스템과 이번 과정의 학습 목표 이해하기</x:v>
       </x:c>
       <x:c r="C6" s="141" t="str">
-        <x:v>설비·센서·부품이 각각 어떤 정보를 나타내는지 구분한다. 쿨러의 온도 변화가 센서 값, 이상 징후, 원인 후보, 조치 판단으로 이어지는 경로를 살펴본다. 같은 종류와 개별 대상을 클래스·인스턴스로 나누고, 식별자·속성·관계 방향을 설비 사례에 적용한다.</x:v>
+        <x:v>HYD의 완성 흐름을 먼저 확인하고, 판단 근거를 표현하는 관계도와 그래프를 직접 다룬다. HYD가 유압 설비와 업무 시스템을 연결한 수업용 시스템임을 이해한다. 설비·센서 데이터 수집→상태 관찰→지식에 근거한 판단→사람 승인→조치→결과 확인의 전체 구조를 살펴본다. 포털에서 확인할 설비 화면·지식 지도·에이전트·작업함의 역할을 구분한다. 이번 과정에서 관계 모델을 만들고, 근거를 조회하는 에이전트와 업무 흐름으로 연결할 학습 목표를 확인한다.</x:v>
       </x:c>
       <x:c r="D6" s="142" t="n">
-        <x:v>50</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" s="1" customFormat="1" ht="92" customHeight="1">
+        <x:v>40</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" s="1" customFormat="1" ht="125" customHeight="1">
       <x:c r="A7" s="143" t="str">
         <x:v>실습</x:v>
       </x:c>
       <x:c r="B7" s="143" t="str">
-        <x:v>관계도를 그리고 최소 모델 만들기</x:v>
+        <x:v>포털 시연으로 완성 흐름을 확인하고 관계도 그리기</x:v>
       </x:c>
       <x:c r="C7" s="143" t="str">
-        <x:v>arrows.app에서 쿨러·센서·부품·고장·조치를 노드로 만들고 관계를 연결한다. 각 화살표를 문장으로 읽어 방향을 확인한다. 제공 목록과 관계도를 대조해 클래스·고유 ID·속성을 갖춘 schema.json과 예시 인스턴스를 작성한다.</x:v>
+        <x:v>강사가 실제 HYD 포털을 열어 보여 주는 설비 상태·센서 값과 쿨러 열화 시나리오를 따라간다. 경보 발생→에이전트의 원인·조치 추천→운전원 승인→설비 명령→센서 값 재확인과 완료 기록을 보고, 추천·승인·실행의 차이를 구분한다. 지식 지도에서 판단에 사용된 설비·센서·고장·조치 연결을 확인한다. 이어 arrows.app에서 방금 본 대상을 노드와 관계로 그려 각 화살표를 문장으로 읽는다.</x:v>
       </x:c>
       <x:c r="D7" s="144" t="n">
-        <x:v>50</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="8" s="1" customFormat="1" ht="92" customHeight="1">
@@ -6468,15 +6464,15 @@
         <x:v>50</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" s="1" customFormat="1" ht="92" customHeight="1">
+    <x:row r="9" s="1" customFormat="1" ht="118" customHeight="1">
       <x:c r="A9" s="143" t="str">
         <x:v>실습</x:v>
       </x:c>
       <x:c r="B9" s="143" t="str">
-        <x:v>설비 모델을 적재하고 질문별 결과 확인하기</x:v>
+        <x:v>관계도를 설비 모델로 옮기고 적재·조회 결과 확인하기</x:v>
       </x:c>
       <x:c r="C9" s="143" t="str">
-        <x:v>작성한 설비 모델을 제공 절차로 별도 랩 DB에 적재한다. 설비의 센서·부품을 조회해 원자료와 비교하고 빠진 관계·식별자를 수정한다. 포털 기준 지도를 열어 자신의 모델과 연결 방향을 비교한다. 관계도·모델·조회 결과를 저장한다.</x:v>
+        <x:v>앞서 그린 관계도와 제공 자료를 대조해 클래스와 개별 설비를 구분한다. 제공 파일 형식에 맞춰 고유 ID·속성·관계 방향을 갖춘 작은 schema.json과 예시 인스턴스를 작성한다. 제공 절차로 별도 랩 DB에 적재한 뒤 설비의 센서·부품을 조회하고 원자료와 비교한다. 빠진 관계나 잘못된 식별자를 수정하고 관계도·모델·조회 결과를 저장한다. 다음 회차에는 부품의 사용 설비·공급 정보를 찾고 SOP 조건을 조치 판단에 적용한다. Notion 학습노트의 해당 주제에 관계도와 확인 결과를 연결한다.</x:v>
       </x:c>
       <x:c r="D9" s="144" t="n">
         <x:v>50</x:v>
@@ -6521,7 +6517,7 @@
         <x:v>시간(분)</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" s="1" customFormat="1" ht="92" customHeight="1">
+    <x:row r="14" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A14" s="141" t="str">
         <x:v>이론</x:v>
       </x:c>
@@ -6529,10 +6525,10 @@
         <x:v>설비 모델·조건표·판정과 승인 이해하기</x:v>
       </x:c>
       <x:c r="C14" s="141" t="str">
-        <x:v>설비·부품·공급 정보를 연결해 답할 질문을 정한다. SOP의 작업 조건을 결정표로 표현하는 방법을 살펴보고, 조치 후보의 허용·제외 판정과 사람의 실행 승인이 서로 다른 단계임을 이해한다.</x:v>
+        <x:v>설비·부품 연결 조회와 작업 조건표를 조합해 선택 근거가 보이는 조치 검토 결과를 만든다. 설비·부품·공급 정보를 연결해 답할 질문을 정한다. SOP의 작업 조건을 결정표로 표현하는 방법을 살펴보고, 조치 후보의 허용·제외 판정과 사람의 실행 승인이 서로 다른 단계임을 이해한다.</x:v>
       </x:c>
       <x:c r="D14" s="142" t="n">
-        <x:v>50</x:v>
+        <x:v>30</x:v>
       </x:c>
     </x:row>
     <x:row r="15" s="1" customFormat="1" ht="92" customHeight="1">
@@ -6560,10 +6556,10 @@
         <x:v>제공 SOP에서 입력·단위·연산자·경계·출처를 뽑아 조치 조건표를 만든다. 조건에 따라 허용·제외와 사유를 반환하는 기능을 구현하고, 허용 후보의 비용·생산·품질·에너지 성과를 비교한다.</x:v>
       </x:c>
       <x:c r="D16" s="142" t="n">
-        <x:v>50</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" s="1" customFormat="1" ht="92" customHeight="1">
+        <x:v>70</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A17" s="143" t="str">
         <x:v>실습</x:v>
       </x:c>
@@ -6571,7 +6567,7 @@
         <x:v>선택 근거와 확인 사항을 검증해 결과 완성하기</x:v>
       </x:c>
       <x:c r="C17" s="143" t="str">
-        <x:v>정상·경계·금지·누락 입력을 바꾸며 조치 검토 결과를 확인한다. 선택 이유·원문 근거·추가 확인 사항을 하나의 결과로 구성하고, 정보가 빠져도 이미 확인된 제외 근거가 유지되는지 검증한다.</x:v>
+        <x:v>정상·경계·금지·누락 입력을 바꾸며 조치 검토 결과를 확인한다. 선택 이유·원문 근거·추가 확인 사항을 하나의 결과로 구성하고, 정보가 빠져도 이미 확인된 제외 근거가 유지되는지 검증한다. 다음 회차에는 조건의 문서 출처를 연결하여 작업 확인 카드로 활용한다.</x:v>
       </x:c>
       <x:c r="D17" s="144" t="n">
         <x:v>50</x:v>
@@ -6616,7 +6612,7 @@
         <x:v>시간(분)</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" s="1" customFormat="1" ht="92" customHeight="1">
+    <x:row r="22" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A22" s="141" t="str">
         <x:v>이론</x:v>
       </x:c>
@@ -6624,10 +6620,10 @@
         <x:v>문서 추출·검토·출처 재사용 이해하기</x:v>
       </x:c>
       <x:c r="C22" s="141" t="str">
-        <x:v>매뉴얼의 작업 조건을 추출 후보·검토 지식·작업 확인 자료로 전환하는 과정을 살펴본다. 문서 ID·페이지·인용 구간과 개정 정보를 보존하는 이유를 이해하고, 원문에 없는 내용을 판별한다.</x:v>
+        <x:v>매뉴얼의 조건을 추출·검토하고 특정 작업에서 바로 확인할 수 있는 카드로 바꾼다. 매뉴얼의 작업 조건을 추출 후보·검토 지식·작업 확인 자료로 전환하는 과정을 살펴본다. 문서 ID·페이지·인용 구간과 개정 정보를 보존하는 이유를 이해하고, 원문에 없는 내용을 판별한다.</x:v>
       </x:c>
       <x:c r="D22" s="142" t="n">
-        <x:v>50</x:v>
+        <x:v>30</x:v>
       </x:c>
     </x:row>
     <x:row r="23" s="1" customFormat="1" ht="92" customHeight="1">
@@ -6641,7 +6637,7 @@
         <x:v>포털의 제공 매뉴얼 원문과 등록된 추출 결과를 비교한다. VS Code에서 제공 작업의 조건·순서·단위·금지 조건과 출처를 추출하고, 잘못 해석한 항목을 원문과 대조해 수정한다.</x:v>
       </x:c>
       <x:c r="D23" s="144" t="n">
-        <x:v>50</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="24" s="1" customFormat="1" ht="92" customHeight="1">
@@ -6658,7 +6654,7 @@
         <x:v>50</x:v>
       </x:c>
     </x:row>
-    <x:row r="25" s="1" customFormat="1" ht="92" customHeight="1">
+    <x:row r="25" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A25" s="143" t="str">
         <x:v>실습</x:v>
       </x:c>
@@ -6666,10 +6662,10 @@
         <x:v>작업 확인 카드를 만들고 검증하기</x:v>
       </x:c>
       <x:c r="C25" s="143" t="str">
-        <x:v>선택한 작업의 준비·금지·완료 조건을 담은 확인 카드를 생성하는 기능을 만든다. 카드의 각 조건을 원문과 대조해 문서 밖 절차를 제거하고, 다른 제공 작업에도 적용해 결과를 검증한다.</x:v>
+        <x:v>선택한 작업의 준비·금지·완료 조건을 담은 확인 카드를 생성하는 기능을 만든다. 카드의 각 조건을 원문과 대조해 문서 밖 절차를 제거하고, 다른 제공 작업에도 적용해 결과를 검증한다. 다음 회차에는 검토한 설비·문서 근거를 점검 요청 초안에 연결한다.</x:v>
       </x:c>
       <x:c r="D25" s="144" t="n">
-        <x:v>50</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="26" s="1" customFormat="1" ht="28" customHeight="1">
@@ -6711,7 +6707,7 @@
         <x:v>시간(분)</x:v>
       </x:c>
     </x:row>
-    <x:row r="30" s="1" customFormat="1" ht="92" customHeight="1">
+    <x:row r="30" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A30" s="141" t="str">
         <x:v>이론</x:v>
       </x:c>
@@ -6719,10 +6715,10 @@
         <x:v>원인 근거와 점검 요청 구조 이해하기</x:v>
       </x:c>
       <x:c r="C30" s="141" t="str">
-        <x:v>원인 후보를 뒷받침하는 설비·센서·문서 근거를 구분한다. 원인 분석 결과를 점검 대상·근거·확인 항목으로 바꾸는 방법을 살펴보고, 미확정 원인과 실제 확인된 사실을 구분한다.</x:v>
+        <x:v>원인 후보를 나열하는 데서 나아가 점검 대상·근거·확인 항목을 한 요청으로 만든다. 원인 후보를 뒷받침하는 설비·센서·문서 근거를 구분한다. 원인 분석 결과를 점검 대상·근거·확인 항목으로 바꾸는 방법을 살펴보고, 미확정 원인과 실제 확인된 사실을 구분한다.</x:v>
       </x:c>
       <x:c r="D30" s="142" t="n">
-        <x:v>50</x:v>
+        <x:v>30</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="92" customHeight="1">
@@ -6736,7 +6732,7 @@
         <x:v>포털 에이전트의 도구와 근거를 확인한다. VS Code에서 설비 증거를 읽어 원인 후보와 점검 순서를 제안하는 기능을 만들고, 제안의 각 항목에 사용한 근거가 표시되는지 확인한다.</x:v>
       </x:c>
       <x:c r="D31" s="144" t="n">
-        <x:v>50</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="32" s="1" customFormat="1" ht="92" customHeight="1">
@@ -6753,7 +6749,7 @@
         <x:v>50</x:v>
       </x:c>
     </x:row>
-    <x:row r="33" s="1" customFormat="1" ht="92" customHeight="1">
+    <x:row r="33" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A33" s="143" t="str">
         <x:v>실습</x:v>
       </x:c>
@@ -6761,10 +6757,10 @@
         <x:v>점검 요청 초안을 만들고 검증하기</x:v>
       </x:c>
       <x:c r="C33" s="143" t="str">
-        <x:v>점검 대상·근거·확인 항목을 담은 요청 초안을 만든다. 자료가 누락되거나 원인이 확정되지 않은 입력을 넣어 확인 질문이나 가설 표시가 남는지 검증한다. 근거 없는 단정을 수정해 요청 결과를 완성한다.</x:v>
+        <x:v>점검 대상·근거·확인 항목을 담은 요청 초안을 만든다. 자료가 누락되거나 원인이 확정되지 않은 입력을 넣어 확인 질문이나 가설 표시가 남는지 검증한다. 근거 없는 단정을 수정해 요청 결과를 완성한다. 다음 회차에는 반복하는 후속 업무를 스킬로 만들고 변경 자료를 확인해 협의 안건을 정리한다.</x:v>
       </x:c>
       <x:c r="D33" s="144" t="n">
-        <x:v>50</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="34" s="1" customFormat="1" ht="28" customHeight="1">
@@ -6806,7 +6802,7 @@
         <x:v>시간(분)</x:v>
       </x:c>
     </x:row>
-    <x:row r="38" s="1" customFormat="1" ht="92" customHeight="1">
+    <x:row r="38" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A38" s="141" t="str">
         <x:v>이론</x:v>
       </x:c>
@@ -6814,10 +6810,10 @@
         <x:v>스킬·도구 조합·변경 근거 이해하기</x:v>
       </x:c>
       <x:c r="C38" s="141" t="str">
-        <x:v>재사용할 업무 지침과 실행 도구의 역할을 구분한다. 회의록의 결정·담당·기한과 Git 변경 기록·시각 정보를 연결해 완료·미결·변경 내용을 판단하는 기준을 이해한다.</x:v>
+        <x:v>회의에서 정한 업무와 변경 기록을 비교하여 다음에 확인할 안건을 근거와 함께 만든다. 재사용할 업무 지침과 실행 도구의 역할을 구분한다. 회의록의 결정·담당·기한과 Git 변경 기록·시각 정보를 연결해 완료·미결·변경 내용을 판단하는 기준을 이해한다.</x:v>
       </x:c>
       <x:c r="D38" s="142" t="n">
-        <x:v>50</x:v>
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="39" s="1" customFormat="1" ht="92" customHeight="1">
@@ -6831,7 +6827,7 @@
         <x:v>공통 읽기 도구와 파일·Git·시간 MCP를 연결해 호출 결과를 확인한다. 제공 회의록 두 건과 점검 메모에서 결정·담당·기한·근거를 추출하는 스킬을 만들고, 없는 정보는 미정으로 남기는지 확인한다.</x:v>
       </x:c>
       <x:c r="D39" s="144" t="n">
-        <x:v>50</x:v>
+        <x:v>55</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="92" customHeight="1">
@@ -6848,7 +6844,7 @@
         <x:v>50</x:v>
       </x:c>
     </x:row>
-    <x:row r="41" s="1" customFormat="1" ht="92" customHeight="1">
+    <x:row r="41" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A41" s="143" t="str">
         <x:v>실습</x:v>
       </x:c>
@@ -6856,10 +6852,10 @@
         <x:v>다음 협의 안건을 만들고 검증하기</x:v>
       </x:c>
       <x:c r="C41" s="143" t="str">
-        <x:v>회의 업무 목록과 변경 기록을 합쳐 완료·미결·변경 사항 및 다음 협의에서 확인할 안건을 생성한다. 안건의 근거를 원문과 대조하고 같은 입력을 다시 실행해 필수 정보가 유지되는지 확인한다.</x:v>
+        <x:v>회의 업무 목록과 변경 기록을 합쳐 완료·미결·변경 사항 및 다음 협의에서 확인할 안건을 생성한다. 안건의 근거를 원문과 대조하고 같은 입력을 다시 실행해 필수 정보가 유지되는지 확인한다. 다음 회차에는 점검 요청 기능의 누락 입력과 변경 요구를 명세하고 검증한다.</x:v>
       </x:c>
       <x:c r="D41" s="144" t="n">
-        <x:v>50</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="42" s="1" customFormat="1" ht="28" customHeight="1">
@@ -6901,7 +6897,7 @@
         <x:v>시간(분)</x:v>
       </x:c>
     </x:row>
-    <x:row r="46" s="1" customFormat="1" ht="92" customHeight="1">
+    <x:row r="46" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A46" s="141" t="str">
         <x:v>이론</x:v>
       </x:c>
@@ -6909,10 +6905,10 @@
         <x:v>질문·승인·명세와 기대 결과 이해하기</x:v>
       </x:c>
       <x:c r="C46" s="141" t="str">
-        <x:v>필수 입력이 없을 때의 질문·보류와 사람 승인을 구분한다. 기능의 입력·출력·제약·완료 기준을 명세하고, 정상·누락·변경·기존 기능을 검증할 기대 결과로 바꾸는 방법을 익힌다.</x:v>
+        <x:v>점검 요청의 정보 누락·추가 답변·기능 변경을 처리하면서 기존 승인 조건을 보존한다. 필수 입력이 없을 때의 질문·보류와 사람 승인을 구분한다. 기능의 입력·출력·제약·완료 기준을 명세하고, 정상·누락·변경·기존 기능을 검증할 기대 결과로 바꾸는 방법을 익힌다.</x:v>
       </x:c>
       <x:c r="D46" s="142" t="n">
-        <x:v>50</x:v>
+        <x:v>30</x:v>
       </x:c>
     </x:row>
     <x:row r="47" s="1" customFormat="1" ht="92" customHeight="1">
@@ -6926,7 +6922,7 @@
         <x:v>포털의 승인·보류 상태를 확인한다. 점검 요청 초안의 필수 정보가 빠졌을 때 질문하고, 추가 답변을 반영해 다시 판단하는 흐름을 구현한다. 사람이 승인할 결과가 자동 확정되지 않는지 확인한다.</x:v>
       </x:c>
       <x:c r="D47" s="144" t="n">
-        <x:v>50</x:v>
+        <x:v>45</x:v>
       </x:c>
     </x:row>
     <x:row r="48" s="1" customFormat="1" ht="92" customHeight="1">
@@ -6940,10 +6936,10 @@
         <x:v>기존 점검 요청 기능에서 필요한 변경 한 건을 정한다. 입력·출력·사람 확인·완료 기준을 spec.md에 적고 기능을 구현한다. 변경 전부터 유지해야 할 출력 형식과 승인 조건을 함께 대조한다.</x:v>
       </x:c>
       <x:c r="D48" s="142" t="n">
-        <x:v>50</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="49" ht="92" customHeight="1">
+        <x:v>65</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="108" customHeight="1">
       <x:c r="A49" s="143" t="str">
         <x:v>실습</x:v>
       </x:c>
@@ -6951,10 +6947,10 @@
         <x:v>정상·누락·회귀 시나리오 검증하기</x:v>
       </x:c>
       <x:c r="C49" s="143" t="str">
-        <x:v>직접 정한 정상·정보 누락·변경 요구의 기대 결과를 Given/When/Then으로 작성한다. 실제 출력을 비교해 어긋난 조건을 수정하고, 기존 점검 요청과 승인 조건도 다시 실행해 회귀 오류가 없는지 확인한다.</x:v>
+        <x:v>직접 정한 정상·정보 누락·변경 요구의 기대 결과를 Given/When/Then으로 작성한다. 실제 출력을 비교해 어긋난 조건을 수정하고, 기존 점검 요청과 승인 조건도 다시 실행해 회귀 오류가 없는지 확인한다. 다음 회차에는 검증한 작업을 승인·반려 경로가 있는 BPMN으로 표현한다.</x:v>
       </x:c>
       <x:c r="D49" s="144" t="n">
-        <x:v>50</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="50" s="1" customFormat="1" ht="28" customHeight="1">
@@ -6996,7 +6992,7 @@
         <x:v>시간(분)</x:v>
       </x:c>
     </x:row>
-    <x:row r="54" s="1" customFormat="1" ht="92" customHeight="1">
+    <x:row r="54" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A54" s="141" t="str">
         <x:v>이론</x:v>
       </x:c>
@@ -7004,10 +7000,10 @@
         <x:v>BPMN 역할·분기·지연·실행 연결 이해하기</x:v>
       </x:c>
       <x:c r="C54" s="141" t="str">
-        <x:v>시작·종료 이벤트, 작업, 역할별 Lane, 승인 분기와 지연 알림의 의미를 설비 대응 사례로 구분한다. BPMN 그림의 각 작업이 에이전트·사람·시스템 중 누구에게 연결되는지 살펴보고, 승인 거절과 승인 대기 상태의 차이를 확인한다.</x:v>
+        <x:v>작업 순서·승인 역할·실행 연결을 구분하여 같은 BPMN을 그림과 실행 관점에서 읽는다. 시작·종료 이벤트, 작업, 역할별 Lane, 승인 분기와 지연 알림의 의미를 설비 대응 사례로 구분한다. BPMN 그림의 각 작업이 에이전트·사람·시스템 중 누구에게 연결되는지 살펴보고, 승인 거절과 승인 대기 상태의 차이를 확인한다.</x:v>
       </x:c>
       <x:c r="D54" s="142" t="n">
-        <x:v>50</x:v>
+        <x:v>30</x:v>
       </x:c>
     </x:row>
     <x:row r="55" s="1" customFormat="1" ht="92" customHeight="1">
@@ -7021,7 +7017,7 @@
         <x:v>bpmn.io에서 시작→요청 확인→승인 또는 반려→종료를 그린다. 이어 쿨러 경보→원인 분석·조치 제안→운전원 승인→설비 명령→효과 확인→보고로 흐름을 확장하고, 담당 역할에 맞게 작업을 Lane에 배치한다.</x:v>
       </x:c>
       <x:c r="D55" s="144" t="n">
-        <x:v>50</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="56" s="1" customFormat="1" ht="92" customHeight="1">
@@ -7038,7 +7034,7 @@
         <x:v>50</x:v>
       </x:c>
     </x:row>
-    <x:row r="57" s="1" customFormat="1" ht="92" customHeight="1">
+    <x:row r="57" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A57" s="143" t="str">
         <x:v>실습</x:v>
       </x:c>
@@ -7046,10 +7042,10 @@
         <x:v>BPMN과 등록된 실행 연결 비교하기</x:v>
       </x:c>
       <x:c r="C57" s="143" t="str">
-        <x:v>bpmn.io에서 작성한 설비 대응 흐름과 포털에 등록된 기준 흐름을 비교한다. 제공 매핑 자료에서 시작 이벤트·에이전트·운전원 승인·설비 명령·재관측 작업의 연결을 찾는다. 자신이 그린 각 작업이 어떤 실행 기능에 대응하는지 표시하고, 그림 파일과 실행 정의를 구분한다.</x:v>
+        <x:v>bpmn.io에서 작성한 설비 대응 흐름과 포털에 등록된 기준 흐름을 비교한다. 제공 매핑 자료에서 시작 이벤트·에이전트·운전원 승인·설비 명령·재관측 작업의 연결을 찾는다. 자신이 그린 각 작업이 어떤 실행 기능에 대응하는지 표시하고, 그림 파일과 실행 정의를 구분한다. 다음 회차에는 등록된 흐름의 실행 이력을 대조하고 교대 인수인계 흐름을 구성한다.</x:v>
       </x:c>
       <x:c r="D57" s="144" t="n">
-        <x:v>50</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="58" s="1" customFormat="1" ht="28" customHeight="1">
@@ -7091,7 +7087,7 @@
         <x:v>시간(분)</x:v>
       </x:c>
     </x:row>
-    <x:row r="62" s="1" customFormat="1" ht="92" customHeight="1">
+    <x:row r="62" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A62" s="141" t="str">
         <x:v>실습</x:v>
       </x:c>
@@ -7099,10 +7095,10 @@
         <x:v>실행 상태를 이해하고 정상·예외 경로 확인하기</x:v>
       </x:c>
       <x:c r="C62" s="141" t="str">
-        <x:v>포털에 이미 등록된 설비 대응 흐름을 쿨러 열화 시나리오로 실행한다. 에이전트 판단→운전원 승인→설비 명령→재관측→완료 기록을 따라간다. 승인 대기와 반려 결과를 비교하고, 자신이 그린 BPMN의 작업·분기와 실행 이력을 대조한다.</x:v>
+        <x:v>설비 대응의 실행 이력에서 조건과 결과를 확인하고 교대의 검토·보완 흐름을 구성한다. 포털에 이미 등록된 설비 대응 흐름을 쿨러 열화 시나리오로 실행한다. 에이전트 판단→운전원 승인→설비 명령→재관측→완료 기록을 따라간다. 승인 대기와 반려 결과를 비교하고, 자신이 그린 BPMN의 작업·분기와 실행 이력을 대조한다.</x:v>
       </x:c>
       <x:c r="D62" s="142" t="n">
-        <x:v>50</x:v>
+        <x:v>45</x:v>
       </x:c>
     </x:row>
     <x:row r="63" s="1" customFormat="1" ht="92" customHeight="1">
@@ -7116,7 +7112,7 @@
         <x:v>자신의 BPMN 그림과 실행 이력의 작업·역할·분기 차이를 찾아 그림을 수정한다. 교대 인수인계에 필요한 설비·교대·기준 시각·작업 메모를 정하고, 인계자 검토와 인수자 확인을 완료 조건으로 작성한다.</x:v>
       </x:c>
       <x:c r="D63" s="144" t="n">
-        <x:v>50</x:v>
+        <x:v>30</x:v>
       </x:c>
     </x:row>
     <x:row r="64" s="1" customFormat="1" ht="98" customHeight="1">
@@ -7130,10 +7126,10 @@
         <x:v>강사 코드로 열린 교대 실습에서 제공 보충 매뉴얼을 선택한다. 준비된 추출 결과의 절차·조건·근거를 원문과 비교하고 검토한 항목을 기존 제조 지식에 추가한다. 추가된 지식의 식별자와 원문 연결을 확인한다. 교대 실습에서 허용된 설비·정비·ERP 조회 도구로 인계안을 작성하는 에이전트·스킬을 구성한다. 이름·설명·스킬에 확인할 항목을 적고, 완료 메모와 열린 작업지시 또는 입고 예정과 실제 재고가 다를 때 확인 사항으로 남기는지 결과와 원천을 대조한다.</x:v>
       </x:c>
       <x:c r="D64" s="142" t="n">
-        <x:v>50</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="65" s="1" customFormat="1" ht="92" customHeight="1">
+        <x:v>75</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A65" s="143" t="str">
         <x:v>실습</x:v>
       </x:c>
@@ -7141,7 +7137,7 @@
         <x:v>제공 인수인계 BPMN의 에이전트 배정·등록하기</x:v>
       </x:c>
       <x:c r="C65" s="143" t="str">
-        <x:v>제공 교대 BPMN을 bpmn.io에서 열어 작업 이름과 배치를 정리한다. 시작 입력·검토·보완 분기를 유지하고 세 초안 단계에 교대 에이전트를 배정하여 별도 판본을 등록한다. 설비·교대 정보를 입력해 인계안 작성→인계자 검토→인수자 보완 요청→재검토→인수 확인을 수행하고 근거와 완료 기록을 확인한다.</x:v>
+        <x:v>제공 교대 BPMN을 bpmn.io에서 열어 이름과 배치를 정리한다. 시작 입력·검토·보완 분기를 유지하고 세 초안 단계에 교대 에이전트를 배정하여 별도 판본을 등록한다. 시작 폼의 설비·교대 입력과 각 단계 배정을 확인한다. 다음 회차에는 정비·구매 기록을 확인하고 교대 흐름의 인수 확인까지 완료한다.</x:v>
       </x:c>
       <x:c r="D65" s="144" t="n">
         <x:v>50</x:v>
@@ -7186,7 +7182,7 @@
         <x:v>시간(분)</x:v>
       </x:c>
     </x:row>
-    <x:row r="70" s="1" customFormat="1" ht="92" customHeight="1">
+    <x:row r="70" s="1" customFormat="1" ht="108" customHeight="1">
       <x:c r="A70" s="141" t="str">
         <x:v>실습</x:v>
       </x:c>
@@ -7194,10 +7190,10 @@
         <x:v>업무별 시작 조건을 비교하고 정비 흐름 설계하기</x:v>
       </x:c>
       <x:c r="C70" s="141" t="str">
-        <x:v>냉각 경보·정기 점검 도래·재고 부족의 시작 조건과 완료 결과를 비교한다. 정기 점검→정비 계획→설비보전팀장 승인 또는 거절→정비 오더→생산팀 공지 흐름을 bpmn.io에서 작성하고 담당 역할과 분기 조건을 연결한다.</x:v>
+        <x:v>정비·구매의 완료 의미를 비교하고 교대 인계 내용과 검토·확인 기록을 연결한다. 냉각 경보·정기 점검 도래·재고 부족의 시작 조건과 완료 결과를 비교한다. 정기 점검→정비 계획→설비보전팀장 승인 또는 거절→정비 오더→생산팀 공지 흐름을 bpmn.io에서 작성하고 담당 역할과 분기 조건을 연결한다.</x:v>
       </x:c>
       <x:c r="D70" s="142" t="n">
-        <x:v>50</x:v>
+        <x:v>30</x:v>
       </x:c>
     </x:row>
     <x:row r="71" s="1" customFormat="1" ht="92" customHeight="1">
@@ -7211,7 +7207,7 @@
         <x:v>포털의 정기 점검 시나리오로 등록된 정비 흐름을 실행한다. 정비 계획·승인·작업지시·예약 또는 출고·생산 공지의 처리 기록을 확인한다. 승인과 반려 사례를 비교하여 정비 오더가 만들어지는 조건을 자신의 BPMN과 대조한다.</x:v>
       </x:c>
       <x:c r="D71" s="144" t="n">
-        <x:v>50</x:v>
+        <x:v>40</x:v>
       </x:c>
     </x:row>
     <x:row r="72" s="1" customFormat="1" ht="92" customHeight="1">
@@ -7225,10 +7221,10 @@
         <x:v>bpmn.io에서 재고 부족→구매 제안→승인 또는 반려→발주→통지→입고 반영 흐름을 그린다. 포털의 재고 보충 시나리오로 등록된 구매 흐름을 실행한다. 수업용 업무 시스템에서 발주·공급사 통지·입고·재고 반영 기록을 확인하고, 반려 사례의 처리 결과와 비교한다. 자신의 BPMN에서 각 결과에 대응하는 작업을 찾는다.</x:v>
       </x:c>
       <x:c r="D72" s="142" t="n">
-        <x:v>50</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="73" s="1" customFormat="1" ht="92" customHeight="1">
+        <x:v>60</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" s="1" customFormat="1" ht="145" customHeight="1">
       <x:c r="A73" s="143" t="str">
         <x:v>실습</x:v>
       </x:c>
@@ -7236,10 +7232,10 @@
         <x:v>교대 인수인계를 완성하고 ProcessGPT 연결 보기</x:v>
       </x:c>
       <x:c r="C73" s="143" t="str">
-        <x:v>교대 인수인계 흐름에 설비·교대 정보를 입력하고 정상·기록 불일치·정보 누락 사례를 실행한다. 인계자 검토, 인수자의 보완 요청과 확인을 거쳐 인계 내용·근거·완료 기록을 대조한다(30분). ProcessGPT 시연을 보며 자신이 만든 지식·에이전트·업무 흐름이 제품의 작업함과 실행 기록에 어떻게 연결되는지 비교한다(20분).</x:v>
+        <x:v>교대 흐름에 설비·교대 정보를 입력하고 인계안의 근거와 원천 기록을 대조한다. 인계자 검토→인수자 보완 요청→재검토→인수 확인을 거쳐 완료 기록을 확인한다. 실제 결과에서 빠진 정보나 불일치가 있으면 확인 사항으로 남긴다(50분). 이어 ProcessGPT 시연에서 지식·에이전트·사람 작업·실행 기록이 어떻게 연결되는지 자신이 수행한 흐름과 비교한다(20분). 각자 인계 결과의 근거와 추가 확인할 사항을 설명한다.</x:v>
       </x:c>
       <x:c r="D73" s="144" t="n">
-        <x:v>50</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="74" s="1" customFormat="1" ht="28" customHeight="1">

</xml_diff>

<commit_message>
Fix offline periods at 50 minutes and rebalance instructor roles
</commit_message>
<xml_diff>
--- a/문서/교재/실라버스/피지컬AI_실라버스_최종본.xlsx
+++ b/문서/교재/실라버스/피지컬AI_실라버스_최종본.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="통합반 온라인 44H" sheetId="1" r:id="R8bf50ea5b26f4890"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="실전반 온라인 32H" sheetId="2" r:id="R604ce3e088134b2b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="통합반 오프라인 정규 10회" sheetId="3" r:id="Rf4d11f162fb44998"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="실전반 오프라인 정규 9회" sheetId="4" r:id="Rbb8e2240d91e468a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="통합반 온라인 44H" sheetId="1" r:id="Re93bdb10729e45f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="실전반 온라인 32H" sheetId="2" r:id="R47caf9fe29b5499e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="통합반 오프라인 정규 10회" sheetId="3" r:id="R680531491d234437"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="실전반 오프라인 정규 9회" sheetId="4" r:id="R3521eeae494949c8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4795,7 +4795,7 @@
     </x:row>
     <x:row r="2" s="1" customFormat="1" ht="48" customHeight="1">
       <x:c r="A2" s="135" t="str">
-        <x:v>온라인 선행학습 후 목적·핵심 개념을 연결하고 주요 실습을 직접 수행합니다. 수업200분·휴식40분의 기본 배정이며 실제 진행은 강사가 조절합니다. 이전 개인 결과 없이 제공 시작본으로 시작할 수 있습니다.</x:v>
+        <x:v>매회 50분 수업·10분 휴식 × 4교시입니다(수업200분·휴식40분). 온라인 선행학습을 바탕으로 목적·핵심 개념을 연결하고 실습합니다. 이전 개인 결과 없이 제공 시작본으로 시작할 수 있습니다.</x:v>
       </x:c>
       <x:c r="B2" s="135"/>
       <x:c r="C2" s="135"/>
@@ -4840,7 +4840,7 @@
         <x:v>HYD의 완성 흐름을 먼저 확인하고, 판단 근거를 표현하는 관계도와 그래프를 직접 다룬다. HYD가 유압 설비와 업무 시스템을 연결한 수업용 시스템임을 이해한다. 설비·센서 데이터 수집→상태 관찰→지식에 근거한 판단→사람 승인→조치→결과 확인의 전체 구조를 살펴본다. 포털에서 확인할 설비 화면·지식 지도·에이전트·작업함의 역할을 구분한다. 이번 과정에서 관계 모델을 만들고, 근거를 조회하는 에이전트와 업무 흐름으로 연결할 학습 목표를 확인한다.</x:v>
       </x:c>
       <x:c r="D6" s="142" t="n">
-        <x:v>40</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="7" s="1" customFormat="1" ht="125" customHeight="1">
@@ -4854,7 +4854,7 @@
         <x:v>강사가 실제 HYD 포털을 열어 보여 주는 설비 상태·센서 값과 쿨러 열화 시나리오를 따라간다. 경보 발생→에이전트의 원인·조치 추천→운전원 승인→설비 명령→센서 값 재확인과 완료 기록을 보고, 추천·승인·실행의 차이를 구분한다. 지식 지도에서 판단에 사용된 설비·센서·고장·조치 연결을 확인한다. 이어 arrows.app에서 방금 본 대상을 노드와 관계로 그려 각 화살표를 문장으로 읽는다.</x:v>
       </x:c>
       <x:c r="D7" s="144" t="n">
-        <x:v>60</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="8" s="1" customFormat="1" ht="92" customHeight="1">
@@ -4935,7 +4935,7 @@
         <x:v>앞서 만든 작은 모델을 다시 적재해도 중복되지 않게 하고 작업 절차를 연결한다. 고유 식별자로 같은 대상을 구분하는 방법과 반복 적재 시 중복을 막는 원리를 살펴본다. 필수값·자료형·관계 끝점 제약을 설비 모델에 대어 확인하고, 고장·조치와 SOP의 전제·금지·완료 조건이 연결되는 구조를 이해한다.</x:v>
       </x:c>
       <x:c r="D14" s="142" t="n">
-        <x:v>35</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="15" s="1" customFormat="1" ht="92" customHeight="1">
@@ -4949,7 +4949,7 @@
         <x:v>설비 모델의 고유 ID·자료형·필수값·관계 끝점을 원자료와 대조해 보완한다. 모델을 적재하고 설비별 센서·부품을 조회한다. 같은 자료를 다시 적재한 뒤 노드와 관계가 불필요하게 늘어나지 않았는지 확인한다.</x:v>
       </x:c>
       <x:c r="D15" s="144" t="n">
-        <x:v>55</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="16" s="1" customFormat="1" ht="92" customHeight="1">
@@ -4977,7 +4977,7 @@
         <x:v>제공 SOP에서 작업의 전제·금지·수행 단계·완료 조건을 구분한다. 고장 유형과 조치 방법을 기존 설비 모델의 식별자에 연결하고, 선택한 고장에 적용할 절차와 금지 조건을 조회해 원문과 비교한다. 다음 회차에는 연결한 SOP 조건으로 조치의 허용·제외와 성과를 판정한다.</x:v>
       </x:c>
       <x:c r="D17" s="144" t="n">
-        <x:v>60</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="18" s="1" customFormat="1" ht="28" customHeight="1">
@@ -5030,7 +5030,7 @@
         <x:v>관계와 절차를 읽는 데서 나아가 입력 조건에 따라 가능한 조치와 그 이유를 반환한다. SOP의 작업 순서와 DMN의 판단 조건을 구분한다. 입력값·단위·연산자·경계값으로 조치 허용·제외를 표현하고, 허용된 후보끼리 비용·생산·품질·에너지 성과를 비교하는 이유를 사례로 확인한다.</x:v>
       </x:c>
       <x:c r="D22" s="142" t="n">
-        <x:v>40</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="23" s="1" customFormat="1" ht="92" customHeight="1">
@@ -5044,7 +5044,7 @@
         <x:v>포털 What-if에서 운전 조건을 바꿔 조치 허용·제외와 순위 변화를 비교한다. 제공 SOP에서 입력·단위·경계·출처를 뽑아 결정표를 작성하고, 각 조건이 어떤 조치를 허용하거나 제외하는지 표시한다.</x:v>
       </x:c>
       <x:c r="D23" s="144" t="n">
-        <x:v>45</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="24" s="1" customFormat="1" ht="92" customHeight="1">
@@ -5058,7 +5058,7 @@
         <x:v>VS Code에서 결정표를 입력으로 사용해 조치의 허용·제외와 사유를 반환하는 기능을 만든다. 정상 조건, 경계값, 여러 규칙이 동시에 맞는 경우, 금지 조건을 입력해 실제 결과를 조건표와 대조한다.</x:v>
       </x:c>
       <x:c r="D24" s="142" t="n">
-        <x:v>60</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="25" s="1" customFormat="1" ht="108" customHeight="1">
@@ -5072,7 +5072,7 @@
         <x:v>허용된 조치 후보만 비용·생산 영향·품질·에너지 기준으로 비교한다. 경계값이나 필수 정보 누락에 따라 결과가 달라지는지 확인하고, 선택 이유와 추가 확인 사항을 출력한다. 추천 결과와 사람의 실행 승인을 구분한다. 다음 회차에는 사용한 조건의 원문을 추출·검토하여 근거 지식을 보강한다.</x:v>
       </x:c>
       <x:c r="D25" s="144" t="n">
-        <x:v>55</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="26" s="1" customFormat="1" ht="28" customHeight="1">
@@ -5125,7 +5125,7 @@
         <x:v>판단에 쓰는 조건을 원문까지 확인할 수 있도록 문서 추출·검토·적재를 연결한다. 매뉴얼 원문, AI가 추출한 후보, 검토를 거친 지식을 구분한다. 부정 조건·단위·작업 순서가 잘못 추출된 사례를 원문과 대조하고, 문서 ID·페이지·인용 구간을 지식과 함께 보존하는 이유를 이해한다.</x:v>
       </x:c>
       <x:c r="D30" s="142" t="n">
-        <x:v>35</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="31" s="1" customFormat="1" ht="92" customHeight="1">
@@ -5139,7 +5139,7 @@
         <x:v>포털의 제공 매뉴얼 원문과 등록된 추출 결과를 비교한다. VS Code에서 제공 문서의 표·작업 절차·수치·단위·금지 조건을 구조화하는 기능을 만들고 문서 ID·페이지 또는 구간·인용을 함께 출력한다.</x:v>
       </x:c>
       <x:c r="D31" s="144" t="n">
-        <x:v>55</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="32" s="1" customFormat="1" ht="92" customHeight="1">
@@ -5153,7 +5153,7 @@
         <x:v>추출 후보의 조건·단위·순서를 원문과 비교해 채택·수정·제외한다. 채택한 항목을 기존 랩 그래프의 클래스와 식별자에 맞춰 적재하고, 고장→원인→조치→근거 문서 관계를 조회한다.</x:v>
       </x:c>
       <x:c r="D32" s="142" t="n">
-        <x:v>65</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="33" s="1" customFormat="1" ht="108" customHeight="1">
@@ -5167,7 +5167,7 @@
         <x:v>제공된 다른 매뉴얼에 같은 추출 기능을 적용한다. 빠진 조건이나 잘못 연결된 대상이 있는지 원문과 대조하고 수정한다. 그래프에 반영한 지식에서 문서 출처를 다시 찾아 검토 결과와 일치하는지 확인한다. 이 검토 지식과 센서 자료를 다음 회차 에이전트의 근거로 사용한다.</x:v>
       </x:c>
       <x:c r="D33" s="144" t="n">
-        <x:v>45</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="34" s="1" customFormat="1" ht="28" customHeight="1">
@@ -5220,7 +5220,7 @@
         <x:v>검토한 지식과 현재 입력을 이용해 원인 후보·후속 업무·이상 구간을 확인한다. LLM의 답변, RAG의 근거 검색, 에이전트의 목표·도구·반복 실행을 구분한다. 설비 지식과 현재 센서 값을 각각 어디서 얻는지 살펴보고, 근거 부족이나 도구 오류가 생겼을 때 멈추거나 확인을 요청할 조건을 정한다.</x:v>
       </x:c>
       <x:c r="D38" s="142" t="n">
-        <x:v>35</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="39" s="1" customFormat="1" ht="92" customHeight="1">
@@ -5234,7 +5234,7 @@
         <x:v>포털 에이전트의 목표·도구·근거를 확인한다. VS Code에서 설비·센서·고장·SOP 관계와 센서 입력을 읽어 원인 후보·증거·다음 점검 순서를 제안하는 에이전트를 만든다. 확인되지 않은 원인이 가설로 표시되는지 검토한다.</x:v>
       </x:c>
       <x:c r="D39" s="144" t="n">
-        <x:v>65</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="92" customHeight="1">
@@ -5248,7 +5248,7 @@
         <x:v>제공 불량 접수 메시지와 분류 기준으로 품질 유형·추가 확인 항목·담당 부서·대응 초안을 출력하는 에이전트를 만든다. 원인이 확정되지 않은 사례를 입력해 단정 대신 조사 요청을 남기는지 확인한다.</x:v>
       </x:c>
       <x:c r="D40" s="142" t="n">
-        <x:v>55</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="41" s="1" customFormat="1" ht="108" customHeight="1">
@@ -5262,7 +5262,7 @@
         <x:v>센서 CSV의 시간·온도·압력 변화를 읽어 이상 구간을 시각화한다. 관련 태그와 조회 기간을 함께 표시하고 원자료와 비교한다. 원인 점검·품질 대응·시각화 결과에서 근거와 미확인 사항이 구분되는지 검토한다. 다음 회차에는 반복 작업의 지침을 스킬로 만들고 파일·Git·시간 도구를 조합한다.</x:v>
       </x:c>
       <x:c r="D41" s="144" t="n">
-        <x:v>45</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="42" s="1" customFormat="1" ht="28" customHeight="1">
@@ -5315,7 +5315,7 @@
         <x:v>에이전트의 반복 작업을 재사용 지침과 도구 호출로 나누어 구성한다. SKILL.md에 담는 목적·입력·출력·절차와 MCP 도구의 역할을 구분한다. 파일·Git·시간 도구의 입력과 반환값을 살펴보고, 읽기·쓰기 권한과 접근 가능한 경로가 작업에 미치는 영향을 확인한다.</x:v>
       </x:c>
       <x:c r="D46" s="142" t="n">
-        <x:v>30</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="47" s="1" customFormat="1" ht="92" customHeight="1">
@@ -5329,7 +5329,7 @@
         <x:v>준비된 MCP의 연결과 호출 결과를 확인한다. 회의록에서 결정사항·담당자·기한·출처를 추출하는 SKILL.md를 작성하고, 담당자나 기한이 없는 항목은 미정으로 남기는지 원문과 비교한다.</x:v>
       </x:c>
       <x:c r="D47" s="144" t="n">
-        <x:v>60</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="48" s="1" customFormat="1" ht="92" customHeight="1">
@@ -5343,7 +5343,7 @@
         <x:v>파일 내용 읽기→Git 변경 기록 확인→시간 정보 확인을 하나의 요청으로 연결한다. 각 도구의 반환값이 결과에 어떻게 사용됐는지 확인하고, 업무 목록의 변경 내용과 시점을 원자료에 대어 검증한다.</x:v>
       </x:c>
       <x:c r="D48" s="142" t="n">
-        <x:v>55</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="108" customHeight="1">
@@ -5357,7 +5357,7 @@
         <x:v>제공 학습 자료를 바탕으로 문항 생성→답변 입력→정답·원문 근거 피드백으로 이어지는 대화형 학습 코치를 만든다. 답변을 달리 입력해 피드백이 바뀌는지 확인하고, 피드백의 출처가 학습 자료에 있는지 대조한다. 다음 회차에는 정보 누락과 요구 변경에도 결과를 확인할 수 있도록 질문·명세·검증을 연결한다.</x:v>
       </x:c>
       <x:c r="D49" s="144" t="n">
-        <x:v>55</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="50" s="1" customFormat="1" ht="28" customHeight="1">
@@ -5410,7 +5410,7 @@
         <x:v>앞서 만든 업무 요청 기능의 누락 입력과 변경 요구를 다루고 기존 동작이 유지되는지 확인한다. 정보 확인 질문과 사람의 승인을 구분한다. 입력·출력·금지 조건·수용 기준을 명세로 표현하고, Given/When/Then으로 기대 행동을 정하는 방법을 익힌다. 새 기능의 동작과 기존 기능 보존을 함께 확인하는 이유를 이해한다.</x:v>
       </x:c>
       <x:c r="D54" s="142" t="n">
-        <x:v>40</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="55" s="1" customFormat="1" ht="108" customHeight="1">
@@ -5438,7 +5438,7 @@
         <x:v>같은 업무 요청 프로젝트에서 변경할 기능을 정하고 입력·출력·금지 조건·완료 기준을 spec.md로 작성한다. AI 코딩 도구로 변경을 구현한 뒤 기존 일반 요청과 변경 요청의 출력을 비교한다.</x:v>
       </x:c>
       <x:c r="D56" s="142" t="n">
-        <x:v>55</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="57" s="1" customFormat="1" ht="108" customHeight="1">
@@ -5452,7 +5452,7 @@
         <x:v>정상·정보 누락·변경 요구의 기대 결과를 Given/When/Then으로 작성해 실제 출력과 비교한다. 제공 센서·정비·부품 자료를 연결해 완료·미완료·다음 조치·근거 시각을 담은 인수인계 결과를 만들고 원자료와 대조한다. 다음 회차에는 검증한 작업을 사람의 승인과 함께 BPMN으로 표현한다.</x:v>
       </x:c>
       <x:c r="D57" s="144" t="n">
-        <x:v>55</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="28" customHeight="1">
@@ -5505,7 +5505,7 @@
         <x:v>개별 작업의 결과가 다음 작업으로 넘어가는 조건과 담당 역할을 그림으로 명확히 한다. 시작·종료 이벤트, 작업, 역할별 Lane, 승인 분기와 지연 알림의 의미를 설비 대응 사례로 구분한다. BPMN 그림의 각 작업이 에이전트·사람·시스템 중 누구에게 연결되는지 살펴보고, 승인 거절과 승인 대기 상태의 차이를 확인한다.</x:v>
       </x:c>
       <x:c r="D62" s="142" t="n">
-        <x:v>35</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="63" s="1" customFormat="1" ht="92" customHeight="1">
@@ -5519,7 +5519,7 @@
         <x:v>bpmn.io에서 시작→요청 확인→승인 또는 반려→종료를 그린다. 이어 쿨러 경보→원인 분석·조치 제안→운전원 승인→설비 명령→효과 확인→보고로 흐름을 확장하고, 담당 역할에 맞게 작업을 Lane에 배치한다.</x:v>
       </x:c>
       <x:c r="D63" s="144" t="n">
-        <x:v>65</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="64" s="1" customFormat="1" ht="92" customHeight="1">
@@ -5533,7 +5533,7 @@
         <x:v>승인·거절 분기와 각각의 종료 경로를 연결한다. 거절 경로에서 설비 명령으로 진행되지 않는지 확인하고, 승인 작업을 취소하지 않는 지연 알림 Timer를 추가한다. 각 경로를 따라가며 분기 조건과 연결 누락을 점검한다.</x:v>
       </x:c>
       <x:c r="D64" s="142" t="n">
-        <x:v>55</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="65" s="1" customFormat="1" ht="108" customHeight="1">
@@ -5547,7 +5547,7 @@
         <x:v>bpmn.io에서 작성한 설비 대응 흐름과 포털에 등록된 기준 흐름을 비교한다. 제공 매핑 자료에서 시작 이벤트·에이전트·운전원 승인·설비 명령·재관측 작업의 연결을 찾는다. 자신이 그린 각 작업이 어떤 실행 기능에 대응하는지 표시하고, 그림 파일과 실행 정의를 구분한다. 다음 회차에는 등록된 흐름을 실행해 이 그림과 실제 처리 이력을 대조한다.</x:v>
       </x:c>
       <x:c r="D65" s="144" t="n">
-        <x:v>45</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="66" s="1" customFormat="1" ht="28" customHeight="1">
@@ -5600,7 +5600,7 @@
         <x:v>앞서 그린 BPMN과 실제 실행을 비교하고 같은 구조를 교대 검토·확인 흐름에 연결한다. 포털에 이미 등록된 설비 대응 흐름을 쿨러 열화 시나리오로 실행한다. 에이전트 판단→운전원 승인→설비 명령→재관측→완료 기록을 따라간다. 승인 대기와 반려 결과를 비교하고, 자신이 그린 BPMN의 작업·분기와 실행 이력을 대조한다.</x:v>
       </x:c>
       <x:c r="D70" s="142" t="n">
-        <x:v>45</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="71" s="1" customFormat="1" ht="92" customHeight="1">
@@ -5614,7 +5614,7 @@
         <x:v>자신의 BPMN 그림과 실행 이력의 작업·역할·분기 차이를 찾아 그림을 수정한다. 교대 인수인계에 필요한 설비·교대·기준 시각·작업 메모를 정하고, 인계자 검토와 인수자 확인을 완료 조건으로 작성한다.</x:v>
       </x:c>
       <x:c r="D71" s="144" t="n">
-        <x:v>35</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="72" s="1" customFormat="1" ht="98" customHeight="1">
@@ -5628,7 +5628,7 @@
         <x:v>강사 코드로 열린 교대 실습에서 제공 보충 매뉴얼을 선택한다. 준비된 추출 결과의 절차·조건·근거를 원문과 비교하고 검토한 항목을 기존 제조 지식에 추가한다. 추가된 지식의 식별자와 원문 연결을 확인한다. 교대 실습에서 허용된 설비·정비·ERP 조회 도구로 인계안을 작성하는 에이전트·스킬을 구성한다. 이름·설명·스킬에 확인할 항목을 적고, 완료 메모와 열린 작업지시 또는 입고 예정과 실제 재고가 다를 때 확인 사항으로 남기는지 결과와 원천을 대조한다.</x:v>
       </x:c>
       <x:c r="D72" s="142" t="n">
-        <x:v>70</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="73" s="1" customFormat="1" ht="108" customHeight="1">
@@ -5695,7 +5695,7 @@
         <x:v>설비 대응에서 익힌 패턴을 정비·구매에 적용하고 교대 인수인계의 검토·확인까지 마친다. 냉각 경보·정기 점검 도래·재고 부족의 시작 조건과 완료 결과를 비교한다. 정기 점검→정비 계획→설비보전팀장 승인 또는 거절→정비 오더→생산팀 공지 흐름을 bpmn.io에서 작성하고 담당 역할과 분기 조건을 연결한다.</x:v>
       </x:c>
       <x:c r="D78" s="142" t="n">
-        <x:v>35</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="79" s="1" customFormat="1" ht="92" customHeight="1">
@@ -5709,7 +5709,7 @@
         <x:v>포털의 정기 점검 시나리오로 등록된 정비 흐름을 실행한다. 정비 계획·승인·작업지시·예약 또는 출고·생산 공지의 처리 기록을 확인한다. 승인과 반려 사례를 비교하여 정비 오더가 만들어지는 조건을 자신의 BPMN과 대조한다.</x:v>
       </x:c>
       <x:c r="D79" s="144" t="n">
-        <x:v>35</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="80" s="1" customFormat="1" ht="92" customHeight="1">
@@ -5723,7 +5723,7 @@
         <x:v>bpmn.io에서 재고 부족→구매 제안→승인 또는 반려→발주→통지→입고 반영 흐름을 그린다. 포털의 재고 보충 시나리오로 등록된 구매 흐름을 실행한다. 수업용 업무 시스템에서 발주·공급사 통지·입고·재고 반영 기록을 확인하고, 반려 사례의 처리 결과와 비교한다. 자신의 BPMN에서 각 결과에 대응하는 작업을 찾는다.</x:v>
       </x:c>
       <x:c r="D80" s="142" t="n">
-        <x:v>60</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="81" s="1" customFormat="1" ht="145" customHeight="1">
@@ -5734,10 +5734,10 @@
         <x:v>교대 인수인계를 완성하고 ProcessGPT 연결 보기</x:v>
       </x:c>
       <x:c r="C81" s="143" t="str">
-        <x:v>교대 흐름에 설비·교대 정보를 입력하고 인계안의 근거와 원천 기록을 대조한다. 인계자 검토→인수자 보완 요청→재검토→인수 확인을 거쳐 완료 기록을 확인한다. 실제 결과에서 빠진 정보나 불일치가 있으면 확인 사항으로 남긴다(50분). 이어 ProcessGPT 시연에서 지식·에이전트·사람 작업·실행 기록이 어떻게 연결되는지 자신이 수행한 흐름과 비교한다(20분). 관계 모델·판단 근거·실행 기록을 연결하여 전체 과정을 설명한다.</x:v>
+        <x:v>교대 흐름에 설비·교대 정보를 입력하고 인계안의 근거와 원천 기록을 대조한다. 인계자 검토→인수자 보완 요청→재검토→인수 확인을 거쳐 완료 기록을 확인한다. 실제 결과에서 빠진 정보나 불일치가 있으면 확인 사항으로 남긴다(30분). 이어 ProcessGPT 시연에서 지식·에이전트·사람 작업·실행 기록이 어떻게 연결되는지 자신이 수행한 흐름과 비교한다(20분). 관계 모델·판단 근거·실행 기록을 연결하여 전체 과정을 설명한다.</x:v>
       </x:c>
       <x:c r="D81" s="144" t="n">
-        <x:v>70</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="82" s="1" customFormat="1" ht="28" customHeight="1">
@@ -6388,7 +6388,7 @@
     </x:row>
     <x:row r="2" s="1" customFormat="1" ht="48" customHeight="1">
       <x:c r="A2" s="135" t="str">
-        <x:v>온라인 선행학습 후 목적·핵심 개념을 연결하고 주요 실습을 직접 수행합니다. 수업200분·휴식40분의 기본 배정이며 실제 진행은 강사가 조절합니다. 이전 개인 결과 없이 제공 시작본으로 시작할 수 있습니다.</x:v>
+        <x:v>매회 50분 수업·10분 휴식 × 4교시입니다(수업200분·휴식40분). 온라인 선행학습을 바탕으로 목적·핵심 개념을 연결하고 실습합니다. 이전 개인 결과 없이 제공 시작본으로 시작할 수 있습니다.</x:v>
       </x:c>
       <x:c r="B2" s="135"/>
       <x:c r="C2" s="135"/>
@@ -6433,7 +6433,7 @@
         <x:v>HYD의 완성 흐름을 먼저 확인하고, 판단 근거를 표현하는 관계도와 그래프를 직접 다룬다. HYD가 유압 설비와 업무 시스템을 연결한 수업용 시스템임을 이해한다. 설비·센서 데이터 수집→상태 관찰→지식에 근거한 판단→사람 승인→조치→결과 확인의 전체 구조를 살펴본다. 포털에서 확인할 설비 화면·지식 지도·에이전트·작업함의 역할을 구분한다. 이번 과정에서 관계 모델을 만들고, 근거를 조회하는 에이전트와 업무 흐름으로 연결할 학습 목표를 확인한다.</x:v>
       </x:c>
       <x:c r="D6" s="142" t="n">
-        <x:v>40</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="7" s="1" customFormat="1" ht="125" customHeight="1">
@@ -6447,7 +6447,7 @@
         <x:v>강사가 실제 HYD 포털을 열어 보여 주는 설비 상태·센서 값과 쿨러 열화 시나리오를 따라간다. 경보 발생→에이전트의 원인·조치 추천→운전원 승인→설비 명령→센서 값 재확인과 완료 기록을 보고, 추천·승인·실행의 차이를 구분한다. 지식 지도에서 판단에 사용된 설비·센서·고장·조치 연결을 확인한다. 이어 arrows.app에서 방금 본 대상을 노드와 관계로 그려 각 화살표를 문장으로 읽는다.</x:v>
       </x:c>
       <x:c r="D7" s="144" t="n">
-        <x:v>60</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="8" s="1" customFormat="1" ht="92" customHeight="1">
@@ -6528,7 +6528,7 @@
         <x:v>설비·부품 연결 조회와 작업 조건표를 조합해 선택 근거가 보이는 조치 검토 결과를 만든다. 설비·부품·공급 정보를 연결해 답할 질문을 정한다. SOP의 작업 조건을 결정표로 표현하는 방법을 살펴보고, 조치 후보의 허용·제외 판정과 사람의 실행 승인이 서로 다른 단계임을 이해한다.</x:v>
       </x:c>
       <x:c r="D14" s="142" t="n">
-        <x:v>30</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="15" s="1" customFormat="1" ht="92" customHeight="1">
@@ -6556,7 +6556,7 @@
         <x:v>제공 SOP에서 입력·단위·연산자·경계·출처를 뽑아 조치 조건표를 만든다. 조건에 따라 허용·제외와 사유를 반환하는 기능을 구현하고, 허용 후보의 비용·생산·품질·에너지 성과를 비교한다.</x:v>
       </x:c>
       <x:c r="D16" s="142" t="n">
-        <x:v>70</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="17" s="1" customFormat="1" ht="108" customHeight="1">
@@ -6623,7 +6623,7 @@
         <x:v>매뉴얼의 조건을 추출·검토하고 특정 작업에서 바로 확인할 수 있는 카드로 바꾼다. 매뉴얼의 작업 조건을 추출 후보·검토 지식·작업 확인 자료로 전환하는 과정을 살펴본다. 문서 ID·페이지·인용 구간과 개정 정보를 보존하는 이유를 이해하고, 원문에 없는 내용을 판별한다.</x:v>
       </x:c>
       <x:c r="D22" s="142" t="n">
-        <x:v>30</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="23" s="1" customFormat="1" ht="92" customHeight="1">
@@ -6637,7 +6637,7 @@
         <x:v>포털의 제공 매뉴얼 원문과 등록된 추출 결과를 비교한다. VS Code에서 제공 작업의 조건·순서·단위·금지 조건과 출처를 추출하고, 잘못 해석한 항목을 원문과 대조해 수정한다.</x:v>
       </x:c>
       <x:c r="D23" s="144" t="n">
-        <x:v>60</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="24" s="1" customFormat="1" ht="92" customHeight="1">
@@ -6665,7 +6665,7 @@
         <x:v>선택한 작업의 준비·금지·완료 조건을 담은 확인 카드를 생성하는 기능을 만든다. 카드의 각 조건을 원문과 대조해 문서 밖 절차를 제거하고, 다른 제공 작업에도 적용해 결과를 검증한다. 다음 회차에는 검토한 설비·문서 근거를 점검 요청 초안에 연결한다.</x:v>
       </x:c>
       <x:c r="D25" s="144" t="n">
-        <x:v>60</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="26" s="1" customFormat="1" ht="28" customHeight="1">
@@ -6718,7 +6718,7 @@
         <x:v>원인 후보를 나열하는 데서 나아가 점검 대상·근거·확인 항목을 한 요청으로 만든다. 원인 후보를 뒷받침하는 설비·센서·문서 근거를 구분한다. 원인 분석 결과를 점검 대상·근거·확인 항목으로 바꾸는 방법을 살펴보고, 미확정 원인과 실제 확인된 사실을 구분한다.</x:v>
       </x:c>
       <x:c r="D30" s="142" t="n">
-        <x:v>30</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="92" customHeight="1">
@@ -6732,7 +6732,7 @@
         <x:v>포털 에이전트의 도구와 근거를 확인한다. VS Code에서 설비 증거를 읽어 원인 후보와 점검 순서를 제안하는 기능을 만들고, 제안의 각 항목에 사용한 근거가 표시되는지 확인한다.</x:v>
       </x:c>
       <x:c r="D31" s="144" t="n">
-        <x:v>60</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="32" s="1" customFormat="1" ht="92" customHeight="1">
@@ -6760,7 +6760,7 @@
         <x:v>점검 대상·근거·확인 항목을 담은 요청 초안을 만든다. 자료가 누락되거나 원인이 확정되지 않은 입력을 넣어 확인 질문이나 가설 표시가 남는지 검증한다. 근거 없는 단정을 수정해 요청 결과를 완성한다. 다음 회차에는 반복하는 후속 업무를 스킬로 만들고 변경 자료를 확인해 협의 안건을 정리한다.</x:v>
       </x:c>
       <x:c r="D33" s="144" t="n">
-        <x:v>60</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="34" s="1" customFormat="1" ht="28" customHeight="1">
@@ -6813,7 +6813,7 @@
         <x:v>회의에서 정한 업무와 변경 기록을 비교하여 다음에 확인할 안건을 근거와 함께 만든다. 재사용할 업무 지침과 실행 도구의 역할을 구분한다. 회의록의 결정·담당·기한과 Git 변경 기록·시각 정보를 연결해 완료·미결·변경 내용을 판단하는 기준을 이해한다.</x:v>
       </x:c>
       <x:c r="D38" s="142" t="n">
-        <x:v>25</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="39" s="1" customFormat="1" ht="92" customHeight="1">
@@ -6827,7 +6827,7 @@
         <x:v>공통 읽기 도구와 파일·Git·시간 MCP를 연결해 호출 결과를 확인한다. 제공 회의록 두 건과 점검 메모에서 결정·담당·기한·근거를 추출하는 스킬을 만들고, 없는 정보는 미정으로 남기는지 확인한다.</x:v>
       </x:c>
       <x:c r="D39" s="144" t="n">
-        <x:v>55</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="92" customHeight="1">
@@ -6855,7 +6855,7 @@
         <x:v>회의 업무 목록과 변경 기록을 합쳐 완료·미결·변경 사항 및 다음 협의에서 확인할 안건을 생성한다. 안건의 근거를 원문과 대조하고 같은 입력을 다시 실행해 필수 정보가 유지되는지 확인한다. 다음 회차에는 점검 요청 기능의 누락 입력과 변경 요구를 명세하고 검증한다.</x:v>
       </x:c>
       <x:c r="D41" s="144" t="n">
-        <x:v>70</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="42" s="1" customFormat="1" ht="28" customHeight="1">
@@ -6908,7 +6908,7 @@
         <x:v>점검 요청의 정보 누락·추가 답변·기능 변경을 처리하면서 기존 승인 조건을 보존한다. 필수 입력이 없을 때의 질문·보류와 사람 승인을 구분한다. 기능의 입력·출력·제약·완료 기준을 명세하고, 정상·누락·변경·기존 기능을 검증할 기대 결과로 바꾸는 방법을 익힌다.</x:v>
       </x:c>
       <x:c r="D46" s="142" t="n">
-        <x:v>30</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="47" s="1" customFormat="1" ht="92" customHeight="1">
@@ -6922,7 +6922,7 @@
         <x:v>포털의 승인·보류 상태를 확인한다. 점검 요청 초안의 필수 정보가 빠졌을 때 질문하고, 추가 답변을 반영해 다시 판단하는 흐름을 구현한다. 사람이 승인할 결과가 자동 확정되지 않는지 확인한다.</x:v>
       </x:c>
       <x:c r="D47" s="144" t="n">
-        <x:v>45</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="48" s="1" customFormat="1" ht="92" customHeight="1">
@@ -6936,7 +6936,7 @@
         <x:v>기존 점검 요청 기능에서 필요한 변경 한 건을 정한다. 입력·출력·사람 확인·완료 기준을 spec.md에 적고 기능을 구현한다. 변경 전부터 유지해야 할 출력 형식과 승인 조건을 함께 대조한다.</x:v>
       </x:c>
       <x:c r="D48" s="142" t="n">
-        <x:v>65</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="108" customHeight="1">
@@ -6950,7 +6950,7 @@
         <x:v>직접 정한 정상·정보 누락·변경 요구의 기대 결과를 Given/When/Then으로 작성한다. 실제 출력을 비교해 어긋난 조건을 수정하고, 기존 점검 요청과 승인 조건도 다시 실행해 회귀 오류가 없는지 확인한다. 다음 회차에는 검증한 작업을 승인·반려 경로가 있는 BPMN으로 표현한다.</x:v>
       </x:c>
       <x:c r="D49" s="144" t="n">
-        <x:v>60</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="50" s="1" customFormat="1" ht="28" customHeight="1">
@@ -7003,7 +7003,7 @@
         <x:v>작업 순서·승인 역할·실행 연결을 구분하여 같은 BPMN을 그림과 실행 관점에서 읽는다. 시작·종료 이벤트, 작업, 역할별 Lane, 승인 분기와 지연 알림의 의미를 설비 대응 사례로 구분한다. BPMN 그림의 각 작업이 에이전트·사람·시스템 중 누구에게 연결되는지 살펴보고, 승인 거절과 승인 대기 상태의 차이를 확인한다.</x:v>
       </x:c>
       <x:c r="D54" s="142" t="n">
-        <x:v>30</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="55" s="1" customFormat="1" ht="92" customHeight="1">
@@ -7017,7 +7017,7 @@
         <x:v>bpmn.io에서 시작→요청 확인→승인 또는 반려→종료를 그린다. 이어 쿨러 경보→원인 분석·조치 제안→운전원 승인→설비 명령→효과 확인→보고로 흐름을 확장하고, 담당 역할에 맞게 작업을 Lane에 배치한다.</x:v>
       </x:c>
       <x:c r="D55" s="144" t="n">
-        <x:v>60</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="56" s="1" customFormat="1" ht="92" customHeight="1">
@@ -7045,7 +7045,7 @@
         <x:v>bpmn.io에서 작성한 설비 대응 흐름과 포털에 등록된 기준 흐름을 비교한다. 제공 매핑 자료에서 시작 이벤트·에이전트·운전원 승인·설비 명령·재관측 작업의 연결을 찾는다. 자신이 그린 각 작업이 어떤 실행 기능에 대응하는지 표시하고, 그림 파일과 실행 정의를 구분한다. 다음 회차에는 등록된 흐름의 실행 이력을 대조하고 교대 인수인계 흐름을 구성한다.</x:v>
       </x:c>
       <x:c r="D57" s="144" t="n">
-        <x:v>60</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="58" s="1" customFormat="1" ht="28" customHeight="1">
@@ -7098,7 +7098,7 @@
         <x:v>설비 대응의 실행 이력에서 조건과 결과를 확인하고 교대의 검토·보완 흐름을 구성한다. 포털에 이미 등록된 설비 대응 흐름을 쿨러 열화 시나리오로 실행한다. 에이전트 판단→운전원 승인→설비 명령→재관측→완료 기록을 따라간다. 승인 대기와 반려 결과를 비교하고, 자신이 그린 BPMN의 작업·분기와 실행 이력을 대조한다.</x:v>
       </x:c>
       <x:c r="D62" s="142" t="n">
-        <x:v>45</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="63" s="1" customFormat="1" ht="92" customHeight="1">
@@ -7112,7 +7112,7 @@
         <x:v>자신의 BPMN 그림과 실행 이력의 작업·역할·분기 차이를 찾아 그림을 수정한다. 교대 인수인계에 필요한 설비·교대·기준 시각·작업 메모를 정하고, 인계자 검토와 인수자 확인을 완료 조건으로 작성한다.</x:v>
       </x:c>
       <x:c r="D63" s="144" t="n">
-        <x:v>30</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="64" s="1" customFormat="1" ht="98" customHeight="1">
@@ -7126,7 +7126,7 @@
         <x:v>강사 코드로 열린 교대 실습에서 제공 보충 매뉴얼을 선택한다. 준비된 추출 결과의 절차·조건·근거를 원문과 비교하고 검토한 항목을 기존 제조 지식에 추가한다. 추가된 지식의 식별자와 원문 연결을 확인한다. 교대 실습에서 허용된 설비·정비·ERP 조회 도구로 인계안을 작성하는 에이전트·스킬을 구성한다. 이름·설명·스킬에 확인할 항목을 적고, 완료 메모와 열린 작업지시 또는 입고 예정과 실제 재고가 다를 때 확인 사항으로 남기는지 결과와 원천을 대조한다.</x:v>
       </x:c>
       <x:c r="D64" s="142" t="n">
-        <x:v>75</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="65" s="1" customFormat="1" ht="108" customHeight="1">
@@ -7193,7 +7193,7 @@
         <x:v>정비·구매의 완료 의미를 비교하고 교대 인계 내용과 검토·확인 기록을 연결한다. 냉각 경보·정기 점검 도래·재고 부족의 시작 조건과 완료 결과를 비교한다. 정기 점검→정비 계획→설비보전팀장 승인 또는 거절→정비 오더→생산팀 공지 흐름을 bpmn.io에서 작성하고 담당 역할과 분기 조건을 연결한다.</x:v>
       </x:c>
       <x:c r="D70" s="142" t="n">
-        <x:v>30</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="71" s="1" customFormat="1" ht="92" customHeight="1">
@@ -7207,7 +7207,7 @@
         <x:v>포털의 정기 점검 시나리오로 등록된 정비 흐름을 실행한다. 정비 계획·승인·작업지시·예약 또는 출고·생산 공지의 처리 기록을 확인한다. 승인과 반려 사례를 비교하여 정비 오더가 만들어지는 조건을 자신의 BPMN과 대조한다.</x:v>
       </x:c>
       <x:c r="D71" s="144" t="n">
-        <x:v>40</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="72" s="1" customFormat="1" ht="92" customHeight="1">
@@ -7221,7 +7221,7 @@
         <x:v>bpmn.io에서 재고 부족→구매 제안→승인 또는 반려→발주→통지→입고 반영 흐름을 그린다. 포털의 재고 보충 시나리오로 등록된 구매 흐름을 실행한다. 수업용 업무 시스템에서 발주·공급사 통지·입고·재고 반영 기록을 확인하고, 반려 사례의 처리 결과와 비교한다. 자신의 BPMN에서 각 결과에 대응하는 작업을 찾는다.</x:v>
       </x:c>
       <x:c r="D72" s="142" t="n">
-        <x:v>60</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="73" s="1" customFormat="1" ht="145" customHeight="1">
@@ -7232,10 +7232,10 @@
         <x:v>교대 인수인계를 완성하고 ProcessGPT 연결 보기</x:v>
       </x:c>
       <x:c r="C73" s="143" t="str">
-        <x:v>교대 흐름에 설비·교대 정보를 입력하고 인계안의 근거와 원천 기록을 대조한다. 인계자 검토→인수자 보완 요청→재검토→인수 확인을 거쳐 완료 기록을 확인한다. 실제 결과에서 빠진 정보나 불일치가 있으면 확인 사항으로 남긴다(50분). 이어 ProcessGPT 시연에서 지식·에이전트·사람 작업·실행 기록이 어떻게 연결되는지 자신이 수행한 흐름과 비교한다(20분). 각자 인계 결과의 근거와 추가 확인할 사항을 설명한다.</x:v>
+        <x:v>교대 흐름에 설비·교대 정보를 입력하고 인계안의 근거와 원천 기록을 대조한다. 인계자 검토→인수자 보완 요청→재검토→인수 확인을 거쳐 완료 기록을 확인한다. 실제 결과에서 빠진 정보나 불일치가 있으면 확인 사항으로 남긴다(30분). 이어 ProcessGPT 시연에서 지식·에이전트·사람 작업·실행 기록이 어떻게 연결되는지 자신이 수행한 흐름과 비교한다(20분). 각자 인계 결과의 근거와 추가 확인할 사항을 설명한다.</x:v>
       </x:c>
       <x:c r="D73" s="144" t="n">
-        <x:v>70</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="74" s="1" customFormat="1" ht="28" customHeight="1">

</xml_diff>

<commit_message>
docs: make offline Notion labs optional when available
</commit_message>
<xml_diff>
--- a/문서/교재/실라버스/피지컬AI_실라버스_최종본.xlsx
+++ b/문서/교재/실라버스/피지컬AI_실라버스_최종본.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="통합반 온라인 44H" sheetId="1" r:id="Rc10916e20a7c4c8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="실전반 온라인 32H" sheetId="2" r:id="R8c64c90e0aba4c4b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="통합반 오프라인 정규 10회" sheetId="3" r:id="R4bd41221b5ac405f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="실전반 오프라인 정규 9회" sheetId="4" r:id="Rea900fb1e68f4ad8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="통합반 온라인 44H" sheetId="1" r:id="R21568ba90def4a1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="실전반 온라인 32H" sheetId="2" r:id="Rbfc15289e32e4af4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="통합반 오프라인 정규 10회" sheetId="3" r:id="Ra8ec69ab4946483d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="실전반 오프라인 정규 9회" sheetId="4" r:id="Ra430b6b3422a4a78"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5329,10 +5329,10 @@
         <x:v>실습</x:v>
       </x:c>
       <x:c r="B48" s="141" t="str">
-        <x:v>외부 MCP와 직접 만든 조회 도구 조합하기</x:v>
+        <x:v>파일·Git·시간 MCP를 연결하고 반환값 확인하기</x:v>
       </x:c>
       <x:c r="C48" s="141" t="str">
-        <x:v>파일·Git·시간 MCP를 연결하고 제공 서버 골격의 점검 자료 조회 함수를 구현한다. 도구 목록·입력·반환값을 확인한 뒤 기존 에이전트에서 외부 도구와 함께 호출한다. 자료 내용·변경 이력·기준 시각이 결과의 어느 근거에 쓰였는지 대조하고, 조회 실패와 자료 없음을 구분한다.</x:v>
+        <x:v>파일·Git·시간 MCP의 실행과 접근 범위를 설정하고 도구 목록·입력·반환값을 확인한다. 같은 자료의 내용·변경 이력·기준 시각을 대조하여 각 도구가 어떤 정보를 제공하는지 구분한다. 접근 실패와 자료 없음을 구분하고 연결 설정과 확인 결과를 저장한다.</x:v>
       </x:c>
       <x:c r="D48" s="142" t="n">
         <x:v>50</x:v>
@@ -5343,10 +5343,10 @@
         <x:v>실습</x:v>
       </x:c>
       <x:c r="B49" s="143" t="str">
-        <x:v>내 Notion 노트로 퀴즈를 풀고 피드백 확인하기</x:v>
+        <x:v>내 조회 도구를 구현하고 외부 MCP와 조합해 검증하기</x:v>
       </x:c>
       <x:c r="C49" s="143" t="str">
-        <x:v>1회차부터 자기 Notion에 정리한 학습노트의 페이지를 선택하고 MCP 읽기 연결을 설정한다. 노트에서 문항·정답 기준·해설·원문 근거를 구성하는 퀴즈 에이전트를 만들되, 답하기 전에는 정답과 해설을 숨긴다. 학생 답변을 받아 정답·부분 정답·오답과 이유를 알려주고 원문을 다시 열어 확인한다. 다음 문항과 틀린 개념 재도전으로 이어가며 풀이 기록을 저장한다. 표현만 다른 정답·불완전한 답·노트에 없는 질문으로 검증하고, 근거가 부족하면 출제나 채점을 보류한다. Notion 연결이 안 되면 같은 노트의 Markdown 내보내기로 진행하고 실제 MCP 연결 여부를 따로 기록한다. 다음 회차에는 업무 에이전트의 정보 누락·변경 요구를 질문·명세·검증으로 다룬다.</x:v>
+        <x:v>제공 서버 골격에 점검 자료 조회 함수를 구현하고 MCP 도구로 노출한다. 앞에서 연결한 파일·Git·시간 도구와 함께 호출해 자료 내용·변경 이력·시각을 근거로 확인 결과를 만든다. 다른 대상·없는 자료·조회 실패 사례로 결과를 검증하고 코드·설정·출처를 저장한다. 다음 회차에는 점검 요청의 정보 누락과 요구 변경을 질문·명세·검증으로 다룬다. 기본 진행은 Notion 없이 한다. 현장에서 Notion 설치·접속·MCP 연결과 자기 노트 준비가 가능하면, 이 교시의 조회 도구 실습 대신 자기 노트로 문항을 만들고 답변·채점·해설·원문 근거를 확인하는 퀴즈 에이전트 실습을 선택한다. 연결이 안 되면 기본 실습을 계속한다.</x:v>
       </x:c>
       <x:c r="D49" s="144" t="n">
         <x:v>50</x:v>
@@ -6827,10 +6827,10 @@
         <x:v>실습</x:v>
       </x:c>
       <x:c r="B40" s="141" t="str">
-        <x:v>Notion·외부 MCP와 내 조회 도구 연결하기</x:v>
+        <x:v>파일·Git·시간 MCP와 내 조회 도구 연결하기</x:v>
       </x:c>
       <x:c r="C40" s="141" t="str">
-        <x:v>자기 Notion 기록과 파일·Git·시간 MCP의 접근 범위를 설정한다. 제공 서버 골격에 점검 메모 조회 함수를 구현하고 기존 에이전트에서 호출한다. 이전 회의와 후속 자료에서 바뀐 내용·근거 페이지 또는 파일·시각을 연결한다. Notion 미연결 시 같은 자료의 내보내기로 진행하되 실제 연결 성공과 구분한다.</x:v>
+        <x:v>제공 회의록·점검 메모를 읽도록 파일·Git·시간 MCP의 접근 범위를 설정한다. 제공 서버 골격에 점검 메모 조회 함수를 구현하고 기존 에이전트에서 호출한다. 이전 회의와 후속 자료에서 바뀐 내용·근거 파일·시각을 연결하고 조회 실패와 자료 없음을 구분한다. 기본 진행은 Notion 없이 한다. 현장에서 Notion 설치·접속·MCP 연결이 가능하고 자기 기록이 준비되어 있으면, 제공 파일 대신 자기 Notion 기록을 읽어 후속 협의 안건에 활용한다. 연결이 안 되면 제공 파일로 계속한다.</x:v>
       </x:c>
       <x:c r="D40" s="142" t="n">
         <x:v>50</x:v>
@@ -6844,7 +6844,7 @@
         <x:v>다음 협의 안건을 만들고 검증하기</x:v>
       </x:c>
       <x:c r="C41" s="143" t="str">
-        <x:v>앞서 연결한 Notion 기록·회의록·점검 메모와 회의 스킬을 조합해 다음 협의 안건을 만든다. 안건마다 결정할 질문·확인된 사실·남은 확인·페이지 또는 파일 근거를 표시한다. 후속 자료를 반영한 결과를 이전 결과와 대조하여 결정이 사라지거나 중복되지 않는지 확인한다. 직접 쓴 기록이 부족하면 제공 회의 자료를 사용한다. 다음 회차에는 점검 요청의 변경 요구를 명세하고 검증한다.</x:v>
+        <x:v>앞서 연결한 회의록·점검 메모·변경 이력과 회의 스킬을 조합해 다음 협의 안건을 만든다. 안건마다 결정할 질문·확인된 사실·남은 확인·파일 근거를 표시한다. 후속 자료를 반영한 결과를 이전 결과와 대조하여 결정이 사라지거나 중복되지 않는지 확인한다. 다음 회차에는 점검 요청의 변경 요구를 명세하고 검증한다.</x:v>
       </x:c>
       <x:c r="D41" s="144" t="n">
         <x:v>50</x:v>

</xml_diff>